<commit_message>
Complete Phase 1: fixtures, async states, and E2E coverage for feature pages
- Extract backend-bound prototype data from Login, Wallet, Oasis, and
  Creator Dashboard into fixtures/{login,wallet,oasis,creatorDashboard}.js
- Add loading/empty/error/retry states to Wallet, Oasis, and Creator
  Dashboard via useSimulatedFetch
- Expand Playwright coverage for feature-page states and retry paths
- Reconcile CLAUDE.md and HANDOFF.md with the final Phase 1 architecture
- Update master tracker with the June 28 Phase 1 verification

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product/Pumdoki_MasterTracker_V4.xlsx
+++ b/docs/product/Pumdoki_MasterTracker_V4.xlsx
@@ -2877,7 +2877,7 @@
       </c>
       <c r="C13" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Statuses reconciled against the repository and founder decisions through June 21, 2026.</t>
+          <t xml:space="preserve">• Statuses reconciled against the repository and founder decisions through June 28, 2026.</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
     <row r="20">
       <c r="C20" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Sakura Kiss Edition — updated June 21, 2026. Detailed sequencing is maintained in PLAN.md.</t>
+          <t xml:space="preserve">• Sakura Kiss Edition — updated June 28, 2026. Full repository/frontend Phase 1 is verified; detailed sequencing remains in PLAN.md.</t>
         </is>
       </c>
     </row>
@@ -4651,11 +4651,15 @@
       <c r="B53" s="17" t="s">
         <v>167</v>
       </c>
-      <c r="C53" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D53" s="19" t="s">
-        <v>168</v>
+      <c r="C53" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">🔄 In Progress</t>
+        </is>
+      </c>
+      <c r="D53" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repository CI now runs lint, unit tests, production build, and Playwright. Deployment automation remains for Phase 2/staging.</t>
+        </is>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
@@ -6318,7 +6322,7 @@
       </c>
       <c r="D161" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monorepo workspace structure created; backend code not started.</t>
+          <t xml:space="preserve">Full repository/frontend Phase 1 verified June 28, 2026. TypeScript API, contracts, and database implementation begins in Phase 2.</t>
         </is>
       </c>
     </row>
@@ -8653,7 +8657,7 @@
       </c>
       <c r="B4" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">This workbook is reconciled with the repository and founder decisions through June 21, 2026.</t>
+          <t xml:space="preserve">This workbook is reconciled with the repository and founder decisions through June 28, 2026.</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8964,7 @@
       </c>
       <c r="B44" s="63" t="inlineStr">
         <is>
-          <t xml:space="preserve">The current dependency-ordered implementation roadmap is maintained in repository PLAN.md. The prior week-by-week text in this sheet has been superseded.</t>
+          <t xml:space="preserve">The dependency-ordered roadmap is maintained in repository PLAN.md, which references @CLAUDE.md and requires recorded verification before any phase is marked complete.</t>
         </is>
       </c>
     </row>
@@ -9015,7 +9019,7 @@
     <row r="49" ht="15.75" customHeight="1">
       <c r="B49" s="66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Begin routing, quality tooling, shared frontend shell, and backend foundation.</t>
+          <t xml:space="preserve">Full repository/frontend Phase 1 completed and verified June 28, 2026: lint 0 warnings, unit tests 12/12, production build passed, and Playwright 27/27. Phase 2 backend/database foundation is next.</t>
         </is>
       </c>
       <c r="A49" s="65" t="inlineStr">

</xml_diff>

<commit_message>
feat: complete Phase 3 email-flow slice
</commit_message>
<xml_diff>
--- a/docs/product/Pumdoki_MasterTracker_V4.xlsx
+++ b/docs/product/Pumdoki_MasterTracker_V4.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R38c2234046b8464c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R1b2c8338b93a4688"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R124ff7d611be405f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="Rb08389583c244efc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R767b57c29b174fd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2ead6241c74449ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R89447e311d19443b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R839a0f3f3794457e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="R2f608c88c4c14958"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R1c65a635e98b41f4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2394,7 +2394,7 @@
       </x:c>
       <x:c r="B6" s="7" t="n">
         <x:f>COUNTIF('Master Tracker'!C4:C164,"✅ Done")</x:f>
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D6" s="7" t="s">
         <x:v>7</x:v>
@@ -2419,7 +2419,7 @@
       </x:c>
       <x:c r="B8" s="7" t="n">
         <x:f>COUNTIF('Master Tracker'!C4:C164,"📋 Not Started")</x:f>
-        <x:v>86</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2428,7 +2428,7 @@
       </x:c>
       <x:c r="B9" s="8" t="n">
         <x:f>IF(B5=0,0,B6/B5)</x:f>
-        <x:v>0.08783783783783784</x:v>
+        <x:v>0.10135135135135136</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="13.5" customHeight="1"/>
@@ -2440,15 +2440,15 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="22.5" customHeight="1">
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="9" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="C13" s="31" t="str">
-        <x:v>• Statuses reconciled against the repository and founder decisions through July 16, 2026.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="16.5" customHeight="1">
+        <x:v>• Statuses reconciled against the repository and founder decisions through July 28, 2026.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="9" t="s">
         <x:v>8</x:v>
       </x:c>
@@ -2456,7 +2456,7 @@
         <x:v>12</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="16.5" customHeight="1">
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="9" t="s">
         <x:v>7</x:v>
       </x:c>
@@ -2464,29 +2464,29 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="16.5" customHeight="1">
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="C16" s="10" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="16.5" customHeight="1">
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="C17" s="10" t="s">
         <x:v>15</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="16.5" customHeight="1">
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="C18" s="10" t="s">
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="16.5" customHeight="1">
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="C19" s="10" t="s">
         <x:v>17</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="31.5" customHeight="1">
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="C20" s="37" t="str">
-        <x:v>• Sakura Kiss Edition — updated July 16, 2026. Phase 1 is verified; Phase 2 remains partially complete; Phase 3 core-auth backend slice is implemented and locally verified.</x:v>
+        <x:v>• Sakura Kiss Edition — updated July 28, 2026. Phase 1 is verified; Phase 2 remains partially complete; Phase 3 core-auth and email-flow backend slices are implemented and locally verified.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="16.5" customHeight="1">
@@ -4121,7 +4121,7 @@
         <x:v>141</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="15.75" customHeight="1">
+    <x:row r="47" ht="24" hidden="0" customHeight="1">
       <x:c r="A47" s="16" t="s">
         <x:v>142</x:v>
       </x:c>
@@ -4132,10 +4132,10 @@
         <x:v>🔄 In Progress</x:v>
       </x:c>
       <x:c r="D47" s="19" t="str">
-        <x:v>Local PostgreSQL/Prisma foundation now includes repeatable User, Session, and append-only AcceptanceRecord migrations. Remaining product domains and production RDS schema are pending.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="15.75" customHeight="1">
+        <x:v>Local PostgreSQL/Prisma now includes repeatable User, Session, append-only AcceptanceRecord, and transient VerificationToken migrations. Remaining product domains and production RDS schema are pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="20" t="s">
         <x:v>144</x:v>
       </x:c>
@@ -4149,7 +4149,7 @@
         <x:v>Local environment is defined with validated variables and Docker PostgreSQL. Staging and production infrastructure remain pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="15.75" customHeight="1">
+    <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="16" t="s">
         <x:v>146</x:v>
       </x:c>
@@ -4162,10 +4162,10 @@
         </x:is>
       </x:c>
       <x:c r="D49" s="19" t="str">
-        <x:v>Implemented /api/v1 health/readiness plus core auth endpoints: register, login, logout, logout-all, and /me. Later product domains remain pending.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50" ht="15.75" customHeight="1">
+        <x:v>Implemented /api/v1 health/readiness, core auth, email verification, password reset, logout/logout-all, and /me. Later product domains remain pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="20" t="s">
         <x:v>148</x:v>
       </x:c>
@@ -4179,7 +4179,7 @@
         <x:v>Structured Pino request logging is implemented with request IDs and secret-header redaction. Sentry/operational error monitoring remains pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" ht="15.75" customHeight="1">
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="16" t="s">
         <x:v>150</x:v>
       </x:c>
@@ -4193,7 +4193,7 @@
         <x:v>152</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="15.75" customHeight="1">
+    <x:row r="52" ht="24" hidden="0" customHeight="1">
       <x:c r="A52" s="20" t="s">
         <x:v>153</x:v>
       </x:c>
@@ -4204,10 +4204,10 @@
         <x:v>🔄 In Progress</x:v>
       </x:c>
       <x:c r="D52" s="22" t="str">
-        <x:v>Global per-IP limits and a bounded in-memory per-email+IP login-failure throttle are implemented. Redis-backed multi-instance protection remains pending.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53" ht="15.75" customHeight="1">
+        <x:v>Global per-IP limits plus bounded in-memory login and email-request throttles are implemented. Redis-backed multi-instance protection remains pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="16" t="s">
         <x:v>155</x:v>
       </x:c>
@@ -4223,7 +4223,7 @@
         <x:v>CI runs web lint/tests/build/E2E plus API build, migrations, seed, and DB-backed tests on PostgreSQL 17. Deployment automation remains pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="15.75" customHeight="1">
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="20" t="s">
         <x:v>157</x:v>
       </x:c>
@@ -4245,7 +4245,7 @@
       <x:c r="C55" s="2"/>
       <x:c r="D55" s="3"/>
     </x:row>
-    <x:row r="56" ht="15.75" customHeight="1">
+    <x:row r="56" ht="24" hidden="0" customHeight="1">
       <x:c r="A56" s="16" t="s">
         <x:v>161</x:v>
       </x:c>
@@ -4256,10 +4256,10 @@
         <x:v>🔄 In Progress</x:v>
       </x:c>
       <x:c r="D56" s="19" t="str">
-        <x:v>Phase 3 slice 1 backend is implemented: registration, login, logout, logout-all, Argon2id hashing, duplicate handling, and public-user responses. Frontend integration remains slice 3.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="57" ht="15.75" customHeight="1">
+        <x:v>Phase 3 slices 1–2 backend are implemented: registration, login, logout, logout-all, Argon2id hashing, verification mail, password reset, duplicate handling, and public-user responses. Frontend integration remains slice 3.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="20" t="s">
         <x:v>163</x:v>
       </x:c>
@@ -4273,7 +4273,7 @@
         <x:v>Role enums and API requireAuth/requireRole enforcement are implemented and tested. Admin endpoints and frontend role routing remain pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" ht="15.75" customHeight="1">
+    <x:row r="58" ht="24" hidden="0" customHeight="1">
       <x:c r="A58" s="16" t="s">
         <x:v>165</x:v>
       </x:c>
@@ -4287,7 +4287,7 @@
         <x:v>Opaque SHA-256-hashed sessions, secure HttpOnly cookies, 30-day sliding expiry, daily renewal throttle, revocation, and logout-all are implemented. Frontend persistence remains pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" ht="15.75" customHeight="1">
+    <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="20" t="s">
         <x:v>167</x:v>
       </x:c>
@@ -4305,7 +4305,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="60" ht="15.75" customHeight="1">
+    <x:row r="60" ht="24" hidden="0" customHeight="1">
       <x:c r="A60" s="16" t="s">
         <x:v>169</x:v>
       </x:c>
@@ -4319,7 +4319,7 @@
         <x:v>Registration now records append-only age attestation plus versioned Terms and Privacy acceptance in one transaction. Entry UI and identity/age verification remain pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="15.75" customHeight="1">
+    <x:row r="61" ht="24" hidden="0" customHeight="1">
       <x:c r="A61" s="20" t="s">
         <x:v>171</x:v>
       </x:c>
@@ -4327,13 +4327,13 @@
         <x:v>172</x:v>
       </x:c>
       <x:c r="C61" s="24" t="s">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D61" s="22" t="str">
-        <x:v>User.emailVerifiedAt groundwork exists. Verification tokens, Mailpit/mailer abstraction, delivery, and enforcement begin in Phase 3 slice 2.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62" ht="15.75" customHeight="1">
+        <x:v>Provider-neutral mailer, Mailpit SMTP, hashed 24-hour single-use verification tokens, reissue invalidation, confirm endpoint, request throttle, registration mail, and requireVerifiedEmail are implemented and verified locally. Production provider/deliverability remain open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="24" hidden="0" customHeight="1">
       <x:c r="A62" s="16" t="s">
         <x:v>173</x:v>
       </x:c>
@@ -4341,10 +4341,10 @@
         <x:v>174</x:v>
       </x:c>
       <x:c r="C62" s="24" t="s">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D62" s="19" t="str">
-        <x:v>Planned for Phase 3 slice 2 with the same mailer abstraction; no reset-token flow exists yet.</x:v>
+        <x:v>Neutral reset requests, hashed one-hour single-use tokens, Argon2id password replacement, session revocation, mailbox-based verification, expiry/wrong-kind handling, and Mailpit delivery are implemented and verified locally. Frontend reset screens remain slice 3.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="27.75" customHeight="1">
@@ -5777,7 +5777,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="157" ht="31.5" customHeight="1">
+    <x:row r="157" ht="24" hidden="0" customHeight="1">
       <x:c r="A157" s="16" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Select transactional email provider</x:t>
@@ -5793,13 +5793,11 @@
           <x:t xml:space="preserve">📋 Not Started</x:t>
         </x:is>
       </x:c>
-      <x:c r="D157" s="19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Use reserved sample addresses such as support@pumdoki.example until real inboxes exist.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="158" ht="31.5" customHeight="1">
+      <x:c r="D157" s="19" t="str">
+        <x:v>Provider-neutral SMTP/console abstraction and local Mailpit are implemented. Production provider selection, adult-business support, deliverability, TLS, DKIM, SPF, and DMARC remain open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" ht="15" hidden="0" customHeight="1">
       <x:c r="A158" s="20" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Choose LLC state and privacy structure</x:t>
@@ -5821,7 +5819,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="159" ht="31.5" customHeight="1">
+    <x:row r="159" ht="15" hidden="0" customHeight="1">
       <x:c r="A159" s="16" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Decide commission and payout model</x:t>
@@ -5843,7 +5841,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="160" ht="31.5" customHeight="1">
+    <x:row r="160" ht="24" hidden="0" customHeight="1">
       <x:c r="A160" s="20" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Define MVP Admin architecture</x:t>
@@ -5863,7 +5861,7 @@
         <x:v>Recommended protected /admin architecture is documented in PLAN.md. API role enforcement now exists, but admin routes, sensitive permissions, and audit logging remain pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="161" ht="31.5" customHeight="1">
+    <x:row r="161" ht="24" hidden="0" customHeight="1">
       <x:c r="A161" s="16" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Adopt TypeScript backend and shared contracts</x:t>
@@ -5880,7 +5878,7 @@
         </x:is>
       </x:c>
       <x:c r="D161" s="19" t="str">
-        <x:v>TypeScript API/contracts/database foundation is active. Core auth backend and DB-backed tests are implemented; the JavaScript frontend remains intentionally unchanged until integration.</x:v>
+        <x:v>TypeScript API/contracts/database foundation now includes core auth, email verification/password reset, mail transports, and DB-backed tests. The JavaScript frontend remains unchanged until slice 3 integration.</x:v>
       </x:c>
     </x:row>
     <x:row r="162" ht="31.5" customHeight="1">
@@ -8492,34 +8490,34 @@
       </x:c>
     </x:row>
     <x:row r="42" ht="15.75" customHeight="1"/>
-    <x:row r="43" ht="15.75" customHeight="1">
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="61" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">🚀 Current Delivery Plan</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="44" ht="36" customHeight="1">
+    <x:row r="44" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A44" s="71" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Plan source</x:t>
         </x:is>
       </x:c>
       <x:c r="B44" s="71" t="str">
-        <x:v>The dependency-ordered roadmap remains in repository PLAN.md. Phase 1 is verified, Phase 2 is partially complete, and Phase 3 is split into four independently verified slices.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="36" customHeight="1">
+        <x:v>The dependency-ordered roadmap remains in repository PLAN.md. Phase 1 is verified, Phase 2 is partially complete, and Phase 3 is split into four independently verified slices; slices 1–2 are locally verified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A45" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 1</x:t>
         </x:is>
       </x:c>
       <x:c r="B45" s="73" t="str">
-        <x:v>Phase 3 slice 1 core-auth backend is implemented and locally verified. Next engineering slice: email verification and password reset using Mailpit plus a provider-neutral mailer abstraction.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="36" customHeight="1">
+        <x:v>Phase 3 slice 2 email verification and password reset are implemented and locally verified with provider-neutral mail, Mailpit, single-use hashed tokens, session revocation, and DB-backed tests. Next engineering slice: frontend auth integration.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A46" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 2</x:t>
@@ -8529,7 +8527,7 @@
         <x:v>Keep Phase 2 labeled partially complete; decide AWS/Sentry/Redis direction and finish staging, backups/restore, monitoring, queueing, and idempotency.</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="36" customHeight="1">
+    <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 3</x:t>
@@ -8539,7 +8537,7 @@
         <x:v>Begin privacy-focused LLC attorney/CPA research, counsel-reviewed retention rules, and merchant compliance preparation in parallel.</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="36" customHeight="1">
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 4</x:t>
@@ -8549,31 +8547,31 @@
         <x:v>Obtain CCBill/Epoch requirements, fee quotes, and written cascade guidance; continue identity-provider and launch-country research.</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="36" customHeight="1">
+    <x:row r="49" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A49" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 5</x:t>
         </x:is>
       </x:c>
       <x:c r="B49" s="73" t="str">
-        <x:v>Verification is recorded in HANDOFF.md. The corrected design commit remains local until an explicit public-repository push is approved.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50" ht="15.75" customHeight="1">
+        <x:v>Local verification is recorded in HANDOFF.md. Publication to the confirmed public repository is pending the required GitHub CLI/authentication prerequisite and CI verification.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="64"/>
       <x:c r="B50" s="64"/>
     </x:row>
-    <x:row r="51" ht="15.75" customHeight="1">
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="65"/>
       <x:c r="B51" s="66"/>
     </x:row>
-    <x:row r="52" ht="19.5" customHeight="1">
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="65" t="str">
         <x:v>✅ July 7, 2026 — Confirmed Founder Decisions</x:v>
       </x:c>
       <x:c r="B52" s="66"/>
     </x:row>
-    <x:row r="53" ht="34.5" customHeight="1">
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="74" t="str">
         <x:v>•</x:v>
       </x:c>
@@ -8581,7 +8579,7 @@
         <x:v>Phase 3 starts on the local stack while Phase 2 remains explicitly partially complete.</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="34.5" customHeight="1">
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="74" t="str">
         <x:v>•</x:v>
       </x:c>
@@ -8589,7 +8587,7 @@
         <x:v>First beta uses email/password only; Google OAuth is not beta scope.</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="34.5" customHeight="1">
+    <x:row r="55" ht="15" hidden="0" customHeight="1">
       <x:c r="A55" s="74" t="str">
         <x:v>•</x:v>
       </x:c>
@@ -8597,7 +8595,7 @@
         <x:v>Phase 3 is decomposed into four slices: core auth backend, email flows, frontend integration, and Settings.</x:v>
       </x:c>
     </x:row>
-    <x:row r="56" ht="34.5" customHeight="1">
+    <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="74" t="str">
         <x:v>•</x:v>
       </x:c>
@@ -8605,7 +8603,7 @@
         <x:v>Sessions use opaque tokens with 30-day sliding expiry, renewed at most once per day.</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="34.5" customHeight="1">
+    <x:row r="57" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A57" s="81" t="str">
         <x:v>•</x:v>
       </x:c>
@@ -8613,15 +8611,15 @@
         <x:v>Acceptance records are append-only with restrictive deletion; future account deletion must follow counsel-approved retention and pseudonymization rules.</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" ht="34.5" customHeight="1">
+    <x:row r="58" ht="15" hidden="0" customHeight="1">
       <x:c r="A58" s="74" t="str">
         <x:v>•</x:v>
       </x:c>
       <x:c r="B58" s="79" t="str">
-        <x:v>Phase 3 slice 1 is backend-only; no frontend authentication behavior is claimed yet.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59" ht="34.5" customHeight="1">
+        <x:v>Phase 3 slices 1–2 are backend-only; no real frontend authentication behavior is claimed yet.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="74" t="str">
         <x:v>•</x:v>
       </x:c>
@@ -8629,30 +8627,48 @@
         <x:v>Core-auth implementation uses Argon2id and transparently upgrades the development scrypt seed format after a successful login.</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" ht="34.5" customHeight="1">
+    <x:row r="60" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A60" s="74" t="str">
         <x:v>•</x:v>
       </x:c>
       <x:c r="B60" s="79" t="str">
-        <x:v>Email verification enforcement, password reset, frontend auth, Settings, OAuth, and Redis-backed throttling remain later slices or deferred work.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61" ht="15.75" customHeight="1">
+        <x:v>Email verification and password reset are implemented locally. Frontend auth, Settings, OAuth, a production email provider, and Redis-backed throttling remain later slices or deferred work.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="15" hidden="0" customHeight="1">
       <x:c r="A61" s="65"/>
       <x:c r="B61" s="66"/>
     </x:row>
-    <x:row r="62" ht="15.75" customHeight="1">
-      <x:c r="A62" s="65"/>
+    <x:row r="62" ht="15" hidden="0" customHeight="1">
+      <x:c r="A62" s="65" t="str">
+        <x:v>✅ July 28, 2026 — Phase 3 Slice 2 Verification</x:v>
+      </x:c>
       <x:c r="B62" s="66"/>
     </x:row>
-    <x:row r="63" ht="15.75" customHeight="1">
-      <x:c r="A63" s="64"/>
-      <x:c r="B63" s="67"/>
-    </x:row>
-    <x:row r="64" ht="15.75" customHeight="1">
-      <x:c r="B64" s="66"/>
-    </x:row>
-    <x:row r="65" ht="15.75" customHeight="1"/>
+    <x:row r="63" ht="15" hidden="0" customHeight="1">
+      <x:c r="A63" s="64" t="str">
+        <x:v>•</x:v>
+      </x:c>
+      <x:c r="B63" s="67" t="str">
+        <x:v>Provider-neutral SMTP/console mail, local Mailpit, verification and reset templates, and validated mail environment variables are implemented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="15" hidden="0" customHeight="1">
+      <x:c r="A64" t="str">
+        <x:v>•</x:v>
+      </x:c>
+      <x:c r="B64" s="66" t="str">
+        <x:v>Verification and reset tokens are random, hashed at rest, expiring, single-use, and invalidated on reissue; password reset revokes all sessions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="15" hidden="0" customHeight="1">
+      <x:c r="A65" t="str">
+        <x:v>•</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>Production email provider selection and deliverability controls remain open; Phase 3 slice 3 is frontend authentication integration.</x:v>
+      </x:c>
+    </x:row>
     <x:row r="66" ht="15.75" customHeight="1">
       <x:c r="A66" s="61" t="inlineStr">
         <x:is>
@@ -9931,6 +9947,7 @@
     <x:mergeCell ref="A43:B43"/>
     <x:mergeCell ref="A66:B66"/>
     <x:mergeCell ref="A52:B52"/>
+    <x:mergeCell ref="A62:B62"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat: complete Phase 3 frontend auth integration
</commit_message>
<xml_diff>
--- a/docs/product/Pumdoki_MasterTracker_V4.xlsx
+++ b/docs/product/Pumdoki_MasterTracker_V4.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2ead6241c74449ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R89447e311d19443b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R839a0f3f3794457e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="R2f608c88c4c14958"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R1c65a635e98b41f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6f36460bd2144711"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R73c3899e5fae4b40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R8796ddf8c1b048df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="R4a98665446be48dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R65b6aee0e9dc4edf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -593,18 +593,12 @@
     <x:t xml:space="preserve">Account entry screens for creators and members.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Auth screen complete. Welcome back card, Google SSO, create account flow present.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Implement story rail / For You model</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Translate the interaction/feed architecture into actual UI behavior.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Architecture defined; build not confirmed.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Implement locked-content previews</x:t>
   </x:si>
   <x:si>
@@ -857,15 +851,6 @@
     <x:t xml:space="preserve">🛡️  PHASE 9 — Admin Dashboard &amp; Moderation</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Protect /admin route</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Restrict to admin-role only. Login-gated, founder-only access. Separate from creator dashboard.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Admin route planned; not confirmed built.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Build admin overview / operations page</x:t>
   </x:si>
   <x:si>
@@ -1440,9 +1425,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">NSFW content allowed from day 1. +18 toggle required in settings and feed.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Admin dashboard: protected page inside Pumdoki, login-gated, founder-only. 13 subtasks defined.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Dark Knight theme: second default theme. Charcoal/near-black + pink accent. CSS variable swap.</x:t>
@@ -2394,7 +2376,7 @@
       </x:c>
       <x:c r="B6" s="7" t="n">
         <x:f>COUNTIF('Master Tracker'!C4:C164,"✅ Done")</x:f>
-        <x:v>15</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D6" s="7" t="s">
         <x:v>7</x:v>
@@ -2410,7 +2392,7 @@
       </x:c>
       <x:c r="B7" s="6" t="n">
         <x:f>COUNTIF('Master Tracker'!C4:C164,"🔄 In Progress")</x:f>
-        <x:v>49</x:v>
+        <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2428,7 +2410,7 @@
       </x:c>
       <x:c r="B9" s="8" t="n">
         <x:f>IF(B5=0,0,B6/B5)</x:f>
-        <x:v>0.10135135135135136</x:v>
+        <x:v>0.12837837837837837</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="13.5" customHeight="1"/>
@@ -2445,7 +2427,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C13" s="31" t="str">
-        <x:v>• Statuses reconciled against the repository and founder decisions through July 28, 2026.</x:v>
+        <x:v>Counts are derived from the Master Tracker through August 1, 2026. Section headers are excluded.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -2486,7 +2468,7 @@
     </x:row>
     <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="C20" s="37" t="str">
-        <x:v>• Sakura Kiss Edition — updated July 28, 2026. Phase 1 is verified; Phase 2 remains partially complete; Phase 3 core-auth and email-flow backend slices are implemented and locally verified.</x:v>
+        <x:v>Phase 1 is verified; Phase 2 remains partial; Phase 3 Slices 1–3 are implemented and locally verified. Slice 4 (Settings and explicit-content controls) remains next.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="16.5" customHeight="1">
@@ -4253,10 +4235,10 @@
         <x:v>162</x:v>
       </x:c>
       <x:c r="C56" s="24" t="str">
-        <x:v>🔄 In Progress</x:v>
+        <x:v>✅ Done</x:v>
       </x:c>
       <x:c r="D56" s="19" t="str">
-        <x:v>Phase 3 slices 1–2 backend are implemented: registration, login, logout, logout-all, Argon2id hashing, verification mail, password reset, duplicate handling, and public-user responses. Frontend integration remains slice 3.</x:v>
+        <x:v>Slice 3 connects registration, login, logout, and authenticated route restoration to the live API.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
@@ -4267,10 +4249,10 @@
         <x:v>164</x:v>
       </x:c>
       <x:c r="C57" s="24" t="str">
-        <x:v>🔄 In Progress</x:v>
+        <x:v>✅ Done</x:v>
       </x:c>
       <x:c r="D57" s="22" t="str">
-        <x:v>Role enums and API requireAuth/requireRole enforcement are implemented and tested. Admin endpoints and frontend role routing remain pending.</x:v>
+        <x:v>Slice 3 enforces uppercase MEMBER/CREATOR/ADMIN role routing and protected-route authorization in the frontend.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="24" hidden="0" customHeight="1">
@@ -4281,10 +4263,10 @@
         <x:v>166</x:v>
       </x:c>
       <x:c r="C58" s="24" t="str">
-        <x:v>🔄 In Progress</x:v>
+        <x:v>✅ Done</x:v>
       </x:c>
       <x:c r="D58" s="19" t="str">
-        <x:v>Opaque SHA-256-hashed sessions, secure HttpOnly cookies, 30-day sliding expiry, daily renewal throttle, revocation, and logout-all are implemented. Frontend persistence remains pending.</x:v>
+        <x:v>Slice 3 restores HttpOnly-cookie sessions with /me, handles expiry/401 globally, and supports logout from the member shell.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
@@ -4294,15 +4276,11 @@
       <x:c r="B59" s="21" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="C59" s="23" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">🔄 In Progress</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D59" s="19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Creator onboarding UI prototype exists. Real identity, agreement, tax, role, and approval workflows are pending.</x:t>
-        </x:is>
+      <x:c r="C59" s="23" t="str">
+        <x:v>🔄 In Progress</x:v>
+      </x:c>
+      <x:c r="D59" s="19" t="str">
+        <x:v>Frontend prototypes exist; creator/member first-run onboarding and creator theme selection remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="24" hidden="0" customHeight="1">
@@ -4330,7 +4308,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="D61" s="22" t="str">
-        <x:v>Provider-neutral mailer, Mailpit SMTP, hashed 24-hour single-use verification tokens, reissue invalidation, confirm endpoint, request throttle, registration mail, and requireVerifiedEmail are implemented and verified locally. Production provider/deliverability remain open.</x:v>
+        <x:v>Slice 3 adds the email verification screen, persistent unverified banner, resend states, and Mailpit-backed browser coverage.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="24" hidden="0" customHeight="1">
@@ -4344,7 +4322,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="D62" s="19" t="str">
-        <x:v>Neutral reset requests, hashed one-hour single-use tokens, Argon2id password replacement, session revocation, mailbox-based verification, expiry/wrong-kind handling, and Mailpit delivery are implemented and verified locally. Frontend reset screens remain slice 3.</x:v>
+        <x:v>Slice 3 adds forgot/reset password screens, neutral request messaging, token handling, session revocation, and browser coverage.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="27.75" customHeight="1">
@@ -4432,33 +4410,33 @@
       <x:c r="B69" s="21" t="s">
         <x:v>192</x:v>
       </x:c>
-      <x:c r="C69" s="23" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D69" s="22" t="s">
-        <x:v>193</x:v>
+      <x:c r="C69" s="23" t="str">
+        <x:v>✅ Done</x:v>
+      </x:c>
+      <x:c r="D69" s="22" t="str">
+        <x:v>Slice 3 replaces prototype login/signup behavior with validated live-API flows and adds forgot/reset/verify screens.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="15.75" customHeight="1">
       <x:c r="A70" s="16" t="s">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="B70" s="17" t="s">
         <x:v>194</x:v>
       </x:c>
-      <x:c r="B70" s="17" t="s">
-        <x:v>195</x:v>
-      </x:c>
-      <x:c r="C70" s="18" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="D70" s="19" t="s">
-        <x:v>196</x:v>
+      <x:c r="C70" s="18" t="str">
+        <x:v>✅ Done</x:v>
+      </x:c>
+      <x:c r="D70" s="19" t="str">
+        <x:v>Heart rail + Following/For You hybrid implemented in design.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="15.75" customHeight="1">
       <x:c r="A71" s="20" t="s">
-        <x:v>197</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="B71" s="21" t="s">
-        <x:v>198</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="C71" s="23" t="inlineStr">
         <x:is>
@@ -4473,10 +4451,10 @@
     </x:row>
     <x:row r="72" ht="15.75" customHeight="1">
       <x:c r="A72" s="16" t="s">
-        <x:v>199</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="B72" s="17" t="s">
-        <x:v>200</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C72" s="23" t="inlineStr">
         <x:is>
@@ -4491,10 +4469,10 @@
     </x:row>
     <x:row r="73" ht="15.75" customHeight="1">
       <x:c r="A73" s="20" t="s">
-        <x:v>201</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="B73" s="21" t="s">
-        <x:v>202</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="C73" s="23" t="s">
         <x:v>8</x:v>
@@ -4507,10 +4485,10 @@
     </x:row>
     <x:row r="74" ht="15.75" customHeight="1">
       <x:c r="A74" s="16" t="s">
-        <x:v>203</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="B74" s="17" t="s">
-        <x:v>204</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C74" s="23" t="s">
         <x:v>8</x:v>
@@ -4523,7 +4501,7 @@
     </x:row>
     <x:row r="75" ht="15.75" customHeight="1">
       <x:c r="A75" s="20" t="s">
-        <x:v>205</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="B75" s="17" t="inlineStr">
         <x:is>
@@ -4543,10 +4521,10 @@
     </x:row>
     <x:row r="76" ht="15.75" customHeight="1">
       <x:c r="A76" s="16" t="s">
-        <x:v>206</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="B76" s="17" t="s">
-        <x:v>207</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="C76" s="23" t="inlineStr">
         <x:is>
@@ -4561,7 +4539,7 @@
     </x:row>
     <x:row r="77" ht="15.75" customHeight="1">
       <x:c r="A77" s="20" t="s">
-        <x:v>208</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="B77" s="17" t="inlineStr">
         <x:is>
@@ -4579,94 +4557,94 @@
     </x:row>
     <x:row r="78" ht="15.75" customHeight="1">
       <x:c r="A78" s="16" t="s">
-        <x:v>209</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="B78" s="17" t="s">
-        <x:v>210</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="C78" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D78" s="19" t="s">
-        <x:v>211</x:v>
+        <x:v>209</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="15.75" customHeight="1">
       <x:c r="A79" s="20" t="s">
-        <x:v>212</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="B79" s="21" t="s">
-        <x:v>213</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C79" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D79" s="22" t="s">
-        <x:v>214</x:v>
+        <x:v>212</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="15.75" customHeight="1">
       <x:c r="A80" s="16" t="s">
-        <x:v>215</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="B80" s="17" t="s">
-        <x:v>216</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="C80" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D80" s="19" t="s">
-        <x:v>217</x:v>
+        <x:v>215</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="15.75" customHeight="1">
       <x:c r="A81" s="20" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="B81" s="21" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="C81" s="18" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D81" s="22" t="s">
-        <x:v>220</x:v>
+        <x:v>218</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="15.75" customHeight="1">
       <x:c r="A82" s="16" t="s">
-        <x:v>221</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="B82" s="17" t="s">
-        <x:v>222</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="C82" s="18" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D82" s="19" t="s">
-        <x:v>223</x:v>
+        <x:v>221</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="15.75" customHeight="1">
       <x:c r="A83" s="20" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="B83" s="21" t="s">
-        <x:v>225</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="C83" s="18" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D83" s="22" t="s">
-        <x:v>226</x:v>
+        <x:v>224</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="30.75" customHeight="1">
       <x:c r="A84" s="16" t="s">
-        <x:v>227</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="B84" s="17" t="s">
-        <x:v>228</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="C84" s="23" t="inlineStr">
         <x:is>
@@ -4681,21 +4659,21 @@
     </x:row>
     <x:row r="85" ht="18.75" customHeight="1">
       <x:c r="A85" s="25" t="s">
-        <x:v>229</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="B85" s="26" t="s">
-        <x:v>230</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="C85" s="18" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D85" s="27" t="s">
-        <x:v>231</x:v>
+        <x:v>229</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="15.75" customHeight="1">
       <x:c r="A86" s="15" t="s">
-        <x:v>232</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="B86" s="2"/>
       <x:c r="C86" s="2"/>
@@ -4703,91 +4681,91 @@
     </x:row>
     <x:row r="87" ht="15.75" customHeight="1">
       <x:c r="A87" s="16" t="s">
-        <x:v>233</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="B87" s="17" t="s">
-        <x:v>234</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="C87" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D87" s="19" t="s">
-        <x:v>235</x:v>
+        <x:v>233</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="15.75" customHeight="1">
       <x:c r="A88" s="20" t="s">
-        <x:v>236</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="B88" s="21" t="s">
-        <x:v>237</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C88" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D88" s="22" t="s">
-        <x:v>238</x:v>
+        <x:v>236</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="15.75" customHeight="1">
       <x:c r="A89" s="16" t="s">
-        <x:v>239</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="B89" s="17" t="s">
-        <x:v>240</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="C89" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D89" s="19" t="s">
-        <x:v>241</x:v>
+        <x:v>239</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="15.75" customHeight="1">
       <x:c r="A90" s="20" t="s">
-        <x:v>242</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="B90" s="21" t="s">
-        <x:v>243</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="C90" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D90" s="22" t="s">
-        <x:v>244</x:v>
+        <x:v>242</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="15.75" customHeight="1">
       <x:c r="A91" s="16" t="s">
-        <x:v>245</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="B91" s="17" t="s">
-        <x:v>246</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="C91" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D91" s="19" t="s">
-        <x:v>247</x:v>
+        <x:v>245</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="27.75" customHeight="1">
       <x:c r="A92" s="28" t="s">
-        <x:v>248</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="B92" s="29" t="s">
-        <x:v>249</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="C92" s="30" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D92" s="31" t="s">
-        <x:v>250</x:v>
+        <x:v>248</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="15.75" customHeight="1">
       <x:c r="A93" s="15" t="s">
-        <x:v>251</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="B93" s="2"/>
       <x:c r="C93" s="2"/>
@@ -4795,10 +4773,10 @@
     </x:row>
     <x:row r="94" ht="15.75" customHeight="1">
       <x:c r="A94" s="32" t="s">
-        <x:v>252</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="B94" s="33" t="s">
-        <x:v>253</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="C94" s="24" t="inlineStr">
         <x:is>
@@ -4813,10 +4791,10 @@
     </x:row>
     <x:row r="95" ht="15.75" customHeight="1">
       <x:c r="A95" s="20" t="s">
-        <x:v>254</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="B95" s="21" t="s">
-        <x:v>255</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="C95" s="24" t="inlineStr">
         <x:is>
@@ -4831,10 +4809,10 @@
     </x:row>
     <x:row r="96" ht="15.75" customHeight="1">
       <x:c r="A96" s="16" t="s">
-        <x:v>256</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="B96" s="17" t="s">
-        <x:v>257</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="C96" s="24" t="s">
         <x:v>7</x:v>
@@ -4847,66 +4825,66 @@
     </x:row>
     <x:row r="97" ht="15.75" customHeight="1">
       <x:c r="A97" s="20" t="s">
-        <x:v>258</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="B97" s="21" t="s">
-        <x:v>259</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="C97" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D97" s="22" t="s">
-        <x:v>260</x:v>
+        <x:v>258</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="15.75" customHeight="1">
       <x:c r="A98" s="16" t="s">
-        <x:v>261</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="B98" s="17" t="s">
-        <x:v>262</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="C98" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D98" s="19" t="s">
-        <x:v>263</x:v>
+        <x:v>261</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="15.75" customHeight="1">
       <x:c r="A99" s="20" t="s">
-        <x:v>264</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="B99" s="21" t="s">
-        <x:v>265</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="C99" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D99" s="22" t="s">
-        <x:v>266</x:v>
+        <x:v>264</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="15.75" customHeight="1">
       <x:c r="A100" s="16" t="s">
-        <x:v>267</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="B100" s="17" t="s">
-        <x:v>268</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="C100" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D100" s="19" t="s">
-        <x:v>269</x:v>
+        <x:v>267</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="15.75" customHeight="1">
       <x:c r="A101" s="20" t="s">
-        <x:v>270</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="B101" s="21" t="s">
-        <x:v>271</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="C101" s="23" t="inlineStr">
         <x:is>
@@ -4921,10 +4899,10 @@
     </x:row>
     <x:row r="102" ht="15.75" customHeight="1">
       <x:c r="A102" s="16" t="s">
-        <x:v>272</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="B102" s="17" t="s">
-        <x:v>273</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="C102" s="24" t="s">
         <x:v>7</x:v>
@@ -4937,225 +4915,225 @@
     </x:row>
     <x:row r="103" ht="15.75" customHeight="1">
       <x:c r="A103" s="20" t="s">
-        <x:v>274</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="B103" s="21" t="s">
-        <x:v>275</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="C103" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D103" s="22" t="s">
-        <x:v>276</x:v>
+        <x:v>274</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="27.75" customHeight="1">
       <x:c r="A104" s="36" t="s">
-        <x:v>277</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="B104" s="37" t="s">
-        <x:v>278</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="C104" s="30" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D104" s="38" t="s">
-        <x:v>279</x:v>
+        <x:v>277</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="15.75" customHeight="1">
       <x:c r="A105" s="15" t="s">
-        <x:v>280</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="B105" s="2"/>
       <x:c r="C105" s="2"/>
       <x:c r="D105" s="3"/>
     </x:row>
     <x:row r="106" ht="15.75" customHeight="1">
-      <x:c r="A106" s="32" t="s">
-        <x:v>281</x:v>
-      </x:c>
-      <x:c r="B106" s="33" t="s">
-        <x:v>282</x:v>
+      <x:c r="A106" s="32" t="str">
+        <x:v>Build private operations application</x:v>
+      </x:c>
+      <x:c r="B106" s="33" t="str">
+        <x:v>Deploy a separately hosted private operations app; do not expose /admin in the public Pumdoki web app. Enforce ADMIN permissions in the API and apply separate operational access controls.</x:v>
       </x:c>
       <x:c r="C106" s="39" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D106" s="35" t="s">
-        <x:v>283</x:v>
+      <x:c r="D106" s="35" t="str">
+        <x:v>Founder decision 2026-08-01: public /admin removed; backend ADMIN role retained; independent apps/admin shell exists, while operational workflows remain Phase 11.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="15.75" customHeight="1">
       <x:c r="A107" s="20" t="s">
-        <x:v>284</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="B107" s="21" t="s">
-        <x:v>285</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="C107" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D107" s="22" t="s">
-        <x:v>286</x:v>
+        <x:v>281</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="15.75" customHeight="1">
       <x:c r="A108" s="16" t="s">
-        <x:v>287</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="B108" s="17" t="s">
-        <x:v>288</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="C108" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D108" s="19" t="s">
-        <x:v>289</x:v>
+        <x:v>284</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="15.75" customHeight="1">
       <x:c r="A109" s="20" t="s">
-        <x:v>290</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="B109" s="21" t="s">
-        <x:v>291</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="C109" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D109" s="22" t="s">
-        <x:v>292</x:v>
+        <x:v>287</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="15.75" customHeight="1">
       <x:c r="A110" s="16" t="s">
-        <x:v>293</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="B110" s="17" t="s">
-        <x:v>294</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="C110" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D110" s="19" t="s">
-        <x:v>295</x:v>
+        <x:v>290</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="15.75" customHeight="1">
       <x:c r="A111" s="20" t="s">
-        <x:v>296</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="B111" s="21" t="s">
-        <x:v>297</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="C111" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D111" s="22" t="s">
-        <x:v>298</x:v>
+        <x:v>293</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="15.75" customHeight="1">
       <x:c r="A112" s="16" t="s">
-        <x:v>299</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="B112" s="17" t="s">
-        <x:v>300</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="C112" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D112" s="19" t="s">
-        <x:v>301</x:v>
+        <x:v>296</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="15.75" customHeight="1">
       <x:c r="A113" s="20" t="s">
-        <x:v>302</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="B113" s="21" t="s">
-        <x:v>303</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="C113" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D113" s="22" t="s">
-        <x:v>304</x:v>
+        <x:v>299</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="15.75" customHeight="1">
       <x:c r="A114" s="16" t="s">
-        <x:v>305</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="B114" s="17" t="s">
-        <x:v>306</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="C114" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D114" s="19" t="s">
-        <x:v>307</x:v>
+        <x:v>302</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="15.75" customHeight="1">
       <x:c r="A115" s="20" t="s">
-        <x:v>308</x:v>
+        <x:v>303</x:v>
       </x:c>
       <x:c r="B115" s="21" t="s">
-        <x:v>309</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="C115" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D115" s="22" t="s">
-        <x:v>310</x:v>
+        <x:v>305</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="15.75" customHeight="1">
       <x:c r="A116" s="16" t="s">
-        <x:v>311</x:v>
+        <x:v>306</x:v>
       </x:c>
       <x:c r="B116" s="17" t="s">
-        <x:v>312</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="C116" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D116" s="19" t="s">
-        <x:v>313</x:v>
+        <x:v>308</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="15.75" customHeight="1">
       <x:c r="A117" s="20" t="s">
-        <x:v>314</x:v>
+        <x:v>309</x:v>
       </x:c>
       <x:c r="B117" s="21" t="s">
-        <x:v>315</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="C117" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D117" s="22" t="s">
-        <x:v>316</x:v>
+        <x:v>311</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="27.75" customHeight="1">
       <x:c r="A118" s="36" t="s">
-        <x:v>317</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="B118" s="37" t="s">
-        <x:v>318</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="C118" s="30" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D118" s="38" t="s">
-        <x:v>319</x:v>
+        <x:v>314</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="15.75" customHeight="1">
       <x:c r="A119" s="15" t="s">
-        <x:v>320</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="B119" s="2"/>
       <x:c r="C119" s="2"/>
@@ -5163,10 +5141,10 @@
     </x:row>
     <x:row r="120" ht="15.75" customHeight="1">
       <x:c r="A120" s="32" t="s">
-        <x:v>321</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="B120" s="33" t="s">
-        <x:v>322</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="C120" s="39" t="s">
         <x:v>7</x:v>
@@ -5177,52 +5155,52 @@
     </x:row>
     <x:row r="121" ht="15.75" customHeight="1">
       <x:c r="A121" s="20" t="s">
-        <x:v>323</x:v>
+        <x:v>318</x:v>
       </x:c>
       <x:c r="B121" s="21" t="s">
-        <x:v>324</x:v>
+        <x:v>319</x:v>
       </x:c>
       <x:c r="C121" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D121" s="22" t="s">
-        <x:v>325</x:v>
+        <x:v>320</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="15.75" customHeight="1">
       <x:c r="A122" s="16" t="s">
-        <x:v>326</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="B122" s="17" t="s">
-        <x:v>327</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="C122" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D122" s="19" t="s">
-        <x:v>328</x:v>
+        <x:v>323</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="15.75" customHeight="1">
       <x:c r="A123" s="20" t="s">
-        <x:v>329</x:v>
+        <x:v>324</x:v>
       </x:c>
       <x:c r="B123" s="21" t="s">
-        <x:v>330</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="C123" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D123" s="22" t="s">
-        <x:v>331</x:v>
+        <x:v>326</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="27.75" customHeight="1">
       <x:c r="A124" s="36" t="s">
-        <x:v>332</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="B124" s="37" t="s">
-        <x:v>333</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="C124" s="30" t="s">
         <x:v>7</x:v>
@@ -5235,7 +5213,7 @@
     </x:row>
     <x:row r="125" ht="15.75" customHeight="1">
       <x:c r="A125" s="15" t="s">
-        <x:v>334</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="B125" s="2"/>
       <x:c r="C125" s="2"/>
@@ -5243,105 +5221,105 @@
     </x:row>
     <x:row r="126" ht="15.75" customHeight="1">
       <x:c r="A126" s="32" t="s">
-        <x:v>335</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="B126" s="33" t="s">
-        <x:v>336</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="C126" s="39" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D126" s="35" t="s">
-        <x:v>337</x:v>
+        <x:v>332</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="15.75" customHeight="1">
       <x:c r="A127" s="20" t="s">
-        <x:v>338</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="B127" s="21" t="s">
-        <x:v>339</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="C127" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D127" s="22" t="s">
-        <x:v>340</x:v>
+        <x:v>335</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="15.75" customHeight="1">
       <x:c r="A128" s="16" t="s">
-        <x:v>341</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="B128" s="17" t="s">
-        <x:v>342</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="C128" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D128" s="19" t="s">
-        <x:v>343</x:v>
+        <x:v>338</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="15.75" customHeight="1">
       <x:c r="A129" s="20" t="s">
-        <x:v>344</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="B129" s="21" t="s">
-        <x:v>345</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="C129" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D129" s="22" t="s">
-        <x:v>346</x:v>
+        <x:v>341</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="15.75" customHeight="1">
       <x:c r="A130" s="16" t="s">
-        <x:v>347</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="B130" s="17" t="s">
-        <x:v>348</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="C130" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D130" s="19" t="s">
-        <x:v>349</x:v>
+        <x:v>344</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="15" customHeight="1">
       <x:c r="A131" s="20" t="s">
-        <x:v>350</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="B131" s="21" t="s">
-        <x:v>351</x:v>
+        <x:v>346</x:v>
       </x:c>
       <x:c r="C131" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D131" s="22" t="s">
-        <x:v>352</x:v>
+        <x:v>347</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="15.75" customHeight="1">
       <x:c r="A132" s="40" t="s">
-        <x:v>353</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="B132" s="41" t="s">
-        <x:v>354</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="C132" s="42" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="D132" s="43" t="s">
-        <x:v>349</x:v>
+        <x:v>344</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="15.75" customHeight="1">
       <x:c r="A133" s="15" t="s">
-        <x:v>355</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="B133" s="2"/>
       <x:c r="C133" s="2"/>
@@ -5349,114 +5327,114 @@
     </x:row>
     <x:row r="134" ht="15.75" customHeight="1">
       <x:c r="A134" s="32" t="s">
-        <x:v>356</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="B134" s="33" t="s">
-        <x:v>357</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="C134" s="44" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="D134" s="35" t="s">
-        <x:v>358</x:v>
+        <x:v>353</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="15.75" customHeight="1">
       <x:c r="A135" s="20" t="s">
-        <x:v>359</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="B135" s="21" t="s">
-        <x:v>360</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="C135" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D135" s="22" t="s">
-        <x:v>361</x:v>
+        <x:v>356</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="15.75" customHeight="1">
       <x:c r="A136" s="16" t="s">
-        <x:v>362</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="B136" s="17" t="s">
-        <x:v>363</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="C136" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D136" s="19" t="s">
-        <x:v>364</x:v>
+        <x:v>359</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="15.75" customHeight="1">
       <x:c r="A137" s="20" t="s">
-        <x:v>365</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="B137" s="21" t="s">
-        <x:v>366</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="C137" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D137" s="22" t="s">
-        <x:v>349</x:v>
+        <x:v>344</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="15.75" customHeight="1">
       <x:c r="A138" s="16" t="s">
-        <x:v>367</x:v>
+        <x:v>362</x:v>
       </x:c>
       <x:c r="B138" s="17" t="s">
-        <x:v>368</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="C138" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D138" s="19" t="s">
-        <x:v>369</x:v>
+        <x:v>364</x:v>
       </x:c>
     </x:row>
     <x:row r="139" ht="15.75" customHeight="1">
       <x:c r="A139" s="20" t="s">
-        <x:v>370</x:v>
+        <x:v>365</x:v>
       </x:c>
       <x:c r="B139" s="21" t="s">
-        <x:v>371</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="C139" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D139" s="22" t="s">
-        <x:v>372</x:v>
+        <x:v>367</x:v>
       </x:c>
     </x:row>
     <x:row r="140" ht="15.75" customHeight="1">
       <x:c r="A140" s="16" t="s">
-        <x:v>373</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="B140" s="17" t="s">
-        <x:v>374</x:v>
+        <x:v>369</x:v>
       </x:c>
       <x:c r="C140" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D140" s="19" t="s">
-        <x:v>375</x:v>
+        <x:v>370</x:v>
       </x:c>
     </x:row>
     <x:row r="141" ht="15.75" customHeight="1">
       <x:c r="A141" s="20" t="s">
-        <x:v>376</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="B141" s="21" t="s">
-        <x:v>377</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="C141" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D141" s="22" t="s">
-        <x:v>378</x:v>
+        <x:v>373</x:v>
       </x:c>
     </x:row>
     <x:row r="142" ht="27.75" customHeight="1">
@@ -5842,15 +5820,11 @@
       </x:c>
     </x:row>
     <x:row r="160" ht="24" hidden="0" customHeight="1">
-      <x:c r="A160" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Define MVP Admin architecture</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B160" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build protected /admin routes inside the web app with API-enforced roles, sensitive permissions, and immutable audit logs.</x:t>
-        </x:is>
+      <x:c r="A160" s="20" t="str">
+        <x:v>Define private operations architecture</x:v>
+      </x:c>
+      <x:c r="B160" s="21" t="str">
+        <x:v>Build a separately deployed private operations application with API-enforced ADMIN permissions, stronger access controls, sensitive-record permissions, and immutable audit logging.</x:v>
       </x:c>
       <x:c r="C160" s="23" t="inlineStr">
         <x:is>
@@ -5858,7 +5832,7 @@
         </x:is>
       </x:c>
       <x:c r="D160" s="22" t="str">
-        <x:v>Recommended protected /admin architecture is documented in PLAN.md. API role enforcement now exists, but admin routes, sensitive permissions, and audit logging remain pending.</x:v>
+        <x:v>The apps/admin build shell now exists. Operational authentication, MFA/SSO, restricted hosting, API integration, permissions, and audit tooling remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="24" hidden="0" customHeight="1">
@@ -5878,7 +5852,7 @@
         </x:is>
       </x:c>
       <x:c r="D161" s="19" t="str">
-        <x:v>TypeScript API/contracts/database foundation now includes core auth, email verification/password reset, mail transports, and DB-backed tests. The JavaScript frontend remains unchanged until slice 3 integration.</x:v>
+        <x:v>The TypeScript API/contracts/database foundation and the React frontend now include core auth, email verification/password reset, role guards, and DB-backed/browser tests. Remaining frontend migration is incremental.</x:v>
       </x:c>
     </x:row>
     <x:row r="162" ht="31.5" customHeight="1">
@@ -6820,50 +6794,50 @@
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
       <x:c r="A1" s="14" t="s">
-        <x:v>379</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="B1" s="14" t="s">
-        <x:v>380</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="C1" s="14" t="s">
-        <x:v>381</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="D1" s="14" t="s">
-        <x:v>382</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="E1" s="14" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="F1" s="14" t="s">
-        <x:v>383</x:v>
+        <x:v>378</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="20" t="s">
-        <x:v>384</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="B2" s="21" t="s">
-        <x:v>385</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="C2" s="21" t="s">
-        <x:v>386</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="D2" s="21" t="s">
-        <x:v>387</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="E2" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F2" s="21" t="s">
-        <x:v>388</x:v>
+        <x:v>383</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="16" t="s">
-        <x:v>389</x:v>
+        <x:v>384</x:v>
       </x:c>
       <x:c r="B3" s="17" t="s">
-        <x:v>385</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="C3" s="21" t="inlineStr">
         <x:is>
@@ -6871,7 +6845,7 @@
         </x:is>
       </x:c>
       <x:c r="D3" s="17" t="s">
-        <x:v>387</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="E3" s="24" t="s">
         <x:v>7</x:v>
@@ -6884,10 +6858,10 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="20" t="s">
-        <x:v>390</x:v>
+        <x:v>385</x:v>
       </x:c>
       <x:c r="B4" s="21" t="s">
-        <x:v>391</x:v>
+        <x:v>386</x:v>
       </x:c>
       <x:c r="C4" s="21" t="inlineStr">
         <x:is>
@@ -6912,10 +6886,10 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="16" t="s">
-        <x:v>392</x:v>
+        <x:v>387</x:v>
       </x:c>
       <x:c r="B5" s="17" t="s">
-        <x:v>391</x:v>
+        <x:v>386</x:v>
       </x:c>
       <x:c r="C5" s="17" t="inlineStr">
         <x:is>
@@ -6940,70 +6914,70 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="20" t="s">
-        <x:v>393</x:v>
+        <x:v>388</x:v>
       </x:c>
       <x:c r="B6" s="21" t="s">
-        <x:v>394</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="C6" s="21" t="s">
-        <x:v>395</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="D6" s="21" t="s">
-        <x:v>387</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="E6" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F6" s="21" t="s">
-        <x:v>388</x:v>
+        <x:v>383</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="16" t="s">
-        <x:v>396</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="B7" s="17" t="s">
-        <x:v>397</x:v>
+        <x:v>392</x:v>
       </x:c>
       <x:c r="C7" s="17" t="s">
-        <x:v>398</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="D7" s="17" t="s">
-        <x:v>399</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="E7" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F7" s="17" t="s">
-        <x:v>388</x:v>
+        <x:v>383</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="20" t="s">
-        <x:v>400</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="B8" s="21" t="s">
-        <x:v>401</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="C8" s="21" t="s">
-        <x:v>402</x:v>
+        <x:v>397</x:v>
       </x:c>
       <x:c r="D8" s="21" t="s">
-        <x:v>399</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="E8" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F8" s="21" t="s">
-        <x:v>403</x:v>
+        <x:v>398</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="16" t="s">
-        <x:v>404</x:v>
+        <x:v>399</x:v>
       </x:c>
       <x:c r="B9" s="17" t="s">
-        <x:v>385</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="C9" s="17" t="inlineStr">
         <x:is>
@@ -7028,162 +7002,162 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="20" t="s">
-        <x:v>405</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="B10" s="21" t="s">
-        <x:v>391</x:v>
+        <x:v>386</x:v>
       </x:c>
       <x:c r="C10" s="21" t="s">
-        <x:v>406</x:v>
+        <x:v>401</x:v>
       </x:c>
       <x:c r="D10" s="21" t="s">
-        <x:v>387</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="E10" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F10" s="21" t="s">
-        <x:v>407</x:v>
+        <x:v>402</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="16" t="s">
-        <x:v>408</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="B11" s="17" t="s">
-        <x:v>391</x:v>
+        <x:v>386</x:v>
       </x:c>
       <x:c r="C11" s="17" t="s">
-        <x:v>409</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="D11" s="17" t="s">
-        <x:v>387</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="E11" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F11" s="17" t="s">
-        <x:v>410</x:v>
+        <x:v>405</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="20" t="s">
-        <x:v>411</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B12" s="21" t="s">
-        <x:v>412</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="C12" s="21" t="s">
-        <x:v>413</x:v>
+        <x:v>408</x:v>
       </x:c>
       <x:c r="D12" s="21" t="s">
-        <x:v>387</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="E12" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F12" s="21" t="s">
-        <x:v>414</x:v>
+        <x:v>409</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="16" t="s">
-        <x:v>415</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="B13" s="17" t="s">
-        <x:v>416</x:v>
+        <x:v>411</x:v>
       </x:c>
       <x:c r="C13" s="17" t="s">
-        <x:v>417</x:v>
+        <x:v>412</x:v>
       </x:c>
       <x:c r="D13" s="17" t="s">
-        <x:v>418</x:v>
+        <x:v>413</x:v>
       </x:c>
       <x:c r="E13" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F13" s="17" t="s">
-        <x:v>419</x:v>
+        <x:v>414</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="20" t="s">
-        <x:v>420</x:v>
+        <x:v>415</x:v>
       </x:c>
       <x:c r="B14" s="21" t="s">
-        <x:v>421</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="C14" s="21" t="s">
-        <x:v>422</x:v>
+        <x:v>417</x:v>
       </x:c>
       <x:c r="D14" s="21" t="s">
-        <x:v>399</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="E14" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F14" s="21" t="s">
-        <x:v>423</x:v>
+        <x:v>418</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="45" t="s">
-        <x:v>424</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="B15" s="46" t="s">
-        <x:v>425</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="C15" s="47" t="s">
-        <x:v>426</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="D15" s="46" t="s">
-        <x:v>387</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="E15" s="48" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F15" s="47" t="s">
-        <x:v>427</x:v>
+        <x:v>422</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="49" t="s">
-        <x:v>428</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="B16" s="50" t="s">
-        <x:v>429</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="C16" s="51" t="s">
-        <x:v>430</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="D16" s="50" t="s">
-        <x:v>399</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="E16" s="48" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F16" s="51" t="s">
-        <x:v>431</x:v>
+        <x:v>426</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="52" t="s">
-        <x:v>432</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="B17" s="53" t="s">
-        <x:v>401</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="C17" s="54" t="s">
-        <x:v>433</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="D17" s="53" t="s">
-        <x:v>399</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="E17" s="48" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F17" s="54" t="s">
-        <x:v>434</x:v>
+        <x:v>429</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1"/>
@@ -8182,21 +8156,21 @@
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>435</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="14" t="s">
-        <x:v>436</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="B3" s="14" t="s">
-        <x:v>437</x:v>
+        <x:v>432</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="55" t="s">
-        <x:v>438</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="B4" s="58" t="str">
         <x:v>This workbook is reconciled with the repository and founder decisions through July 16, 2026.</x:v>
@@ -8204,284 +8178,284 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="57" t="s">
-        <x:v>439</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="B5" s="58" t="s">
-        <x:v>440</x:v>
+        <x:v>435</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="55" t="s">
-        <x:v>441</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="B6" s="56" t="s">
-        <x:v>442</x:v>
+        <x:v>437</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="57" t="s">
-        <x:v>443</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="B7" s="58" t="s">
-        <x:v>444</x:v>
+        <x:v>439</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="55" t="s">
-        <x:v>445</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="B8" s="56" t="s">
-        <x:v>446</x:v>
+        <x:v>441</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="57" t="s">
-        <x:v>447</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="B9" s="58" t="s">
-        <x:v>448</x:v>
+        <x:v>443</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="55" t="s">
-        <x:v>449</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="B10" s="56" t="s">
-        <x:v>450</x:v>
+        <x:v>445</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="57" t="s">
-        <x:v>451</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="B11" s="58" t="s">
-        <x:v>452</x:v>
+        <x:v>447</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="55" t="s">
-        <x:v>453</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="B12" s="56" t="s">
-        <x:v>454</x:v>
+        <x:v>449</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="57" t="s">
-        <x:v>455</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="B13" s="58" t="s">
-        <x:v>456</x:v>
+        <x:v>451</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="55" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B14" s="56" t="s">
-        <x:v>458</x:v>
+        <x:v>453</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="57" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="B15" s="58" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="5" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B18" s="60" t="s">
-        <x:v>463</x:v>
+        <x:v>458</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B19" s="60" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B20" s="60" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1">
       <x:c r="A21" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B21" s="60" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15.75" customHeight="1">
       <x:c r="A22" s="59" t="s">
+        <x:v>457</x:v>
+      </x:c>
+      <x:c r="B22" s="60" t="s">
         <x:v>462</x:v>
-      </x:c>
-      <x:c r="B22" s="60" t="s">
-        <x:v>467</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15.75" customHeight="1">
       <x:c r="A23" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B23" s="60" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15.75" customHeight="1">
       <x:c r="A24" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B24" s="60" t="s">
-        <x:v>469</x:v>
+        <x:v>464</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15.75" customHeight="1">
       <x:c r="A25" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B25" s="60" t="s">
-        <x:v>470</x:v>
+        <x:v>465</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15.75" customHeight="1">
       <x:c r="A26" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B26" s="60" t="s">
-        <x:v>471</x:v>
+        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15.75" customHeight="1">
       <x:c r="A27" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B27" s="60" t="s">
-        <x:v>472</x:v>
+        <x:v>467</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15.75" customHeight="1">
       <x:c r="A28" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B28" s="60" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15.75" customHeight="1">
       <x:c r="A29" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B29" s="60" t="s">
-        <x:v>474</x:v>
+        <x:v>469</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15.75" customHeight="1">
       <x:c r="A30" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B30" s="60" t="s">
-        <x:v>475</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="15.75" customHeight="1">
+        <x:v>470</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="30" customHeight="1">
       <x:c r="A31" s="59" t="s">
-        <x:v>462</x:v>
-      </x:c>
-      <x:c r="B31" s="60" t="s">
-        <x:v>476</x:v>
+        <x:v>457</x:v>
+      </x:c>
+      <x:c r="B31" s="60" t="str">
+        <x:v>Admin operations: separately deployed private app; no public /admin. Backend ADMIN permissions remain API-enforced. 13 subtasks defined.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15.75" customHeight="1">
       <x:c r="A32" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B32" s="60" t="s">
-        <x:v>477</x:v>
+        <x:v>471</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15.75" customHeight="1">
       <x:c r="A33" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B33" s="60" t="s">
-        <x:v>478</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15.75" customHeight="1">
       <x:c r="A34" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B34" s="60" t="s">
-        <x:v>479</x:v>
+        <x:v>473</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15.75" customHeight="1">
       <x:c r="A35" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B35" s="60" t="s">
-        <x:v>480</x:v>
+        <x:v>474</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15.75" customHeight="1">
       <x:c r="A36" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B36" s="60" t="s">
-        <x:v>481</x:v>
+        <x:v>475</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15.75" customHeight="1">
       <x:c r="A37" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B37" s="60" t="s">
-        <x:v>482</x:v>
+        <x:v>476</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15.75" customHeight="1">
       <x:c r="A38" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B38" s="60" t="s">
-        <x:v>483</x:v>
+        <x:v>477</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15.75" customHeight="1">
       <x:c r="A39" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B39" s="60" t="s">
-        <x:v>484</x:v>
+        <x:v>478</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15.75" customHeight="1">
       <x:c r="A40" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B40" s="60" t="s">
-        <x:v>485</x:v>
+        <x:v>479</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15.75" customHeight="1">
       <x:c r="A41" s="59" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B41" s="60" t="inlineStr">
         <x:is>
@@ -8504,7 +8478,7 @@
         </x:is>
       </x:c>
       <x:c r="B44" s="71" t="str">
-        <x:v>The dependency-ordered roadmap remains in repository PLAN.md. Phase 1 is verified, Phase 2 is partially complete, and Phase 3 is split into four independently verified slices; slices 1–2 are locally verified.</x:v>
+        <x:v>The architecture plan source of truth is PLAN.md. Phase 3 is split into four slices: Slices 1–3 are implemented and locally verified; Slice 4 remains.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -8514,7 +8488,7 @@
         </x:is>
       </x:c>
       <x:c r="B45" s="73" t="str">
-        <x:v>Phase 3 slice 2 email verification and password reset are implemented and locally verified with provider-neutral mail, Mailpit, single-use hashed tokens, session revocation, and DB-backed tests. Next engineering slice: frontend auth integration.</x:v>
+        <x:v>Phase 3 Slices 1–3 are complete locally. The next implementation slice is Settings and explicit-content controls.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -8554,7 +8528,7 @@
         </x:is>
       </x:c>
       <x:c r="B49" s="73" t="str">
-        <x:v>Local verification is recorded in HANDOFF.md. Publication to the confirmed public repository is pending the required GitHub CLI/authentication prerequisite and CI verification.</x:v>
+        <x:v>Slice 2 was published to origin/dev and CI passed on July 29, 2026. Slice 3 is implemented and locally verified but not yet published.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
@@ -8616,7 +8590,7 @@
         <x:v>•</x:v>
       </x:c>
       <x:c r="B58" s="79" t="str">
-        <x:v>Phase 3 slices 1–2 are backend-only; no real frontend authentication behavior is claimed yet.</x:v>
+        <x:v>Slice 3 connects the frontend to live auth APIs, including persistent cookie sessions, verification, password reset, role guards, and logout.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
@@ -8632,7 +8606,7 @@
         <x:v>•</x:v>
       </x:c>
       <x:c r="B60" s="79" t="str">
-        <x:v>Email verification and password reset are implemented locally. Frontend auth, Settings, OAuth, a production email provider, and Redis-backed throttling remain later slices or deferred work.</x:v>
+        <x:v>Email verification, password reset, and frontend auth integration are implemented locally. Settings, OAuth, a production email provider, and Redis-backed throttling remain later work.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
@@ -8666,7 +8640,7 @@
         <x:v>•</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>Production email provider selection and deliverability controls remain open; Phase 3 slice 3 is frontend authentication integration.</x:v>
+        <x:v>Phase 3 Slice 3 is locally verified. Slice 4 (Settings and explicit-content controls) is the next planned implementation step.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15.75" customHeight="1">
@@ -8820,16 +8794,14 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="79" ht="28.5" customHeight="1">
+    <x:row r="79" ht="30" customHeight="1">
       <x:c r="A79" s="65" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">•</x:t>
         </x:is>
       </x:c>
-      <x:c r="B79" s="66" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Recommended Admin: protected /admin feature inside the web app for MVP, enforced by API roles.</x:t>
-        </x:is>
+      <x:c r="B79" s="66" t="str">
+        <x:v>Founder decision (2026-08-01): no public /admin route. An independent apps/admin build shell now exists; backend ADMIN authorization remains, while operational access controls and workflows are Phase 11.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="28.5" customHeight="1">
@@ -9969,7 +9941,7 @@
   <x:sheetData>
     <x:row r="1" ht="39.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>486</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -9981,7 +9953,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="13" t="s">
-        <x:v>487</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -9993,22 +9965,22 @@
     </x:row>
     <x:row r="3" ht="25.5" customHeight="1">
       <x:c r="A3" s="68" t="s">
-        <x:v>488</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="B3" s="68" t="s">
-        <x:v>380</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="C3" s="68" t="s">
-        <x:v>489</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="D3" s="68" t="s">
-        <x:v>490</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="E3" s="68" t="s">
-        <x:v>491</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="F3" s="68" t="s">
-        <x:v>492</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="G3" s="68" t="s">
         <x:v>22</x:v>
@@ -10019,7 +9991,7 @@
     </x:row>
     <x:row r="4" ht="25.5" customHeight="1">
       <x:c r="A4" s="15" t="s">
-        <x:v>493</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -10031,122 +10003,122 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="16" t="s">
-        <x:v>494</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="B5" s="17" t="s">
-        <x:v>495</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="C5" s="17" t="s">
-        <x:v>496</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="D5" s="17">
         <x:v>500.0</x:v>
       </x:c>
       <x:c r="E5" s="17"/>
       <x:c r="F5" s="17" t="s">
-        <x:v>497</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="G5" s="24" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H5" s="17" t="s">
-        <x:v>499</x:v>
+        <x:v>493</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="20" t="s">
-        <x:v>500</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="B6" s="21" t="s">
-        <x:v>495</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="C6" s="21" t="s">
-        <x:v>496</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="D6" s="21">
         <x:v>500.0</x:v>
       </x:c>
       <x:c r="E6" s="21"/>
       <x:c r="F6" s="21" t="s">
-        <x:v>497</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="G6" s="24" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H6" s="21" t="s">
-        <x:v>501</x:v>
+        <x:v>495</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="16" t="s">
-        <x:v>502</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="B7" s="17" t="s">
-        <x:v>495</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="C7" s="17" t="s">
-        <x:v>496</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="D7" s="17">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E7" s="17"/>
       <x:c r="F7" s="17" t="s">
+        <x:v>491</x:v>
+      </x:c>
+      <x:c r="G7" s="24" t="s">
+        <x:v>492</x:v>
+      </x:c>
+      <x:c r="H7" s="17" t="s">
         <x:v>497</x:v>
-      </x:c>
-      <x:c r="G7" s="24" t="s">
-        <x:v>498</x:v>
-      </x:c>
-      <x:c r="H7" s="17" t="s">
-        <x:v>503</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="20" t="s">
-        <x:v>504</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="B8" s="21" t="s">
-        <x:v>505</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="C8" s="21" t="s">
-        <x:v>496</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="D8" s="21">
         <x:v>350.0</x:v>
       </x:c>
       <x:c r="E8" s="21"/>
       <x:c r="F8" s="21" t="s">
-        <x:v>497</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="G8" s="24" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H8" s="21" t="s">
-        <x:v>506</x:v>
+        <x:v>500</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="16" t="s">
-        <x:v>507</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="B9" s="17" t="s">
-        <x:v>505</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="C9" s="17" t="s">
-        <x:v>496</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="D9" s="17">
         <x:v>350.0</x:v>
       </x:c>
       <x:c r="E9" s="17"/>
       <x:c r="F9" s="17" t="s">
-        <x:v>497</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="G9" s="24" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H9" s="17" t="s">
-        <x:v>508</x:v>
+        <x:v>502</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -10156,20 +10128,20 @@
         </x:is>
       </x:c>
       <x:c r="B10" s="21" t="s">
-        <x:v>505</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="C10" s="21" t="s">
-        <x:v>496</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="D10" s="21">
         <x:v>155.0</x:v>
       </x:c>
       <x:c r="E10" s="21"/>
       <x:c r="F10" s="21" t="s">
-        <x:v>497</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="G10" s="24" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H10" s="43" t="inlineStr">
         <x:is>
@@ -10179,103 +10151,103 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="25" t="s">
-        <x:v>509</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="B11" s="21" t="s">
-        <x:v>505</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="C11" s="21" t="s">
-        <x:v>496</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="D11" s="26">
         <x:v>125.0</x:v>
       </x:c>
       <x:c r="E11" s="21"/>
       <x:c r="F11" s="21" t="s">
-        <x:v>497</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="G11" s="24" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H11" s="26" t="s">
-        <x:v>510</x:v>
+        <x:v>504</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="16" t="s">
-        <x:v>511</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="B12" s="17" t="s">
-        <x:v>505</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="C12" s="17" t="s">
-        <x:v>512</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="D12" s="17">
         <x:v>125.0</x:v>
       </x:c>
       <x:c r="E12" s="17"/>
       <x:c r="F12" s="17" t="s">
-        <x:v>513</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="G12" s="24" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H12" s="17" t="s">
-        <x:v>514</x:v>
+        <x:v>508</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="20" t="s">
-        <x:v>515</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="B13" s="21" t="s">
-        <x:v>516</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="C13" s="21" t="s">
-        <x:v>512</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="D13" s="21">
         <x:v>15.0</x:v>
       </x:c>
       <x:c r="E13" s="21"/>
       <x:c r="F13" s="21" t="s">
-        <x:v>513</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="G13" s="24" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H13" s="21" t="s">
-        <x:v>517</x:v>
+        <x:v>511</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="16.5" customHeight="1">
       <x:c r="A14" s="16" t="s">
-        <x:v>518</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="B14" s="17" t="s">
-        <x:v>516</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="C14" s="17" t="s">
-        <x:v>512</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="D14" s="17">
         <x:v>30.0</x:v>
       </x:c>
       <x:c r="E14" s="17"/>
       <x:c r="F14" s="17" t="s">
+        <x:v>507</x:v>
+      </x:c>
+      <x:c r="G14" s="24" t="s">
+        <x:v>492</x:v>
+      </x:c>
+      <x:c r="H14" s="17" t="s">
         <x:v>513</x:v>
-      </x:c>
-      <x:c r="G14" s="24" t="s">
-        <x:v>498</x:v>
-      </x:c>
-      <x:c r="H14" s="17" t="s">
-        <x:v>519</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="15" t="s">
-        <x:v>520</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="B15" s="2"/>
       <x:c r="C15" s="2"/>
@@ -10287,175 +10259,175 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="32" t="s">
-        <x:v>521</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="B16" s="33" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="C16" s="33" t="s">
         <x:v>516</x:v>
-      </x:c>
-      <x:c r="C16" s="33" t="s">
-        <x:v>522</x:v>
       </x:c>
       <x:c r="D16" s="33">
         <x:v>18.0</x:v>
       </x:c>
       <x:c r="E16" s="33"/>
       <x:c r="F16" s="33" t="s">
-        <x:v>522</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="G16" s="39" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H16" s="33" t="s">
-        <x:v>523</x:v>
+        <x:v>517</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="20" t="s">
-        <x:v>524</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="B17" s="21" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="C17" s="21" t="s">
         <x:v>516</x:v>
-      </x:c>
-      <x:c r="C17" s="21" t="s">
-        <x:v>522</x:v>
       </x:c>
       <x:c r="D17" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E17" s="21"/>
       <x:c r="F17" s="21" t="s">
-        <x:v>522</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="G17" s="24" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H17" s="21" t="s">
-        <x:v>525</x:v>
+        <x:v>519</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="16" t="s">
-        <x:v>526</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="B18" s="17" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="C18" s="17" t="s">
         <x:v>516</x:v>
-      </x:c>
-      <x:c r="C18" s="17" t="s">
-        <x:v>522</x:v>
       </x:c>
       <x:c r="D18" s="17">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E18" s="17"/>
       <x:c r="F18" s="17" t="s">
-        <x:v>522</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="G18" s="24" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H18" s="17" t="s">
-        <x:v>527</x:v>
+        <x:v>521</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="20" t="s">
-        <x:v>528</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="B19" s="21" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="C19" s="21" t="s">
         <x:v>516</x:v>
-      </x:c>
-      <x:c r="C19" s="21" t="s">
-        <x:v>522</x:v>
       </x:c>
       <x:c r="D19" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E19" s="21"/>
       <x:c r="F19" s="21" t="s">
-        <x:v>522</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="G19" s="24" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H19" s="21" t="s">
-        <x:v>529</x:v>
+        <x:v>523</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="16" t="s">
-        <x:v>530</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="B20" s="17" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="C20" s="17" t="s">
         <x:v>516</x:v>
-      </x:c>
-      <x:c r="C20" s="17" t="s">
-        <x:v>522</x:v>
       </x:c>
       <x:c r="D20" s="17">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E20" s="17"/>
       <x:c r="F20" s="17" t="s">
-        <x:v>522</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="G20" s="24" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H20" s="17" t="s">
-        <x:v>531</x:v>
+        <x:v>525</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1">
       <x:c r="A21" s="20" t="s">
-        <x:v>532</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="B21" s="21" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="C21" s="21" t="s">
         <x:v>516</x:v>
-      </x:c>
-      <x:c r="C21" s="21" t="s">
-        <x:v>522</x:v>
       </x:c>
       <x:c r="D21" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E21" s="21"/>
       <x:c r="F21" s="21" t="s">
-        <x:v>522</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="G21" s="24" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H21" s="21" t="s">
-        <x:v>533</x:v>
+        <x:v>527</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="25.5" customHeight="1">
       <x:c r="A22" s="36" t="s">
-        <x:v>534</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="B22" s="37" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="C22" s="37" t="s">
         <x:v>516</x:v>
-      </x:c>
-      <x:c r="C22" s="37" t="s">
-        <x:v>522</x:v>
       </x:c>
       <x:c r="D22" s="37">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E22" s="37"/>
       <x:c r="F22" s="37" t="s">
-        <x:v>522</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="G22" s="30" t="s">
-        <x:v>498</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="H22" s="37" t="s">
-        <x:v>535</x:v>
+        <x:v>529</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15.75" customHeight="1">
       <x:c r="A23" s="15" t="s">
-        <x:v>536</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="B23" s="2"/>
       <x:c r="C23" s="2"/>
@@ -10467,79 +10439,79 @@
     </x:row>
     <x:row r="24" ht="15.75" customHeight="1">
       <x:c r="A24" s="32" t="s">
-        <x:v>537</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="B24" s="33" t="s">
-        <x:v>495</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="C24" s="33" t="s">
-        <x:v>538</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="D24" s="33">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E24" s="33"/>
       <x:c r="F24" s="33" t="s">
-        <x:v>539</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="G24" s="39" t="s">
-        <x:v>540</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="H24" s="33" t="s">
-        <x:v>541</x:v>
+        <x:v>535</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15.75" customHeight="1">
       <x:c r="A25" s="20" t="s">
-        <x:v>542</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="B25" s="21" t="s">
-        <x:v>495</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="C25" s="21" t="s">
-        <x:v>538</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="D25" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E25" s="21"/>
       <x:c r="F25" s="21" t="s">
-        <x:v>539</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="G25" s="24" t="s">
-        <x:v>540</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="H25" s="21" t="s">
-        <x:v>543</x:v>
+        <x:v>537</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="25.5" customHeight="1">
       <x:c r="A26" s="36" t="s">
-        <x:v>544</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="B26" s="37" t="s">
-        <x:v>495</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="C26" s="37" t="s">
-        <x:v>538</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="D26" s="37">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E26" s="37"/>
       <x:c r="F26" s="37" t="s">
-        <x:v>545</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="G26" s="30" t="s">
+        <x:v>534</x:v>
+      </x:c>
+      <x:c r="H26" s="37" t="s">
         <x:v>540</x:v>
-      </x:c>
-      <x:c r="H26" s="37" t="s">
-        <x:v>546</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15.75" customHeight="1">
       <x:c r="A27" s="15" t="s">
-        <x:v>547</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="B27" s="2"/>
       <x:c r="C27" s="2"/>
@@ -10551,80 +10523,80 @@
     </x:row>
     <x:row r="28" ht="15.75" customHeight="1">
       <x:c r="A28" s="32" t="s">
-        <x:v>548</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="B28" s="33" t="s">
-        <x:v>495</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="C28" s="33" t="s">
-        <x:v>522</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="D28" s="33">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E28" s="33"/>
       <x:c r="F28" s="33" t="s">
-        <x:v>522</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="G28" s="39" t="s">
-        <x:v>549</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="H28" s="33" t="s">
-        <x:v>550</x:v>
+        <x:v>544</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15.75" customHeight="1">
       <x:c r="A29" s="20" t="s">
-        <x:v>551</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="B29" s="21" t="s">
-        <x:v>552</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="C29" s="21" t="s">
-        <x:v>522</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="D29" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E29" s="21"/>
       <x:c r="F29" s="21" t="s">
-        <x:v>522</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="G29" s="24" t="s">
-        <x:v>549</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="H29" s="21" t="s">
-        <x:v>553</x:v>
+        <x:v>547</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15.75" customHeight="1">
       <x:c r="A30" s="16" t="s">
-        <x:v>554</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="B30" s="17" t="s">
-        <x:v>505</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="C30" s="17" t="s">
-        <x:v>522</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="D30" s="17">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E30" s="17"/>
       <x:c r="F30" s="17" t="s">
-        <x:v>522</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="G30" s="24" t="s">
+        <x:v>543</x:v>
+      </x:c>
+      <x:c r="H30" s="17" t="s">
         <x:v>549</x:v>
-      </x:c>
-      <x:c r="H30" s="17" t="s">
-        <x:v>555</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="25.5" customHeight="1"/>
     <x:row r="32" ht="15.75" customHeight="1">
       <x:c r="A32" s="15" t="s">
-        <x:v>556</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="B32" s="2"/>
       <x:c r="C32" s="2"/>
@@ -10636,7 +10608,7 @@
     </x:row>
     <x:row r="33" ht="15.75" customHeight="1">
       <x:c r="A33" s="6" t="s">
-        <x:v>557</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="B33" s="69" t="n">
         <x:f>SUM(D5:D11)</x:f>
@@ -10645,7 +10617,7 @@
     </x:row>
     <x:row r="34" ht="15.75" customHeight="1">
       <x:c r="A34" s="7" t="s">
-        <x:v>558</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="B34" s="70">
         <x:v>170.0</x:v>
@@ -10653,7 +10625,7 @@
     </x:row>
     <x:row r="35" ht="15.75" customHeight="1">
       <x:c r="A35" s="6" t="s">
-        <x:v>559</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="B35" s="69">
         <x:v>18.0</x:v>
@@ -10661,7 +10633,7 @@
     </x:row>
     <x:row r="36" ht="15.75" customHeight="1">
       <x:c r="A36" s="7" t="s">
-        <x:v>560</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="B36" s="70">
         <x:v>1713.0</x:v>

</xml_diff>

<commit_message>
feat: add Slice 4 content preferences
</commit_message>
<xml_diff>
--- a/docs/product/Pumdoki_MasterTracker_V4.xlsx
+++ b/docs/product/Pumdoki_MasterTracker_V4.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6f36460bd2144711"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R73c3899e5fae4b40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R8796ddf8c1b048df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="R4a98665446be48dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R65b6aee0e9dc4edf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R508ff691d17d4fcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R4dc5d1a1797548ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R18719fd98ac84798"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="R6a4eff3f9e634c2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R5eee08496eeb436d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1875,7 +1875,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="82">
+  <x:cellXfs count="83">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -2112,6 +2112,9 @@
     <x:xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2392,7 +2395,7 @@
       </x:c>
       <x:c r="B7" s="6" t="n">
         <x:f>COUNTIF('Master Tracker'!C4:C164,"🔄 In Progress")</x:f>
-        <x:v>45</x:v>
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2401,7 +2404,7 @@
       </x:c>
       <x:c r="B8" s="7" t="n">
         <x:f>COUNTIF('Master Tracker'!C4:C164,"📋 Not Started")</x:f>
-        <x:v>84</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2468,7 +2471,7 @@
     </x:row>
     <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="C20" s="37" t="str">
-        <x:v>Phase 1 is verified; Phase 2 remains partial; Phase 3 Slices 1–3 are implemented and locally verified. Slice 4 (Settings and explicit-content controls) remains next.</x:v>
+        <x:v>Phase 1 is verified; Phase 2 remains partial; Phase 3 Slices 1–3 are published and CI-verified. Slice 4 is in progress with the default-hidden explicit-content preference vertical cut locally verified.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="16.5" customHeight="1">
@@ -4114,7 +4117,7 @@
         <x:v>🔄 In Progress</x:v>
       </x:c>
       <x:c r="D47" s="19" t="str">
-        <x:v>Local PostgreSQL/Prisma now includes repeatable User, Session, append-only AcceptanceRecord, and transient VerificationToken migrations. Remaining product domains and production RDS schema are pending.</x:v>
+        <x:v>Local PostgreSQL/Prisma now includes repeatable User, Session, append-only AcceptanceRecord, transient VerificationToken, and one-to-one UserPreference migrations. Remaining product domains and production RDS schema are pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
@@ -4144,7 +4147,7 @@
         </x:is>
       </x:c>
       <x:c r="D49" s="19" t="str">
-        <x:v>Implemented /api/v1 health/readiness, core auth, email verification, password reset, logout/logout-all, and /me. Later product domains remain pending.</x:v>
+        <x:v>Implemented /api/v1 health/readiness, core auth, email verification, password reset, logout/logout-all, /me, and authenticated preference reads/updates. Later product domains remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
@@ -5656,15 +5659,11 @@
           <x:t xml:space="preserve">Add hide/show 18+ content choice to onboarding, Settings, feed, search, Store, and Connect; default hidden.</x:t>
         </x:is>
       </x:c>
-      <x:c r="C152" s="24" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">📋 Not Started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D152" s="22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Launch-critical. Does not replace age checks.</x:t>
-        </x:is>
+      <x:c r="C152" s="24" t="str">
+        <x:v>🔄 In Progress</x:v>
+      </x:c>
+      <x:c r="D152" s="22" t="str">
+        <x:v>Default-hidden preference now persists through UserPreference, authenticated GET/PATCH endpoints, and a protected Settings UI with deliberate opt-in, reload persistence, immediate opt-out, and automated coverage. Onboarding and server-side feed/search/Store/Connect filtering remain pending; this does not replace age checks.</x:v>
       </x:c>
     </x:row>
     <x:row r="153" ht="31.5" customHeight="1">
@@ -8478,7 +8477,7 @@
         </x:is>
       </x:c>
       <x:c r="B44" s="71" t="str">
-        <x:v>The architecture plan source of truth is PLAN.md. Phase 3 is split into four slices: Slices 1–3 are implemented and locally verified; Slice 4 remains.</x:v>
+        <x:v>The architecture plan source of truth is PLAN.md. Phase 3 is split into four slices: Slices 1–3 are published and CI-verified; Slice 4 is in progress.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -8488,7 +8487,7 @@
         </x:is>
       </x:c>
       <x:c r="B45" s="73" t="str">
-        <x:v>Phase 3 Slices 1–3 are complete locally. The next implementation slice is Settings and explicit-content controls.</x:v>
+        <x:v>Founder reviews the Slice 4 explicit-content preference flow; Engineering continues with profile, email/reverification, password, and active-session Settings.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -8528,7 +8527,7 @@
         </x:is>
       </x:c>
       <x:c r="B49" s="73" t="str">
-        <x:v>Slice 2 was published to origin/dev and CI passed on July 29, 2026. Slice 3 is implemented and locally verified but not yet published.</x:v>
+        <x:v>Slice 3 was published to dev in commit 1089ae0 and GitHub Actions passed on August 1, 2026. Slice 4's first preference vertical cut is locally verified and captured in this local commit; it has not been pushed.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
@@ -8635,12 +8634,12 @@
         <x:v>Verification and reset tokens are random, hashed at rest, expiring, single-use, and invalidated on reissue; password reset revokes all sessions.</x:v>
       </x:c>
     </x:row>
-    <x:row r="65" ht="15" hidden="0" customHeight="1">
+    <x:row r="65" ht="30" hidden="0" customHeight="1">
       <x:c r="A65" t="str">
         <x:v>•</x:v>
       </x:c>
-      <x:c r="B65" t="str">
-        <x:v>Phase 3 Slice 3 is locally verified. Slice 4 (Settings and explicit-content controls) is the next planned implementation step.</x:v>
+      <x:c r="B65" s="82" t="str">
+        <x:v>Phase 3 Slice 4 is in progress: the default-hidden explicit-content preference persists through the API and protected Settings page; broader account Settings and future server-side content filtering remain.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
feat: complete Phase 3 account security settings
</commit_message>
<xml_diff>
--- a/docs/product/Pumdoki_MasterTracker_V4.xlsx
+++ b/docs/product/Pumdoki_MasterTracker_V4.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R508ff691d17d4fcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R4dc5d1a1797548ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R18719fd98ac84798"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="R6a4eff3f9e634c2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R5eee08496eeb436d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R48eada0b153c4900"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="Ra73ec8657be249eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="Re96e49eca29c4983"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="R7fd3e05a626e4e08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="Reca8ad9372854ee0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2469,9 +2469,9 @@
         <x:v>17</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="20" ht="48" hidden="0" customHeight="1">
       <x:c r="C20" s="37" t="str">
-        <x:v>Phase 1 is verified; Phase 2 remains partial; Phase 3 Slices 1–3 are published and CI-verified. Slice 4 is in progress with the default-hidden explicit-content preference vertical cut locally verified.</x:v>
+        <x:v>Phase 1 is verified; Phase 2 remains partial. Phase 3's founder-approved core scope is locally verified through Slice 4B; manual review, commit/publish, and CI remain before Phase 4 implementation begins. Dependency-bound Settings work remains sequenced to later phases.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="16.5" customHeight="1">
@@ -4147,7 +4147,7 @@
         </x:is>
       </x:c>
       <x:c r="D49" s="19" t="str">
-        <x:v>Implemented /api/v1 health/readiness, core auth, email verification, password reset, logout/logout-all, /me, and authenticated preference reads/updates. Later product domains remain pending.</x:v>
+        <x:v>Implemented /api/v1 health/readiness, auth and email flows, /me, persisted preferences, profile/email/password changes, and active-session listing/revocation. Later product domains remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
@@ -4269,7 +4269,7 @@
         <x:v>✅ Done</x:v>
       </x:c>
       <x:c r="D58" s="19" t="str">
-        <x:v>Slice 3 restores HttpOnly-cookie sessions with /me, handles expiry/401 globally, and supports logout from the member shell.</x:v>
+        <x:v>HttpOnly-cookie sessions restore through /me, renew on a bounded sliding window, support logout/logout-all, and can now be listed and individually revoked from protected Settings. Sensitive account changes revoke other sessions.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
@@ -4311,7 +4311,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="D61" s="22" t="str">
-        <x:v>Slice 3 adds the email verification screen, persistent unverified banner, resend states, and Mailpit-backed browser coverage.</x:v>
+        <x:v>Slice 3 provides verification screens and Mailpit-backed confirmation. Slice 4B adds authenticated email change, invalidates stale links, requires reverification, and preserves only the current session.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="24" hidden="0" customHeight="1">
@@ -4325,7 +4325,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="D62" s="19" t="str">
-        <x:v>Slice 3 adds forgot/reset password screens, neutral request messaging, token handling, session revocation, and browser coverage.</x:v>
+        <x:v>Slice 3 provides reset request/confirmation and global revocation. Slice 4B adds current-password-confirmed password change, reset-token invalidation, and other-session revocation.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="27.75" customHeight="1">
@@ -5663,7 +5663,7 @@
         <x:v>🔄 In Progress</x:v>
       </x:c>
       <x:c r="D152" s="22" t="str">
-        <x:v>Default-hidden preference now persists through UserPreference, authenticated GET/PATCH endpoints, and a protected Settings UI with deliberate opt-in, reload persistence, immediate opt-out, and automated coverage. Onboarding and server-side feed/search/Store/Connect filtering remain pending; this does not replace age checks.</x:v>
+        <x:v>Default-hidden persistence, protected Settings UI, deliberate opt-in/immediate opt-out, profile and email editing, password change, and active-session controls are locally verified. Onboarding and server-side feed/search/Store/Connect enforcement remain for later phases.</x:v>
       </x:c>
     </x:row>
     <x:row r="153" ht="31.5" customHeight="1">
@@ -8470,64 +8470,64 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="44" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="44" ht="36" hidden="0" customHeight="1">
       <x:c r="A44" s="71" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Plan source</x:t>
         </x:is>
       </x:c>
       <x:c r="B44" s="71" t="str">
-        <x:v>The architecture plan source of truth is PLAN.md. Phase 3 is split into four slices: Slices 1–3 are published and CI-verified; Slice 4 is in progress.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>PLAN.md is the architecture source of truth. Founder approved a reduced Phase 3 core scope: Slices 1–4B cover auth, roles, core account security, and explicit-content preference persistence; dependency-bound Settings categories remain sequenced later.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="34.5" hidden="0" customHeight="1">
       <x:c r="A45" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 1</x:t>
         </x:is>
       </x:c>
       <x:c r="B45" s="73" t="str">
-        <x:v>Founder reviews the Slice 4 explicit-content preference flow; Engineering continues with profile, email/reverification, password, and active-session Settings.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Founder manually reviews Slice 4B account/security Settings, then commit and publish Slices 4A/4B and require green GitHub CI before starting Phase 4 implementation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="34.5" hidden="0" customHeight="1">
       <x:c r="A46" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 2</x:t>
         </x:is>
       </x:c>
       <x:c r="B46" s="73" t="str">
-        <x:v>Keep Phase 2 labeled partially complete; decide AWS/Sentry/Redis direction and finish staging, backups/restore, monitoring, queueing, and idempotency.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="15" hidden="0" customHeight="1">
+        <x:v>Keep Phase 2 labeled partially complete; decide AWS/Sentry/Redis direction and finish staging, backup/restore, monitoring, queueing, and idempotency.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="43.5" hidden="0" customHeight="1">
       <x:c r="A47" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 3</x:t>
         </x:is>
       </x:c>
       <x:c r="B47" s="73" t="str">
-        <x:v>Begin privacy-focused LLC attorney/CPA research, counsel-reviewed retention rules, and merchant compliance preparation in parallel.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="15" hidden="0" customHeight="1">
+        <x:v>Begin Phase 4 with a legal/trust foundation slice: decision register, versioned creator-agreement/acceptance design, pending-review onboarding outcome, and provider interfaces without claiming counsel or vendor approval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="34.5" hidden="0" customHeight="1">
       <x:c r="A48" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 4</x:t>
         </x:is>
       </x:c>
       <x:c r="B48" s="73" t="str">
-        <x:v>Obtain CCBill/Epoch requirements, fee quotes, and written cascade guidance; continue identity-provider and launch-country research.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Obtain counsel/CPA guidance and real CCBill, identity-provider, and country-allowlist inputs before implementing irreversible compliance workflows.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="34.5" hidden="0" customHeight="1">
       <x:c r="A49" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 5</x:t>
         </x:is>
       </x:c>
       <x:c r="B49" s="73" t="str">
-        <x:v>Slice 3 was published to dev in commit 1089ae0 and GitHub Actions passed on August 1, 2026. Slice 4's first preference vertical cut is locally verified and captured in this local commit; it has not been pushed.</x:v>
+        <x:v>Slice 4A is committed locally as 7972bf2. Slice 4B is implemented and fully locally verified in the working tree; neither local Slice 4 commit has been published or CI-verified yet.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
@@ -8634,12 +8634,12 @@
         <x:v>Verification and reset tokens are random, hashed at rest, expiring, single-use, and invalidated on reissue; password reset revokes all sessions.</x:v>
       </x:c>
     </x:row>
-    <x:row r="65" ht="30" hidden="0" customHeight="1">
+    <x:row r="65" ht="36" hidden="0" customHeight="1">
       <x:c r="A65" t="str">
         <x:v>•</x:v>
       </x:c>
       <x:c r="B65" s="82" t="str">
-        <x:v>Phase 3 Slice 4 is in progress: the default-hidden explicit-content preference persists through the API and protected Settings page; broader account Settings and future server-side content filtering remain.</x:v>
+        <x:v>Phase 3 Slice 4B locally completes the founder-approved core account-security scope: display-name edit, email change/reverification, authenticated password change, and active-session listing/revocation. Notifications wait for Phase 9; billing for payments; export/deletion for counsel-approved retention; theme for design-system work; explicit-content query enforcement for Phase 5 APIs.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
docs: reconcile master tracker after PRs 1-3
</commit_message>
<xml_diff>
--- a/docs/product/Pumdoki_MasterTracker_V4.xlsx
+++ b/docs/product/Pumdoki_MasterTracker_V4.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R48eada0b153c4900"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="Ra73ec8657be249eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="Re96e49eca29c4983"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="R7fd3e05a626e4e08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="Reca8ad9372854ee0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8dde0944bc0748be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R0162ad42202d4e10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R0f1dcbfe8d1e4e95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="R3eb5aa7156fc4ac5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R8ea6e486897741fd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -398,9 +398,6 @@
     <x:t xml:space="preserve">Ensure primary flows work cleanly on mobile and desktop.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Required early; tracked as active design work.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Implement Dark Knight theme</x:t>
   </x:si>
   <x:si>
@@ -641,9 +638,6 @@
     <x:t xml:space="preserve">Account info, password change, notification preferences, theme toggle (Sakura Pink / Dark Knight), NSFW content toggle, payment/billing section.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Keep minimal for MVP. Theme toggle and NSFW toggle are the critical elements.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Build help / support page</x:t>
   </x:si>
   <x:si>
@@ -875,9 +869,6 @@
     <x:t xml:space="preserve">Review incoming creator applications. View submitted ID documents. Approve or reject. Log decision with reason. Trigger creator onboarding email.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Required before any creator goes live. Tied to 2257 compliance.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Build content moderation queue</x:t>
   </x:si>
   <x:si>
@@ -956,9 +947,6 @@
     <x:t xml:space="preserve">Track all admin actions with timestamp, admin user, action type, and affected entity. Immutable log — no deleting entries.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Useful for security, accountability, and legal protection.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">📊  PHASE 10 — Analytics, Support &amp; Notifications</x:t>
   </x:si>
   <x:si>
@@ -1071,9 +1059,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Turn roadmap into a structured test list.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Checklist organization underway.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Plan private beta</x:t>
@@ -2379,7 +2364,7 @@
       </x:c>
       <x:c r="B6" s="7" t="n">
         <x:f>COUNTIF('Master Tracker'!C4:C164,"✅ Done")</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D6" s="7" t="s">
         <x:v>7</x:v>
@@ -2395,7 +2380,7 @@
       </x:c>
       <x:c r="B7" s="6" t="n">
         <x:f>COUNTIF('Master Tracker'!C4:C164,"🔄 In Progress")</x:f>
-        <x:v>46</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2404,7 +2389,7 @@
       </x:c>
       <x:c r="B8" s="7" t="n">
         <x:f>COUNTIF('Master Tracker'!C4:C164,"📋 Not Started")</x:f>
-        <x:v>83</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2413,7 +2398,7 @@
       </x:c>
       <x:c r="B9" s="8" t="n">
         <x:f>IF(B5=0,0,B6/B5)</x:f>
-        <x:v>0.12837837837837837</x:v>
+        <x:v>0.13513513513513514</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="13.5" customHeight="1"/>
@@ -2430,7 +2415,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C13" s="31" t="str">
-        <x:v>Counts are derived from the Master Tracker through August 1, 2026. Section headers are excluded.</x:v>
+        <x:v>Counts are derived from the Master Tracker through August 16, 2026. Section headers are excluded.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -2469,9 +2454,9 @@
         <x:v>17</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="48" hidden="0" customHeight="1">
+    <x:row r="20" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="C20" s="37" t="str">
-        <x:v>Phase 1 is verified; Phase 2 remains partial. Phase 3's founder-approved core scope is locally verified through Slice 4B; manual review, commit/publish, and CI remain before Phase 4 implementation begins. Dependency-bound Settings work remains sequenced to later phases.</x:v>
+        <x:v>Phase 1 and the founder-approved Phase 3 core scope are published and CI-verified. Phase 2 remains partial. PR #1 merged the Phase 4 creator-application and dormant non-approval review foundation, PR #2 merged routing hardening, and PR #3 merged non-secret readiness documentation. The operations router remains unmounted and activation gates G1–G12 are NOT EVALUATED.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="16.5" customHeight="1">
@@ -3572,20 +3557,18 @@
         <x:v>33</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="20" t="s">
         <x:v>34</x:v>
       </x:c>
       <x:c r="B8" s="21" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="C8" s="23" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D8" s="22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Detailed phased roadmap created in repository PLAN.md; tracker reconciliation continues.</x:t>
-        </x:is>
+      <x:c r="C8" s="23" t="str">
+        <x:v>✅ Done</x:v>
+      </x:c>
+      <x:c r="D8" s="22" t="str">
+        <x:v>Dependency-ordered PLAN.md is established and current through the merged PR #1–#3 baseline; tracker reconciliation is now ongoing maintenance.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4028,7 +4011,7 @@
         <x:v>125</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="15.75" customHeight="1">
+    <x:row r="41" ht="24" hidden="0" customHeight="1">
       <x:c r="A41" s="20" t="s">
         <x:v>126</x:v>
       </x:c>
@@ -4038,41 +4021,41 @@
       <x:c r="C41" s="23" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="D41" s="22" t="s">
-        <x:v>128</x:v>
+      <x:c r="D41" s="22" t="str">
+        <x:v>Responsive work remains active. A session-aware branded 404, route-level code splitting, and an in-flow dismissible verification reminder are merged and CI-covered on desktop/mobile paths.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15.75" customHeight="1">
       <x:c r="A42" s="16" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="B42" s="17" t="s">
         <x:v>129</x:v>
-      </x:c>
-      <x:c r="B42" s="17" t="s">
-        <x:v>130</x:v>
       </x:c>
       <x:c r="C42" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D42" s="19" t="s">
-        <x:v>131</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15.75" customHeight="1">
       <x:c r="A43" s="20" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="B43" s="21" t="s">
         <x:v>132</x:v>
-      </x:c>
-      <x:c r="B43" s="21" t="s">
-        <x:v>133</x:v>
       </x:c>
       <x:c r="C43" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D43" s="22" t="s">
-        <x:v>134</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="27.75" customHeight="1">
       <x:c r="A44" s="15" t="s">
-        <x:v>135</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="B44" s="2"/>
       <x:c r="C44" s="2"/>
@@ -4080,110 +4063,110 @@
     </x:row>
     <x:row r="45" ht="15.75" customHeight="1">
       <x:c r="A45" s="16" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="B45" s="17" t="s">
         <x:v>136</x:v>
-      </x:c>
-      <x:c r="B45" s="17" t="s">
-        <x:v>137</x:v>
       </x:c>
       <x:c r="C45" s="18" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D45" s="19" t="s">
-        <x:v>138</x:v>
+        <x:v>137</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15.75" customHeight="1">
       <x:c r="A46" s="20" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="B46" s="21" t="s">
         <x:v>139</x:v>
-      </x:c>
-      <x:c r="B46" s="21" t="s">
-        <x:v>140</x:v>
       </x:c>
       <x:c r="C46" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D46" s="22" t="s">
-        <x:v>141</x:v>
+        <x:v>140</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="24" hidden="0" customHeight="1">
       <x:c r="A47" s="16" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="B47" s="17" t="s">
         <x:v>142</x:v>
-      </x:c>
-      <x:c r="B47" s="17" t="s">
-        <x:v>143</x:v>
       </x:c>
       <x:c r="C47" s="24" t="str">
         <x:v>🔄 In Progress</x:v>
       </x:c>
       <x:c r="D47" s="19" t="str">
-        <x:v>Local PostgreSQL/Prisma now includes repeatable User, Session, append-only AcceptanceRecord, transient VerificationToken, and one-to-one UserPreference migrations. Remaining product domains and production RDS schema are pending.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="15" hidden="0" customHeight="1">
+        <x:v>Local PostgreSQL/Prisma includes User, Session, append-only AcceptanceRecord, VerificationToken, UserPreference, CreatorApplication, creator-policy acceptance, and constrained successful-transition review evidence. Remaining product domains and production RDS deployment are pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="24" hidden="0" customHeight="1">
       <x:c r="A48" s="20" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="B48" s="21" t="s">
         <x:v>144</x:v>
-      </x:c>
-      <x:c r="B48" s="21" t="s">
-        <x:v>145</x:v>
       </x:c>
       <x:c r="C48" s="24" t="str">
         <x:v>🔄 In Progress</x:v>
       </x:c>
       <x:c r="D48" s="22" t="str">
-        <x:v>Local environment is defined with validated variables and Docker PostgreSQL. Staging and production infrastructure remain pending.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="15" hidden="0" customHeight="1">
+        <x:v>Local validated environments plus Docker PostgreSQL/Mailpit exist. PR #3 adds non-secret staging/configuration/verification templates only; staging and production infrastructure, credentials, private origin, and live verification remain pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="24" hidden="0" customHeight="1">
       <x:c r="A49" s="16" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="B49" s="17" t="s">
         <x:v>146</x:v>
       </x:c>
-      <x:c r="B49" s="17" t="s">
+      <x:c r="C49" s="23" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">🔄 In Progress</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D49" s="19" t="str">
+        <x:v>Implemented /api/v1 health/readiness, auth/email, /me, protected Settings/session, and member creator-application flows. The creator-review router remains deliberately unmounted and requires an operations verifier; later product domains remain pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="24" hidden="0" customHeight="1">
+      <x:c r="A50" s="20" t="s">
         <x:v>147</x:v>
       </x:c>
-      <x:c r="C49" s="23" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">🔄 In Progress</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D49" s="19" t="str">
-        <x:v>Implemented /api/v1 health/readiness, auth and email flows, /me, persisted preferences, profile/email/password changes, and active-session listing/revocation. Later product domains remain pending.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50" ht="15" hidden="0" customHeight="1">
-      <x:c r="A50" s="20" t="s">
+      <x:c r="B50" s="21" t="s">
         <x:v>148</x:v>
-      </x:c>
-      <x:c r="B50" s="21" t="s">
-        <x:v>149</x:v>
       </x:c>
       <x:c r="C50" s="24" t="str">
         <x:v>🔄 In Progress</x:v>
       </x:c>
       <x:c r="D50" s="22" t="str">
-        <x:v>Structured Pino request logging is implemented with request IDs and secret-header redaction. Sentry/operational error monitoring remains pending.</x:v>
+        <x:v>Structured Pino request logging, request IDs, and secret-header redaction are implemented. PR #3 adds a provider scorecard/runbook only; monitoring integration, alerts, retention decisions, and live evidence remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="16" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="B51" s="17" t="s">
         <x:v>150</x:v>
-      </x:c>
-      <x:c r="B51" s="17" t="s">
-        <x:v>151</x:v>
       </x:c>
       <x:c r="C51" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D51" s="19" t="s">
+        <x:v>151</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
+      <x:c r="A52" s="20" t="s">
         <x:v>152</x:v>
       </x:c>
-    </x:row>
-    <x:row r="52" ht="24" hidden="0" customHeight="1">
-      <x:c r="A52" s="20" t="s">
+      <x:c r="B52" s="21" t="s">
         <x:v>153</x:v>
-      </x:c>
-      <x:c r="B52" s="21" t="s">
-        <x:v>154</x:v>
       </x:c>
       <x:c r="C52" s="24" t="str">
         <x:v>🔄 In Progress</x:v>
@@ -4192,39 +4175,39 @@
         <x:v>Global per-IP limits plus bounded in-memory login and email-request throttles are implemented. Redis-backed multi-instance protection remains pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="15" hidden="0" customHeight="1">
+    <x:row r="53" ht="24" hidden="0" customHeight="1">
       <x:c r="A53" s="16" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="B53" s="17" t="s">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="B53" s="17" t="s">
-        <x:v>156</x:v>
-      </x:c>
       <x:c r="C53" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">🔄 In Progress</x:t>
         </x:is>
       </x:c>
       <x:c r="D53" s="19" t="str">
-        <x:v>CI runs web lint/tests/build/E2E plus API build, migrations, seed, and DB-backed tests on PostgreSQL 17. Deployment automation remains pending.</x:v>
+        <x:v>CI runs formatting, lint, web/API tests and builds, migrations/seed, private-admin build, and real-stack Playwright with read-only token permissions and bounded timeouts. PR #1–#3 passed reviewed-head CI; deployment automation remains pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="20" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="B54" s="21" t="s">
         <x:v>157</x:v>
-      </x:c>
-      <x:c r="B54" s="21" t="s">
-        <x:v>158</x:v>
       </x:c>
       <x:c r="C54" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D54" s="22" t="s">
-        <x:v>159</x:v>
+        <x:v>158</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="27.75" customHeight="1">
       <x:c r="A55" s="15" t="s">
-        <x:v>160</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B55" s="2"/>
       <x:c r="C55" s="2"/>
@@ -4232,10 +4215,10 @@
     </x:row>
     <x:row r="56" ht="24" hidden="0" customHeight="1">
       <x:c r="A56" s="16" t="s">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="B56" s="17" t="s">
         <x:v>161</x:v>
-      </x:c>
-      <x:c r="B56" s="17" t="s">
-        <x:v>162</x:v>
       </x:c>
       <x:c r="C56" s="24" t="str">
         <x:v>✅ Done</x:v>
@@ -4244,26 +4227,26 @@
         <x:v>Slice 3 connects registration, login, logout, and authenticated route restoration to the live API.</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="15" hidden="0" customHeight="1">
+    <x:row r="57" ht="24" hidden="0" customHeight="1">
       <x:c r="A57" s="20" t="s">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="B57" s="21" t="s">
         <x:v>163</x:v>
-      </x:c>
-      <x:c r="B57" s="21" t="s">
-        <x:v>164</x:v>
       </x:c>
       <x:c r="C57" s="24" t="str">
         <x:v>✅ Done</x:v>
       </x:c>
       <x:c r="D57" s="22" t="str">
-        <x:v>Slice 3 enforces uppercase MEMBER/CREATOR/ADMIN role routing and protected-route authorization in the frontend.</x:v>
+        <x:v>MEMBER/CREATOR route gates and backend role checks are implemented. The public web app has no /admin route; an ADMIN public session is not operational authentication and cannot activate the dormant review router.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="24" hidden="0" customHeight="1">
       <x:c r="A58" s="16" t="s">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="B58" s="17" t="s">
         <x:v>165</x:v>
-      </x:c>
-      <x:c r="B58" s="17" t="s">
-        <x:v>166</x:v>
       </x:c>
       <x:c r="C58" s="24" t="str">
         <x:v>✅ Done</x:v>
@@ -4272,40 +4255,40 @@
         <x:v>HttpOnly-cookie sessions restore through /me, renew on a bounded sliding window, support logout/logout-all, and can now be listed and individually revoked from protected Settings. Sensitive account changes revoke other sessions.</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" ht="15" hidden="0" customHeight="1">
+    <x:row r="59" ht="24" hidden="0" customHeight="1">
       <x:c r="A59" s="20" t="s">
+        <x:v>166</x:v>
+      </x:c>
+      <x:c r="B59" s="21" t="s">
         <x:v>167</x:v>
-      </x:c>
-      <x:c r="B59" s="21" t="s">
-        <x:v>168</x:v>
       </x:c>
       <x:c r="C59" s="23" t="str">
         <x:v>🔄 In Progress</x:v>
       </x:c>
       <x:c r="D59" s="19" t="str">
-        <x:v>Frontend prototypes exist; creator/member first-run onboarding and creator theme selection remain pending.</x:v>
+        <x:v>A verified MEMBER can submit one persisted creator application; it remains PENDING with identity NOT_STARTED and no role promotion or Dashboard access. Member first-run setup, theme choice, identity/tax/banking intake, and operational approval remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="24" hidden="0" customHeight="1">
       <x:c r="A60" s="16" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="B60" s="17" t="s">
         <x:v>169</x:v>
-      </x:c>
-      <x:c r="B60" s="17" t="s">
-        <x:v>170</x:v>
       </x:c>
       <x:c r="C60" s="24" t="str">
         <x:v>🔄 In Progress</x:v>
       </x:c>
       <x:c r="D60" s="19" t="str">
-        <x:v>Registration now records append-only age attestation plus versioned Terms and Privacy acceptance in one transaction. Entry UI and identity/age verification remain pending.</x:v>
+        <x:v>Registration records append-only age attestation and versioned Terms/Privacy acceptance; verified email gates creator-application submission. Entry-gate UI and actual identity/age verification remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="24" hidden="0" customHeight="1">
       <x:c r="A61" s="20" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="B61" s="21" t="s">
         <x:v>171</x:v>
-      </x:c>
-      <x:c r="B61" s="21" t="s">
-        <x:v>172</x:v>
       </x:c>
       <x:c r="C61" s="24" t="s">
         <x:v>6</x:v>
@@ -4316,10 +4299,10 @@
     </x:row>
     <x:row r="62" ht="24" hidden="0" customHeight="1">
       <x:c r="A62" s="16" t="s">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="B62" s="17" t="s">
         <x:v>173</x:v>
-      </x:c>
-      <x:c r="B62" s="17" t="s">
-        <x:v>174</x:v>
       </x:c>
       <x:c r="C62" s="24" t="s">
         <x:v>6</x:v>
@@ -4330,7 +4313,7 @@
     </x:row>
     <x:row r="63" ht="27.75" customHeight="1">
       <x:c r="A63" s="15" t="s">
-        <x:v>175</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="B63" s="2"/>
       <x:c r="C63" s="2"/>
@@ -4338,94 +4321,94 @@
     </x:row>
     <x:row r="64" ht="15.75" customHeight="1">
       <x:c r="A64" s="16" t="s">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="B64" s="17" t="s">
         <x:v>176</x:v>
-      </x:c>
-      <x:c r="B64" s="17" t="s">
-        <x:v>177</x:v>
       </x:c>
       <x:c r="C64" s="18" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D64" s="19" t="s">
-        <x:v>178</x:v>
+        <x:v>177</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="15.75" customHeight="1">
       <x:c r="A65" s="20" t="s">
+        <x:v>178</x:v>
+      </x:c>
+      <x:c r="B65" s="21" t="s">
         <x:v>179</x:v>
-      </x:c>
-      <x:c r="B65" s="21" t="s">
-        <x:v>180</x:v>
       </x:c>
       <x:c r="C65" s="23" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="D65" s="22" t="s">
-        <x:v>181</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15.75" customHeight="1">
       <x:c r="A66" s="16" t="s">
+        <x:v>181</x:v>
+      </x:c>
+      <x:c r="B66" s="17" t="s">
         <x:v>182</x:v>
-      </x:c>
-      <x:c r="B66" s="17" t="s">
-        <x:v>183</x:v>
       </x:c>
       <x:c r="C66" s="23" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="D66" s="19" t="s">
-        <x:v>184</x:v>
+        <x:v>183</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="15.75" customHeight="1">
       <x:c r="A67" s="20" t="s">
+        <x:v>184</x:v>
+      </x:c>
+      <x:c r="B67" s="21" t="s">
         <x:v>185</x:v>
-      </x:c>
-      <x:c r="B67" s="21" t="s">
-        <x:v>186</x:v>
       </x:c>
       <x:c r="C67" s="18" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D67" s="22" t="s">
-        <x:v>187</x:v>
+        <x:v>186</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="15.75" customHeight="1">
       <x:c r="A68" s="16" t="s">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="B68" s="17" t="s">
         <x:v>188</x:v>
-      </x:c>
-      <x:c r="B68" s="17" t="s">
-        <x:v>189</x:v>
       </x:c>
       <x:c r="C68" s="23" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="D68" s="19" t="s">
+        <x:v>189</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="24" hidden="0" customHeight="1">
+      <x:c r="A69" s="20" t="s">
         <x:v>190</x:v>
       </x:c>
-    </x:row>
-    <x:row r="69" ht="15.75" customHeight="1">
-      <x:c r="A69" s="20" t="s">
+      <x:c r="B69" s="21" t="s">
         <x:v>191</x:v>
-      </x:c>
-      <x:c r="B69" s="21" t="s">
-        <x:v>192</x:v>
       </x:c>
       <x:c r="C69" s="23" t="str">
         <x:v>✅ Done</x:v>
       </x:c>
       <x:c r="D69" s="22" t="str">
-        <x:v>Slice 3 replaces prototype login/signup behavior with validated live-API flows and adds forgot/reset/verify screens.</x:v>
+        <x:v>Live validated API login/signup/logout plus forgot/reset/verify flows are published. Registration was redesigned, verification reminders no longer overlay protected content, and deep-link restoration/session-aware recovery are CI-covered.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="15.75" customHeight="1">
       <x:c r="A70" s="16" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="B70" s="17" t="s">
         <x:v>193</x:v>
-      </x:c>
-      <x:c r="B70" s="17" t="s">
-        <x:v>194</x:v>
       </x:c>
       <x:c r="C70" s="18" t="str">
         <x:v>✅ Done</x:v>
@@ -4436,10 +4419,10 @@
     </x:row>
     <x:row r="71" ht="15.75" customHeight="1">
       <x:c r="A71" s="20" t="s">
+        <x:v>194</x:v>
+      </x:c>
+      <x:c r="B71" s="21" t="s">
         <x:v>195</x:v>
-      </x:c>
-      <x:c r="B71" s="21" t="s">
-        <x:v>196</x:v>
       </x:c>
       <x:c r="C71" s="23" t="inlineStr">
         <x:is>
@@ -4454,10 +4437,10 @@
     </x:row>
     <x:row r="72" ht="15.75" customHeight="1">
       <x:c r="A72" s="16" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="B72" s="17" t="s">
         <x:v>197</x:v>
-      </x:c>
-      <x:c r="B72" s="17" t="s">
-        <x:v>198</x:v>
       </x:c>
       <x:c r="C72" s="23" t="inlineStr">
         <x:is>
@@ -4472,10 +4455,10 @@
     </x:row>
     <x:row r="73" ht="15.75" customHeight="1">
       <x:c r="A73" s="20" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="B73" s="21" t="s">
         <x:v>199</x:v>
-      </x:c>
-      <x:c r="B73" s="21" t="s">
-        <x:v>200</x:v>
       </x:c>
       <x:c r="C73" s="23" t="s">
         <x:v>8</x:v>
@@ -4488,10 +4471,10 @@
     </x:row>
     <x:row r="74" ht="15.75" customHeight="1">
       <x:c r="A74" s="16" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="B74" s="17" t="s">
         <x:v>201</x:v>
-      </x:c>
-      <x:c r="B74" s="17" t="s">
-        <x:v>202</x:v>
       </x:c>
       <x:c r="C74" s="23" t="s">
         <x:v>8</x:v>
@@ -4504,7 +4487,7 @@
     </x:row>
     <x:row r="75" ht="15.75" customHeight="1">
       <x:c r="A75" s="20" t="s">
-        <x:v>203</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="B75" s="17" t="inlineStr">
         <x:is>
@@ -4524,130 +4507,128 @@
     </x:row>
     <x:row r="76" ht="15.75" customHeight="1">
       <x:c r="A76" s="16" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="B76" s="17" t="s">
         <x:v>204</x:v>
       </x:c>
-      <x:c r="B76" s="17" t="s">
+      <x:c r="C76" s="23" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">🔄 In Progress</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D76" s="22" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Wallet UI prototype exists. Add/recharge Veso needs an E-Pal Buff-inspired design plus real ledger/payment integration.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="24" hidden="0" customHeight="1">
+      <x:c r="A77" s="20" t="s">
         <x:v>205</x:v>
       </x:c>
-      <x:c r="C76" s="23" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">🔄 In Progress</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D76" s="22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Wallet UI prototype exists. Add/recharge Veso needs an E-Pal Buff-inspired design plus real ledger/payment integration.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="77" ht="15.75" customHeight="1">
-      <x:c r="A77" s="20" t="s">
+      <x:c r="B77" s="17" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User preference to hide or show explicit 18+ content across onboarding, Settings, feeds, search, Store, and Connect. Default hidden.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C77" s="24" t="str">
+        <x:v>🔄 In Progress</x:v>
+      </x:c>
+      <x:c r="D77" s="19" t="str">
+        <x:v>Default-hidden preference persistence and protected Settings opt-in/immediate opt-out are implemented and CI-verified. Onboarding and server-side feed/search/Store/Connect enforcement remain pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="24" hidden="0" customHeight="1">
+      <x:c r="A78" s="16" t="s">
         <x:v>206</x:v>
       </x:c>
-      <x:c r="B77" s="17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">User preference to hide or show explicit 18+ content across onboarding, Settings, feeds, search, Store, and Connect. Default hidden.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C77" s="24" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D77" s="19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Launch-critical and separate from age verification. Preference must be enforced by APIs and queries, not only CSS.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="78" ht="15.75" customHeight="1">
-      <x:c r="A78" s="16" t="s">
+      <x:c r="B78" s="17" t="s">
         <x:v>207</x:v>
       </x:c>
-      <x:c r="B78" s="17" t="s">
-        <x:v>208</x:v>
-      </x:c>
-      <x:c r="C78" s="24" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D78" s="19" t="s">
-        <x:v>209</x:v>
+      <x:c r="C78" s="24" t="str">
+        <x:v>🔄 In Progress</x:v>
+      </x:c>
+      <x:c r="D78" s="19" t="str">
+        <x:v>Protected Settings is implemented for display name, email/reverification, password, active sessions, and explicit-content preference. Notifications, theme, billing, export, and deletion remain deferred to dependency phases.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="15.75" customHeight="1">
       <x:c r="A79" s="20" t="s">
-        <x:v>210</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="B79" s="21" t="s">
-        <x:v>211</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="C79" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D79" s="22" t="s">
-        <x:v>212</x:v>
+        <x:v>210</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="15.75" customHeight="1">
       <x:c r="A80" s="16" t="s">
-        <x:v>213</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="B80" s="17" t="s">
-        <x:v>214</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C80" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D80" s="19" t="s">
-        <x:v>215</x:v>
+        <x:v>213</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="15.75" customHeight="1">
       <x:c r="A81" s="20" t="s">
-        <x:v>216</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="B81" s="21" t="s">
-        <x:v>217</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="C81" s="18" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D81" s="22" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="15.75" customHeight="1">
       <x:c r="A82" s="16" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="B82" s="17" t="s">
-        <x:v>220</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C82" s="18" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D82" s="19" t="s">
-        <x:v>221</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="15.75" customHeight="1">
       <x:c r="A83" s="20" t="s">
-        <x:v>222</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="B83" s="21" t="s">
-        <x:v>223</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="C83" s="18" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D83" s="22" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="30.75" customHeight="1">
       <x:c r="A84" s="16" t="s">
-        <x:v>225</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="B84" s="17" t="s">
-        <x:v>226</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="C84" s="23" t="inlineStr">
         <x:is>
@@ -4662,21 +4643,21 @@
     </x:row>
     <x:row r="85" ht="18.75" customHeight="1">
       <x:c r="A85" s="25" t="s">
-        <x:v>227</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="B85" s="26" t="s">
-        <x:v>228</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="C85" s="18" t="s">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D85" s="27" t="s">
-        <x:v>229</x:v>
+        <x:v>227</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="15.75" customHeight="1">
       <x:c r="A86" s="15" t="s">
-        <x:v>230</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="B86" s="2"/>
       <x:c r="C86" s="2"/>
@@ -4684,91 +4665,91 @@
     </x:row>
     <x:row r="87" ht="15.75" customHeight="1">
       <x:c r="A87" s="16" t="s">
-        <x:v>231</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="B87" s="17" t="s">
-        <x:v>232</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C87" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D87" s="19" t="s">
-        <x:v>233</x:v>
+        <x:v>231</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="15.75" customHeight="1">
       <x:c r="A88" s="20" t="s">
-        <x:v>234</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="B88" s="21" t="s">
-        <x:v>235</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="C88" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D88" s="22" t="s">
-        <x:v>236</x:v>
+        <x:v>234</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="15.75" customHeight="1">
       <x:c r="A89" s="16" t="s">
-        <x:v>237</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="B89" s="17" t="s">
-        <x:v>238</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C89" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D89" s="19" t="s">
-        <x:v>239</x:v>
+        <x:v>237</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="15.75" customHeight="1">
       <x:c r="A90" s="20" t="s">
-        <x:v>240</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="B90" s="21" t="s">
-        <x:v>241</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="C90" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D90" s="22" t="s">
-        <x:v>242</x:v>
+        <x:v>240</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="15.75" customHeight="1">
       <x:c r="A91" s="16" t="s">
-        <x:v>243</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="B91" s="17" t="s">
-        <x:v>244</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="C91" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D91" s="19" t="s">
-        <x:v>245</x:v>
+        <x:v>243</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="27.75" customHeight="1">
       <x:c r="A92" s="28" t="s">
-        <x:v>246</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="B92" s="29" t="s">
-        <x:v>247</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="C92" s="30" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D92" s="31" t="s">
-        <x:v>248</x:v>
+        <x:v>246</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="15.75" customHeight="1">
       <x:c r="A93" s="15" t="s">
-        <x:v>249</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="B93" s="2"/>
       <x:c r="C93" s="2"/>
@@ -4776,10 +4757,10 @@
     </x:row>
     <x:row r="94" ht="15.75" customHeight="1">
       <x:c r="A94" s="32" t="s">
-        <x:v>250</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="B94" s="33" t="s">
-        <x:v>251</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="C94" s="24" t="inlineStr">
         <x:is>
@@ -4794,10 +4775,10 @@
     </x:row>
     <x:row r="95" ht="15.75" customHeight="1">
       <x:c r="A95" s="20" t="s">
-        <x:v>252</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="B95" s="21" t="s">
-        <x:v>253</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="C95" s="24" t="inlineStr">
         <x:is>
@@ -4812,10 +4793,10 @@
     </x:row>
     <x:row r="96" ht="15.75" customHeight="1">
       <x:c r="A96" s="16" t="s">
-        <x:v>254</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="B96" s="17" t="s">
-        <x:v>255</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="C96" s="24" t="s">
         <x:v>7</x:v>
@@ -4828,66 +4809,66 @@
     </x:row>
     <x:row r="97" ht="15.75" customHeight="1">
       <x:c r="A97" s="20" t="s">
-        <x:v>256</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="B97" s="21" t="s">
-        <x:v>257</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="C97" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D97" s="22" t="s">
-        <x:v>258</x:v>
+        <x:v>256</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="15.75" customHeight="1">
       <x:c r="A98" s="16" t="s">
-        <x:v>259</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="B98" s="17" t="s">
-        <x:v>260</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="C98" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D98" s="19" t="s">
-        <x:v>261</x:v>
+        <x:v>259</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="15.75" customHeight="1">
       <x:c r="A99" s="20" t="s">
-        <x:v>262</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="B99" s="21" t="s">
-        <x:v>263</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="C99" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D99" s="22" t="s">
-        <x:v>264</x:v>
+        <x:v>262</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="15.75" customHeight="1">
       <x:c r="A100" s="16" t="s">
-        <x:v>265</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="B100" s="17" t="s">
-        <x:v>266</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="C100" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D100" s="19" t="s">
-        <x:v>267</x:v>
+        <x:v>265</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="15.75" customHeight="1">
       <x:c r="A101" s="20" t="s">
-        <x:v>268</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="B101" s="21" t="s">
-        <x:v>269</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="C101" s="23" t="inlineStr">
         <x:is>
@@ -4902,10 +4883,10 @@
     </x:row>
     <x:row r="102" ht="15.75" customHeight="1">
       <x:c r="A102" s="16" t="s">
-        <x:v>270</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="B102" s="17" t="s">
-        <x:v>271</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="C102" s="24" t="s">
         <x:v>7</x:v>
@@ -4918,225 +4899,225 @@
     </x:row>
     <x:row r="103" ht="15.75" customHeight="1">
       <x:c r="A103" s="20" t="s">
-        <x:v>272</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="B103" s="21" t="s">
-        <x:v>273</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="C103" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D103" s="22" t="s">
-        <x:v>274</x:v>
+        <x:v>272</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="27.75" customHeight="1">
       <x:c r="A104" s="36" t="s">
-        <x:v>275</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="B104" s="37" t="s">
-        <x:v>276</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="C104" s="30" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D104" s="38" t="s">
-        <x:v>277</x:v>
+        <x:v>275</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="15.75" customHeight="1">
       <x:c r="A105" s="15" t="s">
-        <x:v>278</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="B105" s="2"/>
       <x:c r="C105" s="2"/>
       <x:c r="D105" s="3"/>
     </x:row>
-    <x:row r="106" ht="15.75" customHeight="1">
+    <x:row r="106" ht="36" hidden="0" customHeight="1">
       <x:c r="A106" s="32" t="str">
         <x:v>Build private operations application</x:v>
       </x:c>
       <x:c r="B106" s="33" t="str">
         <x:v>Deploy a separately hosted private operations app; do not expose /admin in the public Pumdoki web app. Enforce ADMIN permissions in the API and apply separate operational access controls.</x:v>
       </x:c>
-      <x:c r="C106" s="39" t="s">
-        <x:v>7</x:v>
+      <x:c r="C106" s="39" t="str">
+        <x:v>🔄 In Progress</x:v>
       </x:c>
       <x:c r="D106" s="35" t="str">
-        <x:v>Founder decision 2026-08-01: public /admin removed; backend ADMIN role retained; independent apps/admin shell exists, while operational workflows remain Phase 11.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="107" ht="15.75" customHeight="1">
+        <x:v>An independently buildable apps/admin shell, public /admin removal, a dormant injected-verifier API seam, and a non-secret readiness packet are merged. No deployed private origin, production verifier, hardware-backed assurance, operator provisioning, origin/CSRF controls, restricted DB grants, or usable review UI exists; G1–G12 are NOT EVALUATED.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="15" hidden="0" customHeight="1">
       <x:c r="A107" s="20" t="s">
-        <x:v>279</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="B107" s="21" t="s">
-        <x:v>280</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="C107" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D107" s="22" t="s">
+        <x:v>279</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="15" hidden="0" customHeight="1">
+      <x:c r="A108" s="16" t="s">
+        <x:v>280</x:v>
+      </x:c>
+      <x:c r="B108" s="17" t="s">
         <x:v>281</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="108" ht="15.75" customHeight="1">
-      <x:c r="A108" s="16" t="s">
-        <x:v>282</x:v>
-      </x:c>
-      <x:c r="B108" s="17" t="s">
-        <x:v>283</x:v>
       </x:c>
       <x:c r="C108" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D108" s="19" t="s">
+        <x:v>282</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="24" hidden="0" customHeight="1">
+      <x:c r="A109" s="20" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="B109" s="21" t="s">
         <x:v>284</x:v>
       </x:c>
-    </x:row>
-    <x:row r="109" ht="15.75" customHeight="1">
-      <x:c r="A109" s="20" t="s">
-        <x:v>285</x:v>
-      </x:c>
-      <x:c r="B109" s="21" t="s">
-        <x:v>286</x:v>
-      </x:c>
-      <x:c r="C109" s="24" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D109" s="22" t="s">
-        <x:v>287</x:v>
+      <x:c r="C109" s="24" t="str">
+        <x:v>🔄 In Progress</x:v>
+      </x:c>
+      <x:c r="D109" s="22" t="str">
+        <x:v>Application submission/persistence and dormant server-side NEEDS_INFORMATION/REJECTED transitions with successful-transition evidence are merged. No queue/list/detail UI, ID/selfie intake, APPROVED, role promotion, reviewer deployment, notification, or creator publishing exists.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="15.75" customHeight="1">
       <x:c r="A110" s="16" t="s">
-        <x:v>288</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="B110" s="17" t="s">
-        <x:v>289</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="C110" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D110" s="19" t="s">
-        <x:v>290</x:v>
+        <x:v>287</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="15.75" customHeight="1">
       <x:c r="A111" s="20" t="s">
-        <x:v>291</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="B111" s="21" t="s">
-        <x:v>292</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="C111" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D111" s="22" t="s">
-        <x:v>293</x:v>
+        <x:v>290</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="15.75" customHeight="1">
       <x:c r="A112" s="16" t="s">
-        <x:v>294</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="B112" s="17" t="s">
-        <x:v>295</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="C112" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D112" s="19" t="s">
-        <x:v>296</x:v>
+        <x:v>293</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="15.75" customHeight="1">
       <x:c r="A113" s="20" t="s">
-        <x:v>297</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="B113" s="21" t="s">
-        <x:v>298</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="C113" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D113" s="22" t="s">
-        <x:v>299</x:v>
+        <x:v>296</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="15.75" customHeight="1">
       <x:c r="A114" s="16" t="s">
-        <x:v>300</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="B114" s="17" t="s">
-        <x:v>301</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="C114" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D114" s="19" t="s">
-        <x:v>302</x:v>
+        <x:v>299</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="15.75" customHeight="1">
       <x:c r="A115" s="20" t="s">
-        <x:v>303</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="B115" s="21" t="s">
-        <x:v>304</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="C115" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D115" s="22" t="s">
-        <x:v>305</x:v>
+        <x:v>302</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="15.75" customHeight="1">
       <x:c r="A116" s="16" t="s">
-        <x:v>306</x:v>
+        <x:v>303</x:v>
       </x:c>
       <x:c r="B116" s="17" t="s">
-        <x:v>307</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="C116" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D116" s="19" t="s">
-        <x:v>308</x:v>
+        <x:v>305</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="15.75" customHeight="1">
       <x:c r="A117" s="20" t="s">
-        <x:v>309</x:v>
+        <x:v>306</x:v>
       </x:c>
       <x:c r="B117" s="21" t="s">
-        <x:v>310</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="C117" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D117" s="22" t="s">
-        <x:v>311</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="118" ht="27.75" customHeight="1">
+        <x:v>308</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="24" hidden="0" customHeight="1">
       <x:c r="A118" s="36" t="s">
-        <x:v>312</x:v>
+        <x:v>309</x:v>
       </x:c>
       <x:c r="B118" s="37" t="s">
-        <x:v>313</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="C118" s="30" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D118" s="38" t="s">
-        <x:v>314</x:v>
+      <x:c r="D118" s="38" t="str">
+        <x:v>The merged creator-review event records successful non-approval transitions at application level, but it is not a complete immutable operations audit. The global audit log, restricted audit destination, retention, and operational evidence controls remain unimplemented.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="15.75" customHeight="1">
       <x:c r="A119" s="15" t="s">
-        <x:v>315</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="B119" s="2"/>
       <x:c r="C119" s="2"/>
@@ -5144,10 +5125,10 @@
     </x:row>
     <x:row r="120" ht="15.75" customHeight="1">
       <x:c r="A120" s="32" t="s">
-        <x:v>316</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="B120" s="33" t="s">
-        <x:v>317</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="C120" s="39" t="s">
         <x:v>7</x:v>
@@ -5158,65 +5139,63 @@
     </x:row>
     <x:row r="121" ht="15.75" customHeight="1">
       <x:c r="A121" s="20" t="s">
-        <x:v>318</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="B121" s="21" t="s">
-        <x:v>319</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="C121" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D121" s="22" t="s">
-        <x:v>320</x:v>
+        <x:v>316</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="15.75" customHeight="1">
       <x:c r="A122" s="16" t="s">
-        <x:v>321</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="B122" s="17" t="s">
-        <x:v>322</x:v>
+        <x:v>318</x:v>
       </x:c>
       <x:c r="C122" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D122" s="19" t="s">
-        <x:v>323</x:v>
+        <x:v>319</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="15.75" customHeight="1">
       <x:c r="A123" s="20" t="s">
-        <x:v>324</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="B123" s="21" t="s">
-        <x:v>325</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="C123" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D123" s="22" t="s">
-        <x:v>326</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="124" ht="27.75" customHeight="1">
+        <x:v>322</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="24" hidden="0" customHeight="1">
       <x:c r="A124" s="36" t="s">
-        <x:v>327</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="B124" s="37" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="C124" s="30" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D124" s="22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Provider undecided. Evaluate Amazon SES first, confirm adult-business support, and use .example addresses until real mailboxes exist.</x:t>
-        </x:is>
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="C124" s="30" t="str">
+        <x:v>🔄 In Progress</x:v>
+      </x:c>
+      <x:c r="D124" s="22" t="str">
+        <x:v>Provider-neutral console/SMTP delivery, local Mailpit, and verification/password-reset messages are implemented. Production provider selection, adult-business fit, deliverability/authentication, billing/moderation/booking mail, and platform notifications remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="15.75" customHeight="1">
       <x:c r="A125" s="15" t="s">
-        <x:v>329</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="B125" s="2"/>
       <x:c r="C125" s="2"/>
@@ -5224,220 +5203,220 @@
     </x:row>
     <x:row r="126" ht="15.75" customHeight="1">
       <x:c r="A126" s="32" t="s">
-        <x:v>330</x:v>
+        <x:v>326</x:v>
       </x:c>
       <x:c r="B126" s="33" t="s">
-        <x:v>331</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="C126" s="39" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D126" s="35" t="s">
-        <x:v>332</x:v>
+        <x:v>328</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="15.75" customHeight="1">
       <x:c r="A127" s="20" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="B127" s="21" t="s">
-        <x:v>334</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="C127" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D127" s="22" t="s">
-        <x:v>335</x:v>
+        <x:v>331</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="15.75" customHeight="1">
       <x:c r="A128" s="16" t="s">
-        <x:v>336</x:v>
+        <x:v>332</x:v>
       </x:c>
       <x:c r="B128" s="17" t="s">
-        <x:v>337</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="C128" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D128" s="19" t="s">
-        <x:v>338</x:v>
+        <x:v>334</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="15.75" customHeight="1">
       <x:c r="A129" s="20" t="s">
-        <x:v>339</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="B129" s="21" t="s">
-        <x:v>340</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="C129" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D129" s="22" t="s">
-        <x:v>341</x:v>
+        <x:v>337</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="15.75" customHeight="1">
       <x:c r="A130" s="16" t="s">
-        <x:v>342</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="B130" s="17" t="s">
-        <x:v>343</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="C130" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D130" s="19" t="s">
-        <x:v>344</x:v>
+        <x:v>340</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="15" customHeight="1">
       <x:c r="A131" s="20" t="s">
-        <x:v>345</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="B131" s="21" t="s">
-        <x:v>346</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="C131" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D131" s="22" t="s">
-        <x:v>347</x:v>
+        <x:v>343</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="15.75" customHeight="1">
       <x:c r="A132" s="40" t="s">
-        <x:v>348</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="B132" s="41" t="s">
-        <x:v>349</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="C132" s="42" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="D132" s="43" t="s">
-        <x:v>344</x:v>
+        <x:v>340</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="15.75" customHeight="1">
       <x:c r="A133" s="15" t="s">
-        <x:v>350</x:v>
+        <x:v>346</x:v>
       </x:c>
       <x:c r="B133" s="2"/>
       <x:c r="C133" s="2"/>
       <x:c r="D133" s="3"/>
     </x:row>
-    <x:row r="134" ht="15.75" customHeight="1">
+    <x:row r="134" ht="24" hidden="0" customHeight="1">
       <x:c r="A134" s="32" t="s">
-        <x:v>351</x:v>
+        <x:v>347</x:v>
       </x:c>
       <x:c r="B134" s="33" t="s">
-        <x:v>352</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="C134" s="44" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="D134" s="35" t="s">
-        <x:v>353</x:v>
+      <x:c r="D134" s="35" t="str">
+        <x:v>Repository checks and real-stack browser coverage are established, including merged routing, auth, Settings, and creator-application flows. The broader product, beta, payment, moderation, and launch QA checklist remains incomplete.</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="15.75" customHeight="1">
       <x:c r="A135" s="20" t="s">
-        <x:v>354</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="B135" s="21" t="s">
-        <x:v>355</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="C135" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D135" s="22" t="s">
-        <x:v>356</x:v>
+        <x:v>351</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="15.75" customHeight="1">
       <x:c r="A136" s="16" t="s">
-        <x:v>357</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="B136" s="17" t="s">
-        <x:v>358</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="C136" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D136" s="19" t="s">
-        <x:v>359</x:v>
+        <x:v>354</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="15.75" customHeight="1">
       <x:c r="A137" s="20" t="s">
-        <x:v>360</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="B137" s="21" t="s">
-        <x:v>361</x:v>
+        <x:v>356</x:v>
       </x:c>
       <x:c r="C137" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D137" s="22" t="s">
-        <x:v>344</x:v>
+        <x:v>340</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="15.75" customHeight="1">
       <x:c r="A138" s="16" t="s">
-        <x:v>362</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="B138" s="17" t="s">
-        <x:v>363</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="C138" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D138" s="19" t="s">
-        <x:v>364</x:v>
+        <x:v>359</x:v>
       </x:c>
     </x:row>
     <x:row r="139" ht="15.75" customHeight="1">
       <x:c r="A139" s="20" t="s">
-        <x:v>365</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="B139" s="21" t="s">
-        <x:v>366</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="C139" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D139" s="22" t="s">
-        <x:v>367</x:v>
+        <x:v>362</x:v>
       </x:c>
     </x:row>
     <x:row r="140" ht="15.75" customHeight="1">
       <x:c r="A140" s="16" t="s">
-        <x:v>368</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="B140" s="17" t="s">
-        <x:v>369</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="C140" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D140" s="19" t="s">
-        <x:v>370</x:v>
+        <x:v>365</x:v>
       </x:c>
     </x:row>
     <x:row r="141" ht="15.75" customHeight="1">
       <x:c r="A141" s="20" t="s">
-        <x:v>371</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="B141" s="21" t="s">
-        <x:v>372</x:v>
+        <x:v>367</x:v>
       </x:c>
       <x:c r="C141" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="D141" s="22" t="s">
-        <x:v>373</x:v>
+        <x:v>368</x:v>
       </x:c>
     </x:row>
     <x:row r="142" ht="27.75" customHeight="1">
@@ -5648,7 +5627,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="152" ht="31.5" customHeight="1">
+    <x:row r="152" ht="24" hidden="0" customHeight="1">
       <x:c r="A152" s="20" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Implement explicit-content preference</x:t>
@@ -5663,10 +5642,10 @@
         <x:v>🔄 In Progress</x:v>
       </x:c>
       <x:c r="D152" s="22" t="str">
-        <x:v>Default-hidden persistence, protected Settings UI, deliberate opt-in/immediate opt-out, profile and email editing, password change, and active-session controls are locally verified. Onboarding and server-side feed/search/Store/Connect enforcement remain for later phases.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="153" ht="31.5" customHeight="1">
+        <x:v>Default-hidden preference persistence and protected Settings opt-in/immediate opt-out are implemented and CI-verified. Onboarding and server-side feed/search/Store/Connect enforcement remain pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="15" hidden="0" customHeight="1">
       <x:c r="A153" s="16" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Define international launch allowlist</x:t>
@@ -5688,7 +5667,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="154" ht="31.5" customHeight="1">
+    <x:row r="154" ht="15" hidden="0" customHeight="1">
       <x:c r="A154" s="20" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Support Latin American creator onboarding</x:t>
@@ -5710,7 +5689,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="155" ht="31.5" customHeight="1">
+    <x:row r="155" ht="15" hidden="0" customHeight="1">
       <x:c r="A155" s="16" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Select identity verification approach</x:t>
@@ -5732,7 +5711,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="156" ht="31.5" customHeight="1">
+    <x:row r="156" ht="15" hidden="0" customHeight="1">
       <x:c r="A156" s="20" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Define initial media upload limits</x:t>
@@ -5818,7 +5797,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="160" ht="24" hidden="0" customHeight="1">
+    <x:row r="160" ht="36" hidden="0" customHeight="1">
       <x:c r="A160" s="20" t="str">
         <x:v>Define private operations architecture</x:v>
       </x:c>
@@ -5831,7 +5810,7 @@
         </x:is>
       </x:c>
       <x:c r="D160" s="22" t="str">
-        <x:v>The apps/admin build shell now exists. Operational authentication, MFA/SSO, restricted hosting, API integration, permissions, and audit tooling remain pending.</x:v>
+        <x:v>A separate apps/admin shell, dormant injected-verifier review seam, and merged non-secret G1–G12 readiness packet exist. The router is unmounted; production authentication, restricted hosting, phishing-resistant hardware-backed assurance, operator provisioning, origin/CSRF controls, trusted-proxy handling, restricted DB grants, immutable audit, and deployment are absent; all gates are NOT EVALUATED.</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="24" hidden="0" customHeight="1">
@@ -5851,10 +5830,10 @@
         </x:is>
       </x:c>
       <x:c r="D161" s="19" t="str">
-        <x:v>The TypeScript API/contracts/database foundation and the React frontend now include core auth, email verification/password reset, role guards, and DB-backed/browser tests. Remaining frontend migration is incremental.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="162" ht="31.5" customHeight="1">
+        <x:v>TypeScript API/contracts/database foundations now cover auth, protected Settings, creator applications, and the dormant review seam; frontend conversion remains incremental.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="15" hidden="0" customHeight="1">
       <x:c r="A162" s="20" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Replace prototype contact addresses</x:t>
@@ -5876,7 +5855,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="163" ht="31.5" customHeight="1">
+    <x:row r="163" ht="24" hidden="0" customHeight="1">
       <x:c r="A163" s="16" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Prepare public-member / controlled-creator beta</x:t>
@@ -5892,10 +5871,8 @@
           <x:t xml:space="preserve">🔄 In Progress</x:t>
         </x:is>
       </x:c>
-      <x:c r="D163" s="19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">A few initial creators are available; member volume is not yet defined.</x:t>
-        </x:is>
+      <x:c r="D163" s="19" t="str">
+        <x:v>Public member registration exists, while creator applications remain PENDING and identity NOT_STARTED. No approval, role promotion, identity/tax/banking intake, deployed reviewer workflow, or creator publishing gate exists; controlled beta readiness remains incomplete.</x:v>
       </x:c>
     </x:row>
     <x:row r="164" ht="31.5" customHeight="1">
@@ -6793,50 +6770,50 @@
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
       <x:c r="A1" s="14" t="s">
-        <x:v>374</x:v>
+        <x:v>369</x:v>
       </x:c>
       <x:c r="B1" s="14" t="s">
-        <x:v>375</x:v>
+        <x:v>370</x:v>
       </x:c>
       <x:c r="C1" s="14" t="s">
-        <x:v>376</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="D1" s="14" t="s">
-        <x:v>377</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="E1" s="14" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="F1" s="14" t="s">
-        <x:v>378</x:v>
+        <x:v>373</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="20" t="s">
-        <x:v>379</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="B2" s="21" t="s">
-        <x:v>380</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="C2" s="21" t="s">
-        <x:v>381</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="D2" s="21" t="s">
-        <x:v>382</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="E2" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F2" s="21" t="s">
-        <x:v>383</x:v>
+        <x:v>378</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="16" t="s">
-        <x:v>384</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="B3" s="17" t="s">
-        <x:v>380</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="C3" s="21" t="inlineStr">
         <x:is>
@@ -6844,7 +6821,7 @@
         </x:is>
       </x:c>
       <x:c r="D3" s="17" t="s">
-        <x:v>382</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="E3" s="24" t="s">
         <x:v>7</x:v>
@@ -6857,10 +6834,10 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="20" t="s">
-        <x:v>385</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="B4" s="21" t="s">
-        <x:v>386</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="C4" s="21" t="inlineStr">
         <x:is>
@@ -6885,10 +6862,10 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="16" t="s">
-        <x:v>387</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="B5" s="17" t="s">
-        <x:v>386</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="C5" s="17" t="inlineStr">
         <x:is>
@@ -6913,70 +6890,70 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="20" t="s">
-        <x:v>388</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="B6" s="21" t="s">
-        <x:v>389</x:v>
+        <x:v>384</x:v>
       </x:c>
       <x:c r="C6" s="21" t="s">
-        <x:v>390</x:v>
+        <x:v>385</x:v>
       </x:c>
       <x:c r="D6" s="21" t="s">
-        <x:v>382</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="E6" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F6" s="21" t="s">
-        <x:v>383</x:v>
+        <x:v>378</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="16" t="s">
-        <x:v>391</x:v>
+        <x:v>386</x:v>
       </x:c>
       <x:c r="B7" s="17" t="s">
-        <x:v>392</x:v>
+        <x:v>387</x:v>
       </x:c>
       <x:c r="C7" s="17" t="s">
-        <x:v>393</x:v>
+        <x:v>388</x:v>
       </x:c>
       <x:c r="D7" s="17" t="s">
-        <x:v>394</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="E7" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F7" s="17" t="s">
-        <x:v>383</x:v>
+        <x:v>378</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="20" t="s">
-        <x:v>395</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="B8" s="21" t="s">
-        <x:v>396</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="C8" s="21" t="s">
-        <x:v>397</x:v>
+        <x:v>392</x:v>
       </x:c>
       <x:c r="D8" s="21" t="s">
-        <x:v>394</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="E8" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F8" s="21" t="s">
-        <x:v>398</x:v>
+        <x:v>393</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="16" t="s">
-        <x:v>399</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="B9" s="17" t="s">
-        <x:v>380</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="C9" s="17" t="inlineStr">
         <x:is>
@@ -7001,162 +6978,162 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="20" t="s">
-        <x:v>400</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="B10" s="21" t="s">
-        <x:v>386</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="C10" s="21" t="s">
-        <x:v>401</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="D10" s="21" t="s">
-        <x:v>382</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="E10" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F10" s="21" t="s">
-        <x:v>402</x:v>
+        <x:v>397</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="16" t="s">
-        <x:v>403</x:v>
+        <x:v>398</x:v>
       </x:c>
       <x:c r="B11" s="17" t="s">
-        <x:v>386</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="C11" s="17" t="s">
-        <x:v>404</x:v>
+        <x:v>399</x:v>
       </x:c>
       <x:c r="D11" s="17" t="s">
-        <x:v>382</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="E11" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F11" s="17" t="s">
-        <x:v>405</x:v>
+        <x:v>400</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="20" t="s">
-        <x:v>406</x:v>
+        <x:v>401</x:v>
       </x:c>
       <x:c r="B12" s="21" t="s">
-        <x:v>407</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="C12" s="21" t="s">
-        <x:v>408</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="D12" s="21" t="s">
-        <x:v>382</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="E12" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F12" s="21" t="s">
-        <x:v>409</x:v>
+        <x:v>404</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="16" t="s">
-        <x:v>410</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="B13" s="17" t="s">
-        <x:v>411</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="C13" s="17" t="s">
-        <x:v>412</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="D13" s="17" t="s">
-        <x:v>413</x:v>
+        <x:v>408</x:v>
       </x:c>
       <x:c r="E13" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F13" s="17" t="s">
-        <x:v>414</x:v>
+        <x:v>409</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="20" t="s">
-        <x:v>415</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="B14" s="21" t="s">
-        <x:v>416</x:v>
+        <x:v>411</x:v>
       </x:c>
       <x:c r="C14" s="21" t="s">
-        <x:v>417</x:v>
+        <x:v>412</x:v>
       </x:c>
       <x:c r="D14" s="21" t="s">
-        <x:v>394</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="E14" s="24" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F14" s="21" t="s">
-        <x:v>418</x:v>
+        <x:v>413</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="45" t="s">
-        <x:v>419</x:v>
+        <x:v>414</x:v>
       </x:c>
       <x:c r="B15" s="46" t="s">
-        <x:v>420</x:v>
+        <x:v>415</x:v>
       </x:c>
       <x:c r="C15" s="47" t="s">
-        <x:v>421</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="D15" s="46" t="s">
-        <x:v>382</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="E15" s="48" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F15" s="47" t="s">
-        <x:v>422</x:v>
+        <x:v>417</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="49" t="s">
-        <x:v>423</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="B16" s="50" t="s">
-        <x:v>424</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="C16" s="51" t="s">
-        <x:v>425</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="D16" s="50" t="s">
-        <x:v>394</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="E16" s="48" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F16" s="51" t="s">
-        <x:v>426</x:v>
+        <x:v>421</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="52" t="s">
-        <x:v>427</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="B17" s="53" t="s">
-        <x:v>396</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="C17" s="54" t="s">
-        <x:v>428</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="D17" s="53" t="s">
-        <x:v>394</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="E17" s="48" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="F17" s="54" t="s">
-        <x:v>429</x:v>
+        <x:v>424</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1"/>
@@ -8155,306 +8132,306 @@
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>430</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="14" t="s">
-        <x:v>431</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="B3" s="14" t="s">
-        <x:v>432</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
+        <x:v>427</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="55" t="s">
-        <x:v>433</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="B4" s="58" t="str">
-        <x:v>This workbook is reconciled with the repository and founder decisions through July 16, 2026.</x:v>
+        <x:v>This workbook is reconciled with the repository, founder decisions, and merged PR #1–#3 baseline through August 16, 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="57" t="s">
-        <x:v>434</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="B5" s="58" t="s">
-        <x:v>435</x:v>
+        <x:v>430</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="55" t="s">
-        <x:v>436</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="B6" s="56" t="s">
-        <x:v>437</x:v>
+        <x:v>432</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="57" t="s">
-        <x:v>438</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="B7" s="58" t="s">
-        <x:v>439</x:v>
+        <x:v>434</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="55" t="s">
-        <x:v>440</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="B8" s="56" t="s">
-        <x:v>441</x:v>
+        <x:v>436</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="57" t="s">
-        <x:v>442</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="B9" s="58" t="s">
-        <x:v>443</x:v>
+        <x:v>438</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="55" t="s">
-        <x:v>444</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="B10" s="56" t="s">
-        <x:v>445</x:v>
+        <x:v>440</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="57" t="s">
-        <x:v>446</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="B11" s="58" t="s">
-        <x:v>447</x:v>
+        <x:v>442</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="55" t="s">
-        <x:v>448</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="B12" s="56" t="s">
-        <x:v>449</x:v>
+        <x:v>444</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="57" t="s">
-        <x:v>450</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="B13" s="58" t="s">
-        <x:v>451</x:v>
+        <x:v>446</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="55" t="s">
-        <x:v>452</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="B14" s="56" t="s">
-        <x:v>453</x:v>
+        <x:v>448</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="57" t="s">
-        <x:v>454</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="B15" s="58" t="s">
-        <x:v>455</x:v>
+        <x:v>450</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="5" t="s">
-        <x:v>456</x:v>
+        <x:v>451</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B18" s="60" t="s">
-        <x:v>458</x:v>
+        <x:v>453</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B19" s="60" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B20" s="60" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1">
       <x:c r="A21" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B21" s="60" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15.75" customHeight="1">
       <x:c r="A22" s="59" t="s">
+        <x:v>452</x:v>
+      </x:c>
+      <x:c r="B22" s="60" t="s">
         <x:v>457</x:v>
-      </x:c>
-      <x:c r="B22" s="60" t="s">
-        <x:v>462</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15.75" customHeight="1">
       <x:c r="A23" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B23" s="60" t="s">
-        <x:v>463</x:v>
+        <x:v>458</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15.75" customHeight="1">
       <x:c r="A24" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B24" s="60" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15.75" customHeight="1">
       <x:c r="A25" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B25" s="60" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15.75" customHeight="1">
       <x:c r="A26" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B26" s="60" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15.75" customHeight="1">
       <x:c r="A27" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B27" s="60" t="s">
-        <x:v>467</x:v>
+        <x:v>462</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15.75" customHeight="1">
       <x:c r="A28" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B28" s="60" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15.75" customHeight="1">
       <x:c r="A29" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B29" s="60" t="s">
-        <x:v>469</x:v>
+        <x:v>464</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15.75" customHeight="1">
       <x:c r="A30" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B30" s="60" t="s">
-        <x:v>470</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="30" customHeight="1">
+        <x:v>465</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A31" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B31" s="60" t="str">
-        <x:v>Admin operations: separately deployed private app; no public /admin. Backend ADMIN permissions remain API-enforced. 13 subtasks defined.</x:v>
+        <x:v>Admin operations: separate apps/admin shell; no public /admin. Public ADMIN sessions are insufficient for operations access. The dormant review router stays unmounted until signed operations identity, exact provisioning, phishing-resistant hardware-backed assurance, private-origin/CSRF, trusted-proxy, restricted DB-role, audit, and recovery gates pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15.75" customHeight="1">
       <x:c r="A32" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B32" s="60" t="s">
-        <x:v>471</x:v>
+        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15.75" customHeight="1">
       <x:c r="A33" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B33" s="60" t="s">
-        <x:v>472</x:v>
+        <x:v>467</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15.75" customHeight="1">
       <x:c r="A34" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B34" s="60" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15.75" customHeight="1">
       <x:c r="A35" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B35" s="60" t="s">
-        <x:v>474</x:v>
+        <x:v>469</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15.75" customHeight="1">
       <x:c r="A36" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B36" s="60" t="s">
-        <x:v>475</x:v>
+        <x:v>470</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15.75" customHeight="1">
       <x:c r="A37" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B37" s="60" t="s">
-        <x:v>476</x:v>
+        <x:v>471</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15.75" customHeight="1">
       <x:c r="A38" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B38" s="60" t="s">
-        <x:v>477</x:v>
+        <x:v>472</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15.75" customHeight="1">
       <x:c r="A39" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B39" s="60" t="s">
-        <x:v>478</x:v>
+        <x:v>473</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15.75" customHeight="1">
       <x:c r="A40" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B40" s="60" t="s">
-        <x:v>479</x:v>
+        <x:v>474</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15.75" customHeight="1">
       <x:c r="A41" s="59" t="s">
-        <x:v>457</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B41" s="60" t="inlineStr">
         <x:is>
@@ -8470,64 +8447,64 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="44" ht="36" hidden="0" customHeight="1">
+    <x:row r="44" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A44" s="71" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Plan source</x:t>
         </x:is>
       </x:c>
       <x:c r="B44" s="71" t="str">
-        <x:v>PLAN.md is the architecture source of truth. Founder approved a reduced Phase 3 core scope: Slices 1–4B cover auth, roles, core account security, and explicit-content preference persistence; dependency-bound Settings categories remain sequenced later.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="34.5" hidden="0" customHeight="1">
+        <x:v>PLAN.md remains the architecture source of truth. PR #1 merged Phase 4 creator-application persistence plus the dormant non-approval review foundation; PR #2 merged routing hardening; PR #3 merged non-secret operations-readiness documentation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A45" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 1</x:t>
         </x:is>
       </x:c>
       <x:c r="B45" s="73" t="str">
-        <x:v>Founder manually reviews Slice 4B account/security Settings, then commit and publish Slices 4A/4B and require green GitHub CI before starting Phase 4 implementation.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="34.5" hidden="0" customHeight="1">
+        <x:v>PR #1 (e7352c8), PR #2 (1189404), and PR #3 (80efce5) are merged into dev after green reviewed-head CI. The public API still does not mount the creator-review router, and the readiness packet is planning—not live-control evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A46" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 2</x:t>
         </x:is>
       </x:c>
       <x:c r="B46" s="73" t="str">
-        <x:v>Keep Phase 2 labeled partially complete; decide AWS/Sentry/Redis direction and finish staging, backup/restore, monitoring, queueing, and idempotency.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="43.5" hidden="0" customHeight="1">
+        <x:v>Keep Phase 2 labeled partially complete: staging, backup/restore drills, monitoring/alerts, shared Redis throttling, queue/idempotency architecture, and production email decisions remain open.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A47" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 3</x:t>
         </x:is>
       </x:c>
       <x:c r="B47" s="73" t="str">
-        <x:v>Begin Phase 4 with a legal/trust foundation slice: decision register, versioned creator-agreement/acceptance design, pending-review onboarding outcome, and provider interfaces without claiming counsel or vendor approval.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="34.5" hidden="0" customHeight="1">
+        <x:v>Before any private-operations activation, implement and evaluate G1–G12: signed operations identity, exact operator provisioning, phishing-resistant hardware-backed assurance, private origin plus mutation CSRF/origin validation, trusted-proxy handling, restricted database roles, audit destination, recovery, and abuse tests.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A48" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 4</x:t>
         </x:is>
       </x:c>
       <x:c r="B48" s="73" t="str">
-        <x:v>Obtain counsel/CPA guidance and real CCBill, identity-provider, and country-allowlist inputs before implementing irreversible compliance workflows.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="34.5" hidden="0" customHeight="1">
+        <x:v>Obtain counsel/CPA guidance and concrete identity-provider, country-allowlist, retention, CCBill/Epoch, tax, payout, and operational-mailbox inputs before irreversible compliance or payment workflows.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A49" s="72" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Immediate 5</x:t>
         </x:is>
       </x:c>
       <x:c r="B49" s="73" t="str">
-        <x:v>Slice 4A is committed locally as 7972bf2. Slice 4B is implemented and fully locally verified in the working tree; neither local Slice 4 commit has been published or CI-verified yet.</x:v>
+        <x:v>Keep APPROVED, creator-role promotion, identity files, tax/banking intake, payment/ledger effects, creator publishing, staging deployment, and production activation disabled until their legal, provider, security, and operational gates are concrete.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
@@ -8605,7 +8582,7 @@
         <x:v>•</x:v>
       </x:c>
       <x:c r="B60" s="79" t="str">
-        <x:v>Email verification, password reset, and frontend auth integration are implemented locally. Settings, OAuth, a production email provider, and Redis-backed throttling remain later work.</x:v>
+        <x:v>Email verification, password reset, frontend auth integration, protected Settings, and explicit-content preference persistence are published and CI-verified. OAuth, a production email provider, and Redis-backed throttling remain later work.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
@@ -8634,12 +8611,12 @@
         <x:v>Verification and reset tokens are random, hashed at rest, expiring, single-use, and invalidated on reissue; password reset revokes all sessions.</x:v>
       </x:c>
     </x:row>
-    <x:row r="65" ht="36" hidden="0" customHeight="1">
+    <x:row r="65" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A65" t="str">
         <x:v>•</x:v>
       </x:c>
       <x:c r="B65" s="82" t="str">
-        <x:v>Phase 3 Slice 4B locally completes the founder-approved core account-security scope: display-name edit, email change/reverification, authenticated password change, and active-session listing/revocation. Notifications wait for Phase 9; billing for payments; export/deletion for counsel-approved retention; theme for design-system work; explicit-content query enforcement for Phase 5 APIs.</x:v>
+        <x:v>Phase 3 Slice 4B publishes the founder-approved core account-security scope: display-name edit, email change/reverification, authenticated password change, and active-session listing/revocation. Notifications wait for Phase 9; billing for payments; export/deletion for counsel-approved retention; theme for design-system work; explicit-content query enforcement for Phase 5 APIs.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15.75" customHeight="1">
@@ -8793,14 +8770,14 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="79" ht="30" customHeight="1">
+    <x:row r="79" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A79" s="65" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">•</x:t>
         </x:is>
       </x:c>
       <x:c r="B79" s="66" t="str">
-        <x:v>Founder decision (2026-08-01): no public /admin route. An independent apps/admin build shell now exists; backend ADMIN authorization remains, while operational access controls and workflows are Phase 11.</x:v>
+        <x:v>Founder decision (2026-08-01): no public /admin route. A separate apps/admin shell and dormant injected-verifier review seam exist, but public ADMIN authorization alone is insufficient; production operations identity, access controls, workflow UI, and deployment remain absent.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="28.5" customHeight="1">
@@ -9940,7 +9917,7 @@
   <x:sheetData>
     <x:row r="1" ht="39.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>480</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -9952,7 +9929,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="13" t="s">
-        <x:v>481</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -9964,22 +9941,22 @@
     </x:row>
     <x:row r="3" ht="25.5" customHeight="1">
       <x:c r="A3" s="68" t="s">
-        <x:v>482</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="B3" s="68" t="s">
-        <x:v>375</x:v>
+        <x:v>370</x:v>
       </x:c>
       <x:c r="C3" s="68" t="s">
-        <x:v>483</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="D3" s="68" t="s">
-        <x:v>484</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="E3" s="68" t="s">
-        <x:v>485</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="F3" s="68" t="s">
-        <x:v>486</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="G3" s="68" t="s">
         <x:v>22</x:v>
@@ -9990,7 +9967,7 @@
     </x:row>
     <x:row r="4" ht="25.5" customHeight="1">
       <x:c r="A4" s="15" t="s">
-        <x:v>487</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -10002,122 +9979,122 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="16" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="B5" s="17" t="s">
-        <x:v>489</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="C5" s="17" t="s">
-        <x:v>490</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="D5" s="17">
         <x:v>500.0</x:v>
       </x:c>
       <x:c r="E5" s="17"/>
       <x:c r="F5" s="17" t="s">
-        <x:v>491</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="G5" s="24" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H5" s="17" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="20" t="s">
-        <x:v>494</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="B6" s="21" t="s">
-        <x:v>489</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="C6" s="21" t="s">
-        <x:v>490</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="D6" s="21">
         <x:v>500.0</x:v>
       </x:c>
       <x:c r="E6" s="21"/>
       <x:c r="F6" s="21" t="s">
-        <x:v>491</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="G6" s="24" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H6" s="21" t="s">
-        <x:v>495</x:v>
+        <x:v>490</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="16" t="s">
-        <x:v>496</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="B7" s="17" t="s">
-        <x:v>489</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="C7" s="17" t="s">
-        <x:v>490</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="D7" s="17">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E7" s="17"/>
       <x:c r="F7" s="17" t="s">
-        <x:v>491</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="G7" s="24" t="s">
+        <x:v>487</x:v>
+      </x:c>
+      <x:c r="H7" s="17" t="s">
         <x:v>492</x:v>
-      </x:c>
-      <x:c r="H7" s="17" t="s">
-        <x:v>497</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="20" t="s">
-        <x:v>498</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="B8" s="21" t="s">
-        <x:v>499</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="C8" s="21" t="s">
-        <x:v>490</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="D8" s="21">
         <x:v>350.0</x:v>
       </x:c>
       <x:c r="E8" s="21"/>
       <x:c r="F8" s="21" t="s">
-        <x:v>491</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="G8" s="24" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H8" s="21" t="s">
-        <x:v>500</x:v>
+        <x:v>495</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="16" t="s">
-        <x:v>501</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="B9" s="17" t="s">
-        <x:v>499</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="C9" s="17" t="s">
-        <x:v>490</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="D9" s="17">
         <x:v>350.0</x:v>
       </x:c>
       <x:c r="E9" s="17"/>
       <x:c r="F9" s="17" t="s">
-        <x:v>491</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="G9" s="24" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H9" s="17" t="s">
-        <x:v>502</x:v>
+        <x:v>497</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -10127,20 +10104,20 @@
         </x:is>
       </x:c>
       <x:c r="B10" s="21" t="s">
-        <x:v>499</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="C10" s="21" t="s">
-        <x:v>490</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="D10" s="21">
         <x:v>155.0</x:v>
       </x:c>
       <x:c r="E10" s="21"/>
       <x:c r="F10" s="21" t="s">
-        <x:v>491</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="G10" s="24" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H10" s="43" t="inlineStr">
         <x:is>
@@ -10150,103 +10127,103 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="25" t="s">
-        <x:v>503</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="B11" s="21" t="s">
-        <x:v>499</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="C11" s="21" t="s">
-        <x:v>490</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="D11" s="26">
         <x:v>125.0</x:v>
       </x:c>
       <x:c r="E11" s="21"/>
       <x:c r="F11" s="21" t="s">
-        <x:v>491</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="G11" s="24" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H11" s="26" t="s">
-        <x:v>504</x:v>
+        <x:v>499</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="16" t="s">
-        <x:v>505</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="B12" s="17" t="s">
-        <x:v>499</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="C12" s="17" t="s">
-        <x:v>506</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="D12" s="17">
         <x:v>125.0</x:v>
       </x:c>
       <x:c r="E12" s="17"/>
       <x:c r="F12" s="17" t="s">
-        <x:v>507</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="G12" s="24" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H12" s="17" t="s">
-        <x:v>508</x:v>
+        <x:v>503</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="20" t="s">
-        <x:v>509</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="B13" s="21" t="s">
-        <x:v>510</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="C13" s="21" t="s">
-        <x:v>506</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="D13" s="21">
         <x:v>15.0</x:v>
       </x:c>
       <x:c r="E13" s="21"/>
       <x:c r="F13" s="21" t="s">
-        <x:v>507</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="G13" s="24" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H13" s="21" t="s">
-        <x:v>511</x:v>
+        <x:v>506</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="16.5" customHeight="1">
       <x:c r="A14" s="16" t="s">
-        <x:v>512</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="B14" s="17" t="s">
-        <x:v>510</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="C14" s="17" t="s">
-        <x:v>506</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="D14" s="17">
         <x:v>30.0</x:v>
       </x:c>
       <x:c r="E14" s="17"/>
       <x:c r="F14" s="17" t="s">
-        <x:v>507</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="G14" s="24" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H14" s="17" t="s">
-        <x:v>513</x:v>
+        <x:v>508</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="15" t="s">
-        <x:v>514</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="B15" s="2"/>
       <x:c r="C15" s="2"/>
@@ -10258,175 +10235,175 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="32" t="s">
-        <x:v>515</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="B16" s="33" t="s">
-        <x:v>510</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="C16" s="33" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D16" s="33">
         <x:v>18.0</x:v>
       </x:c>
       <x:c r="E16" s="33"/>
       <x:c r="F16" s="33" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="G16" s="39" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H16" s="33" t="s">
-        <x:v>517</x:v>
+        <x:v>512</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="20" t="s">
-        <x:v>518</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="B17" s="21" t="s">
-        <x:v>510</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="C17" s="21" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D17" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E17" s="21"/>
       <x:c r="F17" s="21" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="G17" s="24" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H17" s="21" t="s">
-        <x:v>519</x:v>
+        <x:v>514</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="16" t="s">
-        <x:v>520</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="B18" s="17" t="s">
-        <x:v>510</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="C18" s="17" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D18" s="17">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E18" s="17"/>
       <x:c r="F18" s="17" t="s">
+        <x:v>511</x:v>
+      </x:c>
+      <x:c r="G18" s="24" t="s">
+        <x:v>487</x:v>
+      </x:c>
+      <x:c r="H18" s="17" t="s">
         <x:v>516</x:v>
-      </x:c>
-      <x:c r="G18" s="24" t="s">
-        <x:v>492</x:v>
-      </x:c>
-      <x:c r="H18" s="17" t="s">
-        <x:v>521</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="20" t="s">
-        <x:v>522</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="B19" s="21" t="s">
-        <x:v>510</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="C19" s="21" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D19" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E19" s="21"/>
       <x:c r="F19" s="21" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="G19" s="24" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H19" s="21" t="s">
-        <x:v>523</x:v>
+        <x:v>518</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="16" t="s">
-        <x:v>524</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="B20" s="17" t="s">
-        <x:v>510</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="C20" s="17" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D20" s="17">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E20" s="17"/>
       <x:c r="F20" s="17" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="G20" s="24" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H20" s="17" t="s">
-        <x:v>525</x:v>
+        <x:v>520</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1">
       <x:c r="A21" s="20" t="s">
-        <x:v>526</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="B21" s="21" t="s">
-        <x:v>510</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="C21" s="21" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D21" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E21" s="21"/>
       <x:c r="F21" s="21" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="G21" s="24" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H21" s="21" t="s">
-        <x:v>527</x:v>
+        <x:v>522</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="25.5" customHeight="1">
       <x:c r="A22" s="36" t="s">
-        <x:v>528</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="B22" s="37" t="s">
-        <x:v>510</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="C22" s="37" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D22" s="37">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E22" s="37"/>
       <x:c r="F22" s="37" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="G22" s="30" t="s">
-        <x:v>492</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="H22" s="37" t="s">
-        <x:v>529</x:v>
+        <x:v>524</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15.75" customHeight="1">
       <x:c r="A23" s="15" t="s">
-        <x:v>530</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="B23" s="2"/>
       <x:c r="C23" s="2"/>
@@ -10438,79 +10415,79 @@
     </x:row>
     <x:row r="24" ht="15.75" customHeight="1">
       <x:c r="A24" s="32" t="s">
-        <x:v>531</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="B24" s="33" t="s">
-        <x:v>489</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="C24" s="33" t="s">
-        <x:v>532</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="D24" s="33">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E24" s="33"/>
       <x:c r="F24" s="33" t="s">
-        <x:v>533</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="G24" s="39" t="s">
-        <x:v>534</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="H24" s="33" t="s">
-        <x:v>535</x:v>
+        <x:v>530</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15.75" customHeight="1">
       <x:c r="A25" s="20" t="s">
-        <x:v>536</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="B25" s="21" t="s">
-        <x:v>489</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="C25" s="21" t="s">
-        <x:v>532</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="D25" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E25" s="21"/>
       <x:c r="F25" s="21" t="s">
-        <x:v>533</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="G25" s="24" t="s">
-        <x:v>534</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="H25" s="21" t="s">
-        <x:v>537</x:v>
+        <x:v>532</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="25.5" customHeight="1">
       <x:c r="A26" s="36" t="s">
-        <x:v>538</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="B26" s="37" t="s">
-        <x:v>489</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="C26" s="37" t="s">
-        <x:v>532</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="D26" s="37">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E26" s="37"/>
       <x:c r="F26" s="37" t="s">
-        <x:v>539</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="G26" s="30" t="s">
-        <x:v>534</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="H26" s="37" t="s">
-        <x:v>540</x:v>
+        <x:v>535</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15.75" customHeight="1">
       <x:c r="A27" s="15" t="s">
-        <x:v>541</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="B27" s="2"/>
       <x:c r="C27" s="2"/>
@@ -10522,80 +10499,80 @@
     </x:row>
     <x:row r="28" ht="15.75" customHeight="1">
       <x:c r="A28" s="32" t="s">
-        <x:v>542</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="B28" s="33" t="s">
-        <x:v>489</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="C28" s="33" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D28" s="33">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E28" s="33"/>
       <x:c r="F28" s="33" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="G28" s="39" t="s">
-        <x:v>543</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="H28" s="33" t="s">
-        <x:v>544</x:v>
+        <x:v>539</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15.75" customHeight="1">
       <x:c r="A29" s="20" t="s">
-        <x:v>545</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="B29" s="21" t="s">
-        <x:v>546</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="C29" s="21" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D29" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E29" s="21"/>
       <x:c r="F29" s="21" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="G29" s="24" t="s">
-        <x:v>543</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="H29" s="21" t="s">
-        <x:v>547</x:v>
+        <x:v>542</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15.75" customHeight="1">
       <x:c r="A30" s="16" t="s">
-        <x:v>548</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="B30" s="17" t="s">
-        <x:v>499</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="C30" s="17" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D30" s="17">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E30" s="17"/>
       <x:c r="F30" s="17" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="G30" s="24" t="s">
-        <x:v>543</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="H30" s="17" t="s">
-        <x:v>549</x:v>
+        <x:v>544</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="25.5" customHeight="1"/>
     <x:row r="32" ht="15.75" customHeight="1">
       <x:c r="A32" s="15" t="s">
-        <x:v>550</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="B32" s="2"/>
       <x:c r="C32" s="2"/>
@@ -10607,7 +10584,7 @@
     </x:row>
     <x:row r="33" ht="15.75" customHeight="1">
       <x:c r="A33" s="6" t="s">
-        <x:v>551</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="B33" s="69" t="n">
         <x:f>SUM(D5:D11)</x:f>
@@ -10616,7 +10593,7 @@
     </x:row>
     <x:row r="34" ht="15.75" customHeight="1">
       <x:c r="A34" s="7" t="s">
-        <x:v>552</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="B34" s="70">
         <x:v>170.0</x:v>
@@ -10624,7 +10601,7 @@
     </x:row>
     <x:row r="35" ht="15.75" customHeight="1">
       <x:c r="A35" s="6" t="s">
-        <x:v>553</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="B35" s="69">
         <x:v>18.0</x:v>
@@ -10632,7 +10609,7 @@
     </x:row>
     <x:row r="36" ht="15.75" customHeight="1">
       <x:c r="A36" s="7" t="s">
-        <x:v>554</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="B36" s="70">
         <x:v>1713.0</x:v>

</xml_diff>

<commit_message>
docs: improve tracker clarity and phase evidence
</commit_message>
<xml_diff>
--- a/docs/product/Pumdoki_MasterTracker_V4.xlsx
+++ b/docs/product/Pumdoki_MasterTracker_V4.xlsx
@@ -2,17 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf6630ba481e94be7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="Reeb1534517094ca0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="Re100dde6f21f4557"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="R15e3888a2bc34cdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="Re956c19721934516"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legacy Overview 2026-08-16" sheetId="6" r:id="R00d87ed93e304a53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="7" r:id="Rb691168d53c749e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Roadmap" sheetId="8" r:id="R2c9454b7a7b74252"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Tracker" sheetId="9" r:id="Rd146d55f483e40f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Log" sheetId="10" r:id="R39c42f2eb66d476b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Register" sheetId="11" r:id="Rb26ed71df58647c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc85fc3fbe2e74df0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R28f114d80f1348fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R7a2e21f361534518"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="Re271bb41e4214da8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R0e7115ce53bf44d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legacy Overview 2026-08-16" sheetId="6" r:id="R999a5dfe37e24557"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="7" r:id="Rd3e1530812054b35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Roadmap" sheetId="8" r:id="R61e5aa682ecb4019"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Tracker" sheetId="9" r:id="Re238eabfe7084ebe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Blocker Queue" sheetId="10" r:id="Re9c8b707730a45d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Log" sheetId="11" r:id="Refb2f3deb3b540d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Register" sheetId="12" r:id="R64af974bd2184856"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2013,7 +2014,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="161">
+  <x:cellXfs count="164">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -2481,6 +2482,15 @@
     <x:xf numFmtId="164" fontId="24" fillId="13" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
@@ -2491,7 +2501,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="27">
+  <x:dxfs count="34">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -2522,6 +2532,28 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFDDF3E4"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF246B3B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDDF3E4"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF805E00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF1C9"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -2594,6 +2626,28 @@
     <x:dxf>
       <x:font>
         <x:b/>
+        <x:color rgb="FF245B84"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDDEBFA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A2432"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF9D7DC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
         <x:color rgb="FF8A2432"/>
       </x:font>
       <x:fill>
@@ -2660,6 +2714,17 @@
     <x:dxf>
       <x:font>
         <x:b/>
+        <x:color rgb="FF5D535C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFECE8EC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
         <x:color rgb="FF3D1A3E"/>
       </x:font>
       <x:fill>
@@ -2687,6 +2752,28 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFAE1EC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF3D1A3E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFAE1EC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF5D535C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFECE8EC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -2794,16 +2881,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PhaseRoadmapTable" displayName="PhaseRoadmapTable" ref="A3:P19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PhaseRoadmapTable" displayName="PhaseRoadmapTable" ref="A3:P19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A3:P19"/>
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="Phase ID"/>
     <x:tableColumn id="2" name="PLAN Phase"/>
     <x:tableColumn id="3" name="Phase State"/>
     <x:tableColumn id="4" name="Maturity"/>
-    <x:tableColumn id="5" name="Done"/>
-    <x:tableColumn id="6" name="Total"/>
-    <x:tableColumn id="7" name="Task Progress"/>
+    <x:tableColumn id="5" name="Records Done"/>
+    <x:tableColumn id="6" name="Execution Records"/>
+    <x:tableColumn id="7" name="Record Progress"/>
     <x:tableColumn id="8" name="In Progress"/>
     <x:tableColumn id="9" name="In Review"/>
     <x:tableColumn id="10" name="Blocked"/>
@@ -2819,8 +2906,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorkItemsTable" displayName="WorkItemsTable" ref="A3:S159" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:S159"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorkItemsTable" displayName="WorkItemsTable" ref="A3:S161" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:S161"/>
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="Work ID"/>
     <x:tableColumn id="2" name="Phase ID"/>
@@ -2847,7 +2934,28 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DailyLogTable" displayName="DailyLogTable" ref="A3:L63" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ReviewQueueTable" displayName="ReviewQueueTable" ref="A3:L9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:L9"/>
+  <x:tableColumns count="12">
+    <x:tableColumn id="1" name="Work ID"/>
+    <x:tableColumn id="2" name="Phase"/>
+    <x:tableColumn id="3" name="PLAN Phase"/>
+    <x:tableColumn id="4" name="Workstream"/>
+    <x:tableColumn id="5" name="Work Item"/>
+    <x:tableColumn id="6" name="Workflow"/>
+    <x:tableColumn id="7" name="Owner"/>
+    <x:tableColumn id="8" name="Waiting On / Reviewer"/>
+    <x:tableColumn id="9" name="Next Action"/>
+    <x:tableColumn id="10" name="Next Check"/>
+    <x:tableColumn id="11" name="Evidence"/>
+    <x:tableColumn id="12" name="Updated"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DailyLogTable" displayName="DailyLogTable" ref="A3:L63" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A3:L63"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Date"/>
@@ -2867,8 +2975,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DecisionRegisterTable" displayName="DecisionRegisterTable" ref="A3:J18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DecisionRegisterTable" displayName="DecisionRegisterTable" ref="A3:J18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A3:J18"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Decision ID"/>
@@ -3118,7 +3226,7 @@
     </x:row>
     <x:row r="2" ht="21.75" customHeight="1">
       <x:c r="A2" s="92" t="str">
-        <x:v>PLAN.md-aligned view · refreshed August 21, 2026 · task counts are not production-readiness claims</x:v>
+        <x:v>PLAN.md-aligned view · refreshed August 21, 2026 · record counts are navigation metrics, not phase completion or production-readiness claims</x:v>
       </x:c>
       <x:c r="B2" s="92"/>
       <x:c r="C2" s="92"/>
@@ -3254,7 +3362,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="138" t="str">
-        <x:v>Total items</x:v>
+        <x:v>Execution records</x:v>
       </x:c>
       <x:c r="B12" s="139"/>
       <x:c r="C12" s="138" t="str">
@@ -3278,19 +3386,19 @@
       </x:c>
       <x:c r="L12" s="139"/>
       <x:c r="M12" s="138" t="str">
-        <x:v>Task progress</x:v>
+        <x:v>Record progress</x:v>
       </x:c>
       <x:c r="N12" s="139"/>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="150" t="n">
         <x:f>COUNTA('Delivery Tracker'!$A$4:$A$400)</x:f>
-        <x:v>156</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B13" s="151"/>
       <x:c r="C13" s="150" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$H$4:$H$400,"Done")</x:f>
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D13" s="151"/>
       <x:c r="E13" s="150" t="n">
@@ -3315,7 +3423,7 @@
       <x:c r="L13" s="151"/>
       <x:c r="M13" s="158" t="n">
         <x:f>IF(A13=0,0,C13/A13)</x:f>
-        <x:v>0.1282051282051282</x:v>
+        <x:v>0.13924050632911392</x:v>
       </x:c>
       <x:c r="N13" s="151"/>
     </x:row>
@@ -3365,19 +3473,19 @@
         <x:v>PLAN phase</x:v>
       </x:c>
       <x:c r="C17" s="98" t="str">
-        <x:v>State</x:v>
+        <x:v>Phase State</x:v>
       </x:c>
       <x:c r="D17" s="98" t="str">
         <x:v>Maturity</x:v>
       </x:c>
       <x:c r="E17" s="98" t="str">
-        <x:v>Done</x:v>
+        <x:v>Records Done</x:v>
       </x:c>
       <x:c r="F17" s="98" t="str">
-        <x:v>Total</x:v>
+        <x:v>Execution Records</x:v>
       </x:c>
       <x:c r="G17" s="98" t="str">
-        <x:v>Progress</x:v>
+        <x:v>Record Progress</x:v>
       </x:c>
       <x:c r="H17" s="98" t="str">
         <x:v>In Progress</x:v>
@@ -3652,15 +3760,15 @@
       </x:c>
       <x:c r="E22" s="111" t="n">
         <x:f>'Phase Roadmap'!E8</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F22" s="111" t="n">
         <x:f>'Phase Roadmap'!F8</x:f>
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="G22" s="119" t="n">
         <x:f>'Phase Roadmap'!G8</x:f>
-        <x:v>0</x:v>
+        <x:v>0.0625</x:v>
       </x:c>
       <x:c r="H22" s="111" t="n">
         <x:f>'Phase Roadmap'!H8</x:f>
@@ -4295,25 +4403,25 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B35" s="109" t="str">
-        <x:v>Use Delivery Tracker for current execution status.</x:v>
+        <x:v>Start with Review &amp; Blocker Queue for immediate attention.</x:v>
       </x:c>
       <x:c r="C35" s="109" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D35" s="109" t="str">
-        <x:v>Use Phase Roadmap for phase-level truth and exit gates.</x:v>
+        <x:v>Use Delivery Tracker for canonical execution status.</x:v>
       </x:c>
       <x:c r="E35" s="109" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F35" s="109" t="str">
-        <x:v>Use Daily Log for each meaningful work-session debrief.</x:v>
+        <x:v>Use Phase Roadmap for evidence-based phase state and exit gates.</x:v>
       </x:c>
       <x:c r="G35" s="109" t="str">
         <x:v>4</x:v>
       </x:c>
       <x:c r="H35" s="109" t="str">
-        <x:v>Use Decision Register for founder/legal/provider blockers.</x:v>
+        <x:v>Use Daily Log for each meaningful work-session debrief.</x:v>
       </x:c>
       <x:c r="I35" s="109" t="str">
         <x:v>5</x:v>
@@ -4402,10 +4510,10 @@
         <x:v>PLAN.md = phase architecture; Delivery Tracker = current execution; HANDOFF.md = active technical evidence.</x:v>
       </x:c>
       <x:c r="C38" s="111" t="str">
-        <x:v>Last refresh</x:v>
+        <x:v>Metric rule</x:v>
       </x:c>
       <x:c r="D38" s="111" t="str">
-        <x:v>2026-08-21</x:v>
+        <x:v>Record progress counts preserved/current records; Phase State is the canonical PLAN judgment.</x:v>
       </x:c>
       <x:c r="E38" s="111" t="str">
         <x:v>Current branch</x:v>
@@ -5426,6 +5534,341 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="9" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="36" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="42" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="13" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="88" t="str">
+        <x:v>🔎 Pumdoki Review &amp; Blocker Queue</x:v>
+      </x:c>
+      <x:c r="B1" s="88"/>
+      <x:c r="C1" s="88"/>
+      <x:c r="D1" s="88"/>
+      <x:c r="E1" s="88"/>
+      <x:c r="F1" s="88"/>
+      <x:c r="G1" s="88"/>
+      <x:c r="H1" s="88"/>
+      <x:c r="I1" s="88"/>
+      <x:c r="J1" s="88"/>
+      <x:c r="K1" s="88"/>
+      <x:c r="L1" s="88"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="92" t="str">
+        <x:v>Focused view derived from Delivery Tracker. Update the canonical source row there; use this sheet for daily review and blocker triage.</x:v>
+      </x:c>
+      <x:c r="B2" s="92"/>
+      <x:c r="C2" s="92"/>
+      <x:c r="D2" s="92"/>
+      <x:c r="E2" s="92"/>
+      <x:c r="F2" s="92"/>
+      <x:c r="G2" s="92"/>
+      <x:c r="H2" s="92"/>
+      <x:c r="I2" s="92"/>
+      <x:c r="J2" s="92"/>
+      <x:c r="K2" s="92"/>
+      <x:c r="L2" s="92"/>
+    </x:row>
+    <x:row r="3" ht="34" customHeight="1">
+      <x:c r="A3" s="98" t="str">
+        <x:v>Work ID</x:v>
+      </x:c>
+      <x:c r="B3" s="98" t="str">
+        <x:v>Phase</x:v>
+      </x:c>
+      <x:c r="C3" s="98" t="str">
+        <x:v>PLAN Phase</x:v>
+      </x:c>
+      <x:c r="D3" s="98" t="str">
+        <x:v>Workstream</x:v>
+      </x:c>
+      <x:c r="E3" s="98" t="str">
+        <x:v>Work Item</x:v>
+      </x:c>
+      <x:c r="F3" s="98" t="str">
+        <x:v>Workflow</x:v>
+      </x:c>
+      <x:c r="G3" s="98" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="H3" s="98" t="str">
+        <x:v>Waiting On / Reviewer</x:v>
+      </x:c>
+      <x:c r="I3" s="98" t="str">
+        <x:v>Next Action</x:v>
+      </x:c>
+      <x:c r="J3" s="98" t="str">
+        <x:v>Next Check</x:v>
+      </x:c>
+      <x:c r="K3" s="98" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="L3" s="98" t="str">
+        <x:v>Updated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="54" customHeight="1">
+      <x:c r="A4" s="109" t="str">
+        <x:v>P00-T03</x:v>
+      </x:c>
+      <x:c r="B4" s="109" t="str">
+        <x:v>P00</x:v>
+      </x:c>
+      <x:c r="C4" s="109" t="str">
+        <x:v>Baseline, tracker, and scope control</x:v>
+      </x:c>
+      <x:c r="D4" s="109" t="str">
+        <x:v>Tracker &amp; scope control</x:v>
+      </x:c>
+      <x:c r="E4" s="109" t="str">
+        <x:v>Reclassify the tracker to PLAN.md Phases 0–14</x:v>
+      </x:c>
+      <x:c r="F4" s="109" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="G4" s="109" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="H4" s="109" t="str">
+        <x:v>Founder review</x:v>
+      </x:c>
+      <x:c r="I4" s="109" t="str">
+        <x:v>Review the reorganized workbook in draft PR #13; preserve the legacy tracker as the source snapshot.</x:v>
+      </x:c>
+      <x:c r="J4" s="110" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+      <x:c r="K4" s="109" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
+      </x:c>
+      <x:c r="L4" s="110" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="54" customHeight="1">
+      <x:c r="A5" s="111" t="str">
+        <x:v>P02-T11</x:v>
+      </x:c>
+      <x:c r="B5" s="111" t="str">
+        <x:v>P02</x:v>
+      </x:c>
+      <x:c r="C5" s="111" t="str">
+        <x:v>Backend and database foundation</x:v>
+      </x:c>
+      <x:c r="D5" s="111" t="str">
+        <x:v>Durable async work</x:v>
+      </x:c>
+      <x:c r="E5" s="111" t="str">
+        <x:v>Add a background-job queue</x:v>
+      </x:c>
+      <x:c r="F5" s="111" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="G5" s="111" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="H5" s="111" t="str">
+        <x:v>Founder review + fresh CI</x:v>
+      </x:c>
+      <x:c r="I5" s="111" t="str">
+        <x:v>Review the application-owned PostgreSQL worker foundation on PR #13; merge remains separately gated.</x:v>
+      </x:c>
+      <x:c r="J5" s="112" t="n">
+        <x:v>46259.666666666664</x:v>
+      </x:c>
+      <x:c r="K5" s="111" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
+      </x:c>
+      <x:c r="L5" s="112" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="54" customHeight="1">
+      <x:c r="A6" s="111" t="str">
+        <x:v>P02-T12A</x:v>
+      </x:c>
+      <x:c r="B6" s="111" t="str">
+        <x:v>P02</x:v>
+      </x:c>
+      <x:c r="C6" s="111" t="str">
+        <x:v>Backend and database foundation</x:v>
+      </x:c>
+      <x:c r="D6" s="111" t="str">
+        <x:v>Durable async work</x:v>
+      </x:c>
+      <x:c r="E6" s="111" t="str">
+        <x:v>Prove canary-specific idempotency and lease fencing</x:v>
+      </x:c>
+      <x:c r="F6" s="111" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="G6" s="111" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="H6" s="111" t="str">
+        <x:v>Founder review + fresh CI</x:v>
+      </x:c>
+      <x:c r="I6" s="111" t="str">
+        <x:v>Review atomic enqueue/replay, stale-token rejection, effect reconciliation, and exact-role evidence in PR #13.</x:v>
+      </x:c>
+      <x:c r="J6" s="112" t="n">
+        <x:v>46259.666666666664</x:v>
+      </x:c>
+      <x:c r="K6" s="111" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
+      </x:c>
+      <x:c r="L6" s="112" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="54" customHeight="1">
+      <x:c r="A7" s="111" t="str">
+        <x:v>P02-NET-001</x:v>
+      </x:c>
+      <x:c r="B7" s="111" t="str">
+        <x:v>P02</x:v>
+      </x:c>
+      <x:c r="C7" s="111" t="str">
+        <x:v>Backend and database foundation</x:v>
+      </x:c>
+      <x:c r="D7" s="111" t="str">
+        <x:v>Local security</x:v>
+      </x:c>
+      <x:c r="E7" s="111" t="str">
+        <x:v>Bind local PostgreSQL host exposure to IPv4 loopback</x:v>
+      </x:c>
+      <x:c r="F7" s="111" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="G7" s="111" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="H7" s="111" t="str">
+        <x:v>Founder review + fresh CI</x:v>
+      </x:c>
+      <x:c r="I7" s="111" t="str">
+        <x:v>Verify the tracked Compose mapping remains 127.0.0.1-only and the named volume is preserved.</x:v>
+      </x:c>
+      <x:c r="J7" s="112" t="n">
+        <x:v>46259.666666666664</x:v>
+      </x:c>
+      <x:c r="K7" s="111" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
+      </x:c>
+      <x:c r="L7" s="112" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="54" customHeight="1">
+      <x:c r="A8" s="111" t="str">
+        <x:v>P07-E2E-001</x:v>
+      </x:c>
+      <x:c r="B8" s="111" t="str">
+        <x:v>P07</x:v>
+      </x:c>
+      <x:c r="C8" s="111" t="str">
+        <x:v>Core end-to-end vertical slice</x:v>
+      </x:c>
+      <x:c r="D8" s="111" t="str">
+        <x:v>Core vertical slice</x:v>
+      </x:c>
+      <x:c r="E8" s="111" t="str">
+        <x:v>Complete the member-to-creator end-to-end product flow</x:v>
+      </x:c>
+      <x:c r="F8" s="111" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="G8" s="111" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="H8" s="111" t="str">
+        <x:v>Phase 4–6 dependencies</x:v>
+      </x:c>
+      <x:c r="I8" s="111" t="str">
+        <x:v>Do not begin the product slice until creator approval, media entitlement, and payment-ledger prerequisites are accepted.</x:v>
+      </x:c>
+      <x:c r="J8" s="112"/>
+      <x:c r="K8" s="111" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/PLAN.md#11-phase-7--core-end-to-end-vertical-slice</x:v>
+      </x:c>
+      <x:c r="L8" s="112" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="54" customHeight="1">
+      <x:c r="A9" s="111" t="str">
+        <x:v>P14-QA-001</x:v>
+      </x:c>
+      <x:c r="B9" s="111" t="str">
+        <x:v>P14</x:v>
+      </x:c>
+      <x:c r="C9" s="111" t="str">
+        <x:v>QA, security, private beta, and launch</x:v>
+      </x:c>
+      <x:c r="D9" s="111" t="str">
+        <x:v>Deterministic E2E</x:v>
+      </x:c>
+      <x:c r="E9" s="111" t="str">
+        <x:v>Make promotion material E2E independent of calendar date</x:v>
+      </x:c>
+      <x:c r="F9" s="111" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="G9" s="111" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="H9" s="111" t="str">
+        <x:v>Fresh CI</x:v>
+      </x:c>
+      <x:c r="I9" s="111" t="str">
+        <x:v>Keep the Playwright test clock fixed before navigation so active-promotion fixtures do not expire with wall time.</x:v>
+      </x:c>
+      <x:c r="J9" s="112" t="n">
+        <x:v>46259.666666666664</x:v>
+      </x:c>
+      <x:c r="K9" s="111" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
+      </x:c>
+      <x:c r="L9" s="112" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:L1"/>
+    <x:mergeCell ref="A2:L2"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="F4:F9">
+    <x:cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Done"/>
+    <x:cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="9" priority="3" operator="containsText" text="In Review"/>
+    <x:cfRule type="containsText" dxfId="13" priority="4" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="17" priority="5" operator="containsText" text="Not Started"/>
+    <x:cfRule type="containsText" dxfId="21" priority="6" operator="containsText" text="Ready"/>
+    <x:cfRule type="containsText" dxfId="25" priority="7" operator="containsText" text="Deferred"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31b72b6e3a224058"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="13" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
@@ -6428,13 +6871,13 @@
     <x:mergeCell ref="A2:L2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="I4:I63">
-    <x:cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Done"/>
-    <x:cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="In Progress"/>
-    <x:cfRule type="containsText" dxfId="7" priority="3" operator="containsText" text="In Review"/>
-    <x:cfRule type="containsText" dxfId="10" priority="4" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="13" priority="5" operator="containsText" text="Not Started"/>
-    <x:cfRule type="containsText" dxfId="16" priority="6" operator="containsText" text="Ready"/>
-    <x:cfRule type="containsText" dxfId="19" priority="7" operator="containsText" text="Deferred"/>
+    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Done"/>
+    <x:cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="10" priority="3" operator="containsText" text="In Review"/>
+    <x:cfRule type="containsText" dxfId="14" priority="4" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="18" priority="5" operator="containsText" text="Not Started"/>
+    <x:cfRule type="containsText" dxfId="22" priority="6" operator="containsText" text="Ready"/>
+    <x:cfRule type="containsText" dxfId="26" priority="7" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="I4:I63">
@@ -6443,12 +6886,12 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb872f174d5f74080"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18a5b4d9a8544742"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -6992,13 +7435,13 @@
     <x:mergeCell ref="A2:J2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="F4:F18">
-    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Done"/>
-    <x:cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="In Progress"/>
-    <x:cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="In Review"/>
-    <x:cfRule type="containsText" dxfId="11" priority="4" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="14" priority="5" operator="containsText" text="Not Started"/>
-    <x:cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="Ready"/>
-    <x:cfRule type="containsText" dxfId="20" priority="7" operator="containsText" text="Deferred"/>
+    <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Done"/>
+    <x:cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="11" priority="3" operator="containsText" text="In Review"/>
+    <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="19" priority="5" operator="containsText" text="Not Started"/>
+    <x:cfRule type="containsText" dxfId="23" priority="6" operator="containsText" text="Ready"/>
+    <x:cfRule type="containsText" dxfId="27" priority="7" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="F4:F18">
@@ -7010,7 +7453,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc78859faa91e439d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb048690bc2e412d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12537,7 +12980,12 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="97" ht="15.75" customHeight="1"/>
+    <x:row r="97" ht="42" customHeight="1">
+      <x:c r="A97" s="161" t="str">
+        <x:v>Historical/current boundary: rows 1–96 preserve the August 16 baseline; current operating notes begin below.</x:v>
+      </x:c>
+      <x:c r="B97" s="161"/>
+    </x:row>
     <x:row r="98" ht="42" customHeight="1">
       <x:c r="A98" s="124" t="str">
         <x:v>📌 Tracker Operating Model — August 21, 2026</x:v>
@@ -12545,7 +12993,7 @@
       <x:c r="B98" s="124"/>
     </x:row>
     <x:row r="99" ht="42" customHeight="1">
-      <x:c r="A99" s="159" t="str">
+      <x:c r="A99" s="162" t="str">
         <x:v>Source of truth</x:v>
       </x:c>
       <x:c r="B99" s="109" t="str">
@@ -12553,7 +13001,7 @@
       </x:c>
     </x:row>
     <x:row r="100" ht="42" customHeight="1">
-      <x:c r="A100" s="160" t="str">
+      <x:c r="A100" s="163" t="str">
         <x:v>Legacy preservation</x:v>
       </x:c>
       <x:c r="B100" s="111" t="str">
@@ -12561,7 +13009,7 @@
       </x:c>
     </x:row>
     <x:row r="101" ht="42" customHeight="1">
-      <x:c r="A101" s="160" t="str">
+      <x:c r="A101" s="163" t="str">
         <x:v>Workflow</x:v>
       </x:c>
       <x:c r="B101" s="111" t="str">
@@ -12569,15 +13017,15 @@
       </x:c>
     </x:row>
     <x:row r="102" ht="42" customHeight="1">
-      <x:c r="A102" s="160" t="str">
+      <x:c r="A102" s="163" t="str">
         <x:v>Maturity</x:v>
       </x:c>
       <x:c r="B102" s="111" t="str">
-        <x:v>Decision Locked, UI Prototype, Backend Implemented, Integrated, Production-Ready, N/A. Workflow Done never automatically means Production-Ready.</x:v>
+        <x:v>Decision Locked means product scope or architecture direction only—never counsel-approved copy or provider approval. Workflow Done never automatically means Production-Ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="42" customHeight="1">
-      <x:c r="A103" s="160" t="str">
+      <x:c r="A103" s="163" t="str">
         <x:v>Daily debrief</x:v>
       </x:c>
       <x:c r="B103" s="111" t="str">
@@ -12585,7 +13033,7 @@
       </x:c>
     </x:row>
     <x:row r="104" ht="42" customHeight="1">
-      <x:c r="A104" s="160" t="str">
+      <x:c r="A104" s="163" t="str">
         <x:v>Current focus</x:v>
       </x:c>
       <x:c r="B104" s="111" t="str">
@@ -12593,7 +13041,7 @@
       </x:c>
     </x:row>
     <x:row r="105" ht="42" customHeight="1">
-      <x:c r="A105" s="160" t="str">
+      <x:c r="A105" s="163" t="str">
         <x:v>Phase 4</x:v>
       </x:c>
       <x:c r="B105" s="111" t="str">
@@ -12601,7 +13049,7 @@
       </x:c>
     </x:row>
     <x:row r="106" ht="42" customHeight="1">
-      <x:c r="A106" s="160" t="str">
+      <x:c r="A106" s="163" t="str">
         <x:v>Expense QC</x:v>
       </x:c>
       <x:c r="B106" s="111" t="str">
@@ -12609,7 +13057,7 @@
       </x:c>
     </x:row>
     <x:row r="107" ht="42" customHeight="1">
-      <x:c r="A107" s="160" t="str">
+      <x:c r="A107" s="163" t="str">
         <x:v>Last refreshed</x:v>
       </x:c>
       <x:c r="B107" s="111" t="str">
@@ -13517,6 +13965,7 @@
     <x:mergeCell ref="A66:B66"/>
     <x:mergeCell ref="A52:B52"/>
     <x:mergeCell ref="A62:B62"/>
+    <x:mergeCell ref="A97:B97"/>
     <x:mergeCell ref="A98:B98"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15503,7 +15952,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="111" t="str">
-        <x:v>Use Overview, Phase Roadmap, Delivery Tracker, Daily Log, and Decision Register for current project management.</x:v>
+        <x:v>Use Overview, Phase Roadmap, Delivery Tracker, Review &amp; Blocker Queue, Daily Log, and Decision Register for current project management.</x:v>
       </x:c>
       <x:c r="B25" s="111"/>
       <x:c r="C25" s="111"/>
@@ -15644,7 +16093,7 @@
         <x:v>Engineering</x:v>
       </x:c>
       <x:c r="G6" s="111" t="str">
-        <x:v>Supplemental</x:v>
+        <x:v>PLAN phase gate</x:v>
       </x:c>
       <x:c r="H6" s="111" t="str">
         <x:v>Partially Complete</x:v>
@@ -15670,7 +16119,7 @@
         <x:v>Operations</x:v>
       </x:c>
       <x:c r="G7" s="111" t="str">
-        <x:v>Legacy-mapped task</x:v>
+        <x:v>Supplemental</x:v>
       </x:c>
       <x:c r="H7" s="111" t="str">
         <x:v>Foundation Complete</x:v>
@@ -15696,7 +16145,7 @@
         <x:v>Counsel</x:v>
       </x:c>
       <x:c r="G8" s="111" t="str">
-        <x:v>Decision</x:v>
+        <x:v>Legacy-mapped task</x:v>
       </x:c>
       <x:c r="H8" s="111" t="str">
         <x:v>Complete</x:v>
@@ -15720,7 +16169,7 @@
         <x:v>Unassigned</x:v>
       </x:c>
       <x:c r="G9" s="111" t="str">
-        <x:v>Exit criterion</x:v>
+        <x:v>Published slice</x:v>
       </x:c>
       <x:c r="H9" s="111" t="str">
         <x:v>Blocked</x:v>
@@ -15741,7 +16190,9 @@
       </x:c>
       <x:c r="E10" s="111" t="str"/>
       <x:c r="F10" s="111" t="str"/>
-      <x:c r="G10" s="111" t="str"/>
+      <x:c r="G10" s="111" t="str">
+        <x:v>Decision</x:v>
+      </x:c>
       <x:c r="H10" s="111" t="str">
         <x:v>Deferred</x:v>
       </x:c>
@@ -15759,7 +16210,9 @@
       <x:c r="D11" s="111" t="str"/>
       <x:c r="E11" s="111" t="str"/>
       <x:c r="F11" s="111" t="str"/>
-      <x:c r="G11" s="111" t="str"/>
+      <x:c r="G11" s="111" t="str">
+        <x:v>Exit criterion</x:v>
+      </x:c>
       <x:c r="H11" s="111" t="str"/>
     </x:row>
     <x:row r="12">
@@ -15952,7 +16405,7 @@
         <x:v>Decision Locked</x:v>
       </x:c>
       <x:c r="E26" s="111" t="str">
-        <x:v>Direction is approved; implementation may still be absent.</x:v>
+        <x:v>Product scope or architecture direction is approved; implementation may be absent. This never means counsel-approved copy, provider approval, or production readiness.</x:v>
       </x:c>
       <x:c r="F26" s="111"/>
       <x:c r="G26" s="111" t="str">
@@ -16140,7 +16593,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="92" t="str">
-        <x:v>Task-count progress is a navigation aid, not a production-readiness claim. Phase State remains an explicit evidence-based judgment.</x:v>
+        <x:v>Record progress includes preserved legacy, PLAN, gate, and supplemental records. It is a navigation aid—not phase completion; Phase State is the canonical evidence-based PLAN judgment.</x:v>
       </x:c>
       <x:c r="B2" s="92"/>
       <x:c r="C2" s="92"/>
@@ -16172,13 +16625,13 @@
         <x:v>Maturity</x:v>
       </x:c>
       <x:c r="E3" s="98" t="str">
-        <x:v>Done</x:v>
+        <x:v>Records Done</x:v>
       </x:c>
       <x:c r="F3" s="98" t="str">
-        <x:v>Total</x:v>
+        <x:v>Execution Records</x:v>
       </x:c>
       <x:c r="G3" s="98" t="str">
-        <x:v>Task Progress</x:v>
+        <x:v>Record Progress</x:v>
       </x:c>
       <x:c r="H3" s="98" t="str">
         <x:v>In Progress</x:v>
@@ -16451,15 +16904,15 @@
       </x:c>
       <x:c r="E8" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A8,'Delivery Tracker'!$H$4:$H$400,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F8" s="111" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$B$4:$B$400,$A8)</x:f>
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="G8" s="119" t="n">
         <x:f>IF(F8=0,0,E8/F8)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.0625</x:v>
       </x:c>
       <x:c r="H8" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A8,'Delivery Tracker'!$H$4:$H$400,"In Progress")</x:f>
@@ -17126,12 +17579,12 @@
     <x:mergeCell ref="A2:P2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="C4:C19">
-    <x:cfRule type="containsText" dxfId="21" priority="1" operator="containsText" text="Complete"/>
-    <x:cfRule type="containsText" dxfId="22" priority="2" operator="containsText" text="Partially Complete"/>
-    <x:cfRule type="containsText" dxfId="23" priority="3" operator="containsText" text="Foundation Complete"/>
-    <x:cfRule type="containsText" dxfId="24" priority="4" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="25" priority="5" operator="containsText" text="Not Started"/>
-    <x:cfRule type="containsText" dxfId="26" priority="6" operator="containsText" text="Deferred"/>
+    <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Complete"/>
+    <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="Partially Complete"/>
+    <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Foundation Complete"/>
+    <x:cfRule type="containsText" dxfId="31" priority="4" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="32" priority="5" operator="containsText" text="Not Started"/>
+    <x:cfRule type="containsText" dxfId="33" priority="6" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="C4:C19">
@@ -17143,7 +17596,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8170aea414c047df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R376c4f1564a14df6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17561,7 +18014,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I9" s="111" t="str">
-        <x:v>Decision Locked</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="J9" s="111" t="str">
         <x:v>Critical</x:v>
@@ -17612,7 +18065,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I10" s="111" t="str">
-        <x:v>Decision Locked</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="J10" s="111" t="str">
         <x:v>Medium</x:v>
@@ -17714,7 +18167,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I12" s="111" t="str">
-        <x:v>Decision Locked</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="J12" s="111" t="str">
         <x:v>High</x:v>
@@ -17818,7 +18271,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I14" s="111" t="str">
-        <x:v>Decision Locked</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="J14" s="111" t="str">
         <x:v>Critical</x:v>
@@ -17869,7 +18322,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I15" s="111" t="str">
-        <x:v>Decision Locked</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="J15" s="111" t="str">
         <x:v>High</x:v>
@@ -17973,7 +18426,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I17" s="111" t="str">
-        <x:v>Decision Locked</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="J17" s="111" t="str">
         <x:v>High</x:v>
@@ -18185,7 +18638,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I21" s="111" t="str">
-        <x:v>Decision Locked</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="J21" s="111" t="str">
         <x:v>Medium</x:v>
@@ -18289,7 +18742,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I23" s="111" t="str">
-        <x:v>Decision Locked</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="J23" s="111" t="str">
         <x:v>High</x:v>
@@ -19947,7 +20400,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I55" s="111" t="str">
-        <x:v>Decision Locked</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="J55" s="111" t="str">
         <x:v>High</x:v>
@@ -25300,31 +25753,31 @@
     </x:row>
     <x:row r="158" ht="46" customHeight="1">
       <x:c r="A158" s="111" t="str">
-        <x:v>P07-E2E-001</x:v>
+        <x:v>P04-S1</x:v>
       </x:c>
       <x:c r="B158" s="111" t="str">
-        <x:v>P07</x:v>
+        <x:v>P04</x:v>
       </x:c>
       <x:c r="C158" s="111" t="str">
-        <x:v>Core end-to-end vertical slice</x:v>
+        <x:v>Legal, trust, and creator onboarding</x:v>
       </x:c>
       <x:c r="D158" s="111" t="str">
-        <x:v>P04, P05, P06</x:v>
+        <x:v>P03</x:v>
       </x:c>
       <x:c r="E158" s="111" t="str">
-        <x:v>PLAN phase gate</x:v>
+        <x:v>Published slice</x:v>
       </x:c>
       <x:c r="F158" s="111" t="str">
-        <x:v>Core vertical slice</x:v>
+        <x:v>Creator onboarding &amp; trust</x:v>
       </x:c>
       <x:c r="G158" s="111" t="str">
-        <x:v>Complete the member-to-creator end-to-end product flow</x:v>
+        <x:v>Publish the creator-application submission foundation</x:v>
       </x:c>
       <x:c r="H158" s="111" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I158" s="111" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Integrated</x:v>
       </x:c>
       <x:c r="J158" s="111" t="str">
         <x:v>High</x:v>
@@ -25332,85 +25785,195 @@
       <x:c r="K158" s="111" t="str">
         <x:v>Engineering</x:v>
       </x:c>
-      <x:c r="L158" s="111" t="str">
-        <x:v>Phase 4–6 dependencies</x:v>
-      </x:c>
+      <x:c r="L158" s="111" t="str"/>
       <x:c r="M158" s="111" t="str">
-        <x:v>Do not begin the product slice until creator approval, media entitlement, and payment-ledger prerequisites are accepted.</x:v>
+        <x:v>Preserve the PENDING-only, no-role-promotion boundary until later trust and legal gates are approved.</x:v>
       </x:c>
       <x:c r="N158" s="112"/>
       <x:c r="O158" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/PLAN.md#11-phase-7--core-end-to-end-vertical-slice</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/commit/ce6c9e4</x:v>
       </x:c>
       <x:c r="P158" s="112" t="n">
         <x:v>46255.666666666664</x:v>
       </x:c>
       <x:c r="Q158" s="111" t="str">
-        <x:v>Member discovers an approved creator, acquires Veso, purchases access, consumes authorized media, and produces auditable records without manual database edits.</x:v>
+        <x:v>Verified members can submit one persisted creator application with versioned prototype acceptances recorded atomically.</x:v>
       </x:c>
       <x:c r="R158" s="111" t="str">
-        <x:v>Explicit dependency marker so Phase 7 is visible even though no legacy tracker row represented it.</x:v>
+        <x:v>Published Phase 4 Slice 1; no identity files, approval, creator role promotion, or Dashboard access.</x:v>
       </x:c>
       <x:c r="S158" s="111" t="str">
-        <x:v>PLAN.md Phase 7 exit gate</x:v>
+        <x:v>PLAN.md Phase 4 published foundation</x:v>
       </x:c>
     </x:row>
     <x:row r="159" ht="46" customHeight="1">
       <x:c r="A159" s="111" t="str">
-        <x:v>P14-QA-001</x:v>
+        <x:v>P04-S2</x:v>
       </x:c>
       <x:c r="B159" s="111" t="str">
-        <x:v>P14</x:v>
+        <x:v>P04</x:v>
       </x:c>
       <x:c r="C159" s="111" t="str">
-        <x:v>QA, security, private beta, and launch</x:v>
+        <x:v>Legal, trust, and creator onboarding</x:v>
       </x:c>
       <x:c r="D159" s="111" t="str">
-        <x:v>P08</x:v>
+        <x:v>P11</x:v>
       </x:c>
       <x:c r="E159" s="111" t="str">
-        <x:v>Supplemental</x:v>
+        <x:v>Published slice</x:v>
       </x:c>
       <x:c r="F159" s="111" t="str">
-        <x:v>Deterministic E2E</x:v>
+        <x:v>Private operations &amp; moderation</x:v>
       </x:c>
       <x:c r="G159" s="111" t="str">
-        <x:v>Make promotion material E2E independent of calendar date</x:v>
+        <x:v>Publish the dormant non-approval review-transition foundation</x:v>
       </x:c>
       <x:c r="H159" s="111" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I159" s="111" t="str">
-        <x:v>Integrated</x:v>
+        <x:v>Backend Implemented</x:v>
       </x:c>
       <x:c r="J159" s="111" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="K159" s="111" t="str">
         <x:v>Engineering</x:v>
       </x:c>
-      <x:c r="L159" s="111" t="str">
-        <x:v>Fresh CI</x:v>
-      </x:c>
+      <x:c r="L159" s="111" t="str"/>
       <x:c r="M159" s="111" t="str">
-        <x:v>Keep the Playwright test clock fixed before navigation so active-promotion fixtures do not expire with wall time.</x:v>
-      </x:c>
-      <x:c r="N159" s="112" t="n">
-        <x:v>46259.666666666664</x:v>
-      </x:c>
+        <x:v>Keep the router unmounted and APPROVED/role-promotion behavior absent until the documented activation gates are satisfied.</x:v>
+      </x:c>
+      <x:c r="N159" s="112"/>
       <x:c r="O159" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/1</x:v>
       </x:c>
       <x:c r="P159" s="112" t="n">
         <x:v>46255.666666666664</x:v>
       </x:c>
       <x:c r="Q159" s="111" t="str">
+        <x:v>Persist strict non-approval review transitions and immutable reviewer evidence in one transaction.</x:v>
+      </x:c>
+      <x:c r="R159" s="111" t="str">
+        <x:v>Published Phase 4 Slice 2 foundation; deliberately not an operational admin workflow.</x:v>
+      </x:c>
+      <x:c r="S159" s="111" t="str">
+        <x:v>PLAN.md Phase 4 published foundation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="46" customHeight="1">
+      <x:c r="A160" s="111" t="str">
+        <x:v>P07-E2E-001</x:v>
+      </x:c>
+      <x:c r="B160" s="111" t="str">
+        <x:v>P07</x:v>
+      </x:c>
+      <x:c r="C160" s="111" t="str">
+        <x:v>Core end-to-end vertical slice</x:v>
+      </x:c>
+      <x:c r="D160" s="111" t="str">
+        <x:v>P04, P05, P06</x:v>
+      </x:c>
+      <x:c r="E160" s="111" t="str">
+        <x:v>PLAN phase gate</x:v>
+      </x:c>
+      <x:c r="F160" s="111" t="str">
+        <x:v>Core vertical slice</x:v>
+      </x:c>
+      <x:c r="G160" s="111" t="str">
+        <x:v>Complete the member-to-creator end-to-end product flow</x:v>
+      </x:c>
+      <x:c r="H160" s="111" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="I160" s="111" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="J160" s="111" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K160" s="111" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="L160" s="111" t="str">
+        <x:v>Phase 4–6 dependencies</x:v>
+      </x:c>
+      <x:c r="M160" s="111" t="str">
+        <x:v>Do not begin the product slice until creator approval, media entitlement, and payment-ledger prerequisites are accepted.</x:v>
+      </x:c>
+      <x:c r="N160" s="112"/>
+      <x:c r="O160" s="111" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/PLAN.md#11-phase-7--core-end-to-end-vertical-slice</x:v>
+      </x:c>
+      <x:c r="P160" s="112" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+      <x:c r="Q160" s="111" t="str">
+        <x:v>Member discovers an approved creator, acquires Veso, purchases access, consumes authorized media, and produces auditable records without manual database edits.</x:v>
+      </x:c>
+      <x:c r="R160" s="111" t="str">
+        <x:v>Explicit dependency marker so Phase 7 is visible even though no legacy tracker row represented it.</x:v>
+      </x:c>
+      <x:c r="S160" s="111" t="str">
+        <x:v>PLAN.md Phase 7 exit gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161" ht="46" customHeight="1">
+      <x:c r="A161" s="111" t="str">
+        <x:v>P14-QA-001</x:v>
+      </x:c>
+      <x:c r="B161" s="111" t="str">
+        <x:v>P14</x:v>
+      </x:c>
+      <x:c r="C161" s="111" t="str">
+        <x:v>QA, security, private beta, and launch</x:v>
+      </x:c>
+      <x:c r="D161" s="111" t="str">
+        <x:v>P08</x:v>
+      </x:c>
+      <x:c r="E161" s="111" t="str">
+        <x:v>Supplemental</x:v>
+      </x:c>
+      <x:c r="F161" s="111" t="str">
+        <x:v>Deterministic E2E</x:v>
+      </x:c>
+      <x:c r="G161" s="111" t="str">
+        <x:v>Make promotion material E2E independent of calendar date</x:v>
+      </x:c>
+      <x:c r="H161" s="111" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="I161" s="111" t="str">
+        <x:v>Integrated</x:v>
+      </x:c>
+      <x:c r="J161" s="111" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K161" s="111" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="L161" s="111" t="str">
+        <x:v>Fresh CI</x:v>
+      </x:c>
+      <x:c r="M161" s="111" t="str">
+        <x:v>Keep the Playwright test clock fixed before navigation so active-promotion fixtures do not expire with wall time.</x:v>
+      </x:c>
+      <x:c r="N161" s="112" t="n">
+        <x:v>46259.666666666664</x:v>
+      </x:c>
+      <x:c r="O161" s="111" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
+      </x:c>
+      <x:c r="P161" s="112" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+      <x:c r="Q161" s="111" t="str">
         <x:v>Freeze the test clock without changing product or fixture behavior.</x:v>
       </x:c>
-      <x:c r="R159" s="111" t="str">
+      <x:c r="R161" s="111" t="str">
         <x:v>Initial PR #13 E2E failure was a date rollover; replacement exact-head CI passed before this tracker update.</x:v>
       </x:c>
-      <x:c r="S159" s="111" t="str">
+      <x:c r="S161" s="111" t="str">
         <x:v>PR #13 CI repair</x:v>
       </x:c>
     </x:row>
@@ -25419,35 +25982,35 @@
     <x:mergeCell ref="A1:S1"/>
     <x:mergeCell ref="A2:S2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="H4:H159">
+  <x:conditionalFormatting sqref="H4:H161">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Done"/>
-    <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="In Progress"/>
-    <x:cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="In Review"/>
-    <x:cfRule type="containsText" dxfId="9" priority="4" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="12" priority="5" operator="containsText" text="Not Started"/>
-    <x:cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="Ready"/>
-    <x:cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="Deferred"/>
+    <x:cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="In Review"/>
+    <x:cfRule type="containsText" dxfId="12" priority="4" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="Not Started"/>
+    <x:cfRule type="containsText" dxfId="20" priority="6" operator="containsText" text="Ready"/>
+    <x:cfRule type="containsText" dxfId="24" priority="7" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="5">
-    <x:dataValidation type="list" sqref="H4:H159">
+    <x:dataValidation type="list" sqref="H4:H161">
       <x:formula1>"Not Started,Ready,In Progress,In Review,Blocked,Done,Deferred"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I4:I159">
+    <x:dataValidation type="list" sqref="I4:I161">
       <x:formula1>"Decision Locked,UI Prototype,Backend Implemented,Integrated,Production-Ready,N/A"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J4:J159">
+    <x:dataValidation type="list" sqref="J4:J161">
       <x:formula1>"Critical,High,Medium,Low"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K4:K159">
+    <x:dataValidation type="list" sqref="K4:K161">
       <x:formula1>"Founder,Engineering,Operations,Counsel,Unassigned"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="E4:E159">
-      <x:formula1>"PLAN task,Supplemental,Legacy-mapped task,Decision,Exit criterion"</x:formula1>
+    <x:dataValidation type="list" sqref="E4:E161">
+      <x:formula1>"PLAN task,PLAN phase gate,Supplemental,Legacy-mapped task,Published slice,Decision,Exit criterion"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1772abacfac542ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbdf806c34dff43b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: reconcile Phase 2 worker publication
</commit_message>
<xml_diff>
--- a/docs/product/Pumdoki_MasterTracker_V4.xlsx
+++ b/docs/product/Pumdoki_MasterTracker_V4.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc85fc3fbe2e74df0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R28f114d80f1348fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R7a2e21f361534518"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="Re271bb41e4214da8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R0e7115ce53bf44d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legacy Overview 2026-08-16" sheetId="6" r:id="R999a5dfe37e24557"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="7" r:id="Rd3e1530812054b35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Roadmap" sheetId="8" r:id="R61e5aa682ecb4019"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Tracker" sheetId="9" r:id="Re238eabfe7084ebe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Blocker Queue" sheetId="10" r:id="Re9c8b707730a45d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Log" sheetId="11" r:id="Refb2f3deb3b540d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Register" sheetId="12" r:id="R64af974bd2184856"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R12e2c5b5ac1b4d7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R30bf9d4c2b7040a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R6f93f56df0fd4ff1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="Re521642b14464a8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R8365b901f1604472"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legacy Overview 2026-08-16" sheetId="6" r:id="Rc70cd342071647eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="7" r:id="R80e8838af68d49d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Roadmap" sheetId="8" r:id="Rd7f006c4824a4aec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Tracker" sheetId="9" r:id="Rd8a4c6d6313d4495"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Blocker Queue" sheetId="10" r:id="R782ce6d6a0d54a1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Log" sheetId="11" r:id="R7aa2384c19104e32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Register" sheetId="12" r:id="R53c371dadb354279"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2934,8 +2934,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ReviewQueueTable" displayName="ReviewQueueTable" ref="A3:L9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:L9"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ReviewQueueTable" displayName="ReviewQueueTable" ref="A3:L4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:L4"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Work ID"/>
     <x:tableColumn id="2" name="Phase"/>
@@ -3268,12 +3268,12 @@
         <x:v>Phase</x:v>
       </x:c>
       <x:c r="B5" s="109" t="str">
-        <x:v>P02 — Backend and database foundation</x:v>
+        <x:v>P04 — Legal, trust, and creator onboarding</x:v>
       </x:c>
       <x:c r="D5"/>
       <x:c r="E5"/>
       <x:c r="I5" s="130" t="str">
-        <x:v>Review the updated PR #13 workbook and fresh exact-head CI. A later merge decision remains separate. The next Phase 4 decision is whether to authorize a private-operations identity/access design—not creator approval activation.</x:v>
+        <x:v>Decide whether to authorize an isolated private-operations identity/access design and local verification slice. This is not approval to mount the review router, approve creators, promote roles, deploy, or configure live identity infrastructure.</x:v>
       </x:c>
       <x:c r="J5" s="130"/>
       <x:c r="K5" s="130"/>
@@ -3286,7 +3286,7 @@
         <x:v>Work</x:v>
       </x:c>
       <x:c r="B6" s="111" t="str">
-        <x:v>Draft PR #13 durable PostgreSQL worker foundation</x:v>
+        <x:v>Private-operations identity/access design decision</x:v>
       </x:c>
       <x:c r="D6"/>
       <x:c r="E6"/>
@@ -3302,7 +3302,7 @@
         <x:v>Workflow</x:v>
       </x:c>
       <x:c r="B7" s="111" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="I7" s="131"/>
       <x:c r="J7" s="131"/>
@@ -3316,7 +3316,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B8" s="111" t="str">
-        <x:v>Fixed non-secret canary only; no product flow or deployment</x:v>
+        <x:v>Design and local verification only; no router mount or APPROVED transition</x:v>
       </x:c>
       <x:c r="I8" s="131"/>
       <x:c r="J8" s="131"/>
@@ -3330,7 +3330,7 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B9" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/docs/operations/README.md</x:v>
       </x:c>
       <x:c r="I9" s="131" t="str">
         <x:v>Phase 4 remains partial: creator application and dormant non-approval foundations are published; operational identity, legal, provider, approval, and publishing gates remain open.</x:v>
@@ -3398,7 +3398,7 @@
       <x:c r="B13" s="151"/>
       <x:c r="C13" s="150" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$H$4:$H$400,"Done")</x:f>
-        <x:v>22</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D13" s="151"/>
       <x:c r="E13" s="150" t="n">
@@ -3408,7 +3408,7 @@
       <x:c r="F13" s="151"/>
       <x:c r="G13" s="150" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$H$4:$H$400,"In Review")</x:f>
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H13" s="151"/>
       <x:c r="I13" s="150" t="n">
@@ -3423,7 +3423,7 @@
       <x:c r="L13" s="151"/>
       <x:c r="M13" s="158" t="n">
         <x:f>IF(A13=0,0,C13/A13)</x:f>
-        <x:v>0.13924050632911392</x:v>
+        <x:v>0.17088607594936708</x:v>
       </x:c>
       <x:c r="N13" s="151"/>
     </x:row>
@@ -3528,7 +3528,7 @@
       </x:c>
       <x:c r="E18" s="109" t="n">
         <x:f>'Phase Roadmap'!E4</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F18" s="109" t="n">
         <x:f>'Phase Roadmap'!F4</x:f>
@@ -3536,7 +3536,7 @@
       </x:c>
       <x:c r="G18" s="118" t="n">
         <x:f>'Phase Roadmap'!G4</x:f>
-        <x:v>0.6666666666666666</x:v>
+        <x:v>0.8333333333333334</x:v>
       </x:c>
       <x:c r="H18" s="109" t="n">
         <x:f>'Phase Roadmap'!H4</x:f>
@@ -3544,7 +3544,7 @@
       </x:c>
       <x:c r="I18" s="109" t="n">
         <x:f>'Phase Roadmap'!I4</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J18" s="109" t="n">
         <x:f>'Phase Roadmap'!J4</x:f>
@@ -3556,15 +3556,15 @@
       </x:c>
       <x:c r="L18" s="109" t="str">
         <x:f>'Phase Roadmap'!L4</x:f>
-        <x:v>Align the execution tracker with PLAN.md and keep decisions/evidence current.</x:v>
+        <x:v>Maintain the PLAN-aligned execution tracker, decision register, review queue, and daily debrief history.</x:v>
       </x:c>
       <x:c r="M18" s="109" t="str">
         <x:f>'Phase Roadmap'!M4</x:f>
-        <x:v>Publish the tracker reconciliation in PR #13, then keep owners and dates current.</x:v>
+        <x:v>Assign and maintain owners and next-check dates for remaining active decisions; preserve legacy records.</x:v>
       </x:c>
       <x:c r="N18" s="109" t="str">
         <x:f>'Phase Roadmap'!O4</x:f>
-        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/PLAN.md</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="48" hidden="0" customHeight="1">
@@ -3644,7 +3644,7 @@
       </x:c>
       <x:c r="E20" s="111" t="n">
         <x:f>'Phase Roadmap'!E6</x:f>
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F20" s="111" t="n">
         <x:f>'Phase Roadmap'!F6</x:f>
@@ -3652,7 +3652,7 @@
       </x:c>
       <x:c r="G20" s="119" t="n">
         <x:f>'Phase Roadmap'!G6</x:f>
-        <x:v>0.0625</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="H20" s="111" t="n">
         <x:f>'Phase Roadmap'!H6</x:f>
@@ -3660,7 +3660,7 @@
       </x:c>
       <x:c r="I20" s="111" t="n">
         <x:f>'Phase Roadmap'!I6</x:f>
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J20" s="111" t="n">
         <x:f>'Phase Roadmap'!J6</x:f>
@@ -3672,11 +3672,11 @@
       </x:c>
       <x:c r="L20" s="111" t="str">
         <x:f>'Phase Roadmap'!L6</x:f>
-        <x:v>Review draft PR #13: application-owned PostgreSQL worker foundation and fixed canary only.</x:v>
+        <x:v>PR #13 published the application-owned PostgreSQL worker foundation and fixed non-secret canary; no product flow uses it.</x:v>
       </x:c>
       <x:c r="M20" s="111" t="str">
         <x:f>'Phase Roadmap'!M6</x:f>
-        <x:v>Fresh exact-head CI and founder review; merge remains separately gated.</x:v>
+        <x:v>Keep Phase 2 partial: staging, restore/backups, monitoring, Redis/shared throttling, general idempotency, and deployment remain open.</x:v>
       </x:c>
       <x:c r="N20" s="111" t="str">
         <x:f>'Phase Roadmap'!O6</x:f>
@@ -4340,7 +4340,7 @@
       </x:c>
       <x:c r="E32" s="111" t="n">
         <x:f>'Phase Roadmap'!E18</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F32" s="111" t="n">
         <x:f>'Phase Roadmap'!F18</x:f>
@@ -4348,7 +4348,7 @@
       </x:c>
       <x:c r="G32" s="119" t="n">
         <x:f>'Phase Roadmap'!G18</x:f>
-        <x:v>0</x:v>
+        <x:v>0.045454545454545456</x:v>
       </x:c>
       <x:c r="H32" s="111" t="n">
         <x:f>'Phase Roadmap'!H18</x:f>
@@ -4356,7 +4356,7 @@
       </x:c>
       <x:c r="I32" s="111" t="n">
         <x:f>'Phase Roadmap'!I18</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J32" s="111" t="n">
         <x:f>'Phase Roadmap'!J18</x:f>
@@ -4368,7 +4368,7 @@
       </x:c>
       <x:c r="L32" s="111" t="str">
         <x:f>'Phase Roadmap'!L18</x:f>
-        <x:v>CI/E2E foundations exist; product E2E, security drills, beta, and launch gates remain open.</x:v>
+        <x:v>CI/E2E foundations and the deterministic promotion clock fix are published; product E2E, security drills, beta, and launch gates remain open.</x:v>
       </x:c>
       <x:c r="M32" s="111" t="str">
         <x:f>'Phase Roadmap'!M18</x:f>
@@ -4376,7 +4376,7 @@
       </x:c>
       <x:c r="N32" s="111" t="str">
         <x:f>'Phase Roadmap'!O18</x:f>
-        <x:v>https://github.com/QK-Connoisseur/PDoki/actions</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/actions/runs/32535922437</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15.75" customHeight="1"/>
@@ -4451,7 +4451,7 @@
         <x:v>Phase 2</x:v>
       </x:c>
       <x:c r="F36" s="111" t="str">
-        <x:v>PR #13 is in review and Phase 2 remains partial.</x:v>
+        <x:v>PR #13 is merged and CI-verified; the fixed canary foundation is Done while Phase 2 remains partial.</x:v>
       </x:c>
       <x:c r="G36" s="111" t="str">
         <x:v>Phase 4</x:v>
@@ -4516,22 +4516,22 @@
         <x:v>Record progress counts preserved/current records; Phase State is the canonical PLAN judgment.</x:v>
       </x:c>
       <x:c r="E38" s="111" t="str">
-        <x:v>Current branch</x:v>
+        <x:v>Published base</x:v>
       </x:c>
       <x:c r="F38" s="111" t="str">
-        <x:v>codex/phase2-worker-foundation</x:v>
+        <x:v>dev @ 6311522</x:v>
       </x:c>
       <x:c r="G38" s="111" t="str">
-        <x:v>Open PR</x:v>
+        <x:v>PR #13</x:v>
       </x:c>
       <x:c r="H38" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="I38" s="111" t="str">
-        <x:v>Merge</x:v>
+        <x:v>Post-merge CI</x:v>
       </x:c>
       <x:c r="J38" s="111" t="str">
-        <x:v>Separately gated</x:v>
+        <x:v>32535922437 — green</x:v>
       </x:c>
       <x:c r="K38" s="111" t="str"/>
       <x:c r="L38" s="111" t="str"/>
@@ -5620,229 +5620,109 @@
     </x:row>
     <x:row r="4" ht="54" customHeight="1">
       <x:c r="A4" s="109" t="str">
-        <x:v>P00-T03</x:v>
+        <x:v>P07-E2E-001</x:v>
       </x:c>
       <x:c r="B4" s="109" t="str">
-        <x:v>P00</x:v>
+        <x:v>P07</x:v>
       </x:c>
       <x:c r="C4" s="109" t="str">
-        <x:v>Baseline, tracker, and scope control</x:v>
+        <x:v>Core end-to-end vertical slice</x:v>
       </x:c>
       <x:c r="D4" s="109" t="str">
-        <x:v>Tracker &amp; scope control</x:v>
+        <x:v>Core vertical slice</x:v>
       </x:c>
       <x:c r="E4" s="109" t="str">
-        <x:v>Reclassify the tracker to PLAN.md Phases 0–14</x:v>
+        <x:v>Complete the member-to-creator end-to-end product flow</x:v>
       </x:c>
       <x:c r="F4" s="109" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G4" s="109" t="str">
         <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H4" s="109" t="str">
-        <x:v>Founder review</x:v>
+        <x:v>Phase 4–6 dependencies</x:v>
       </x:c>
       <x:c r="I4" s="109" t="str">
-        <x:v>Review the reorganized workbook in draft PR #13; preserve the legacy tracker as the source snapshot.</x:v>
-      </x:c>
-      <x:c r="J4" s="110" t="n">
-        <x:v>46255.666666666664</x:v>
-      </x:c>
+        <x:v>Do not begin the product slice until creator approval, media entitlement, and payment-ledger prerequisites are accepted.</x:v>
+      </x:c>
+      <x:c r="J4" s="110"/>
       <x:c r="K4" s="109" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/PLAN.md#11-phase-7--core-end-to-end-vertical-slice</x:v>
       </x:c>
       <x:c r="L4" s="110" t="n">
         <x:v>46255.666666666664</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="54" customHeight="1">
-      <x:c r="A5" s="111" t="str">
-        <x:v>P02-T11</x:v>
-      </x:c>
-      <x:c r="B5" s="111" t="str">
-        <x:v>P02</x:v>
-      </x:c>
-      <x:c r="C5" s="111" t="str">
-        <x:v>Backend and database foundation</x:v>
-      </x:c>
-      <x:c r="D5" s="111" t="str">
-        <x:v>Durable async work</x:v>
-      </x:c>
-      <x:c r="E5" s="111" t="str">
-        <x:v>Add a background-job queue</x:v>
-      </x:c>
-      <x:c r="F5" s="111" t="str">
-        <x:v>In Review</x:v>
-      </x:c>
-      <x:c r="G5" s="111" t="str">
-        <x:v>Engineering</x:v>
-      </x:c>
-      <x:c r="H5" s="111" t="str">
-        <x:v>Founder review + fresh CI</x:v>
-      </x:c>
-      <x:c r="I5" s="111" t="str">
-        <x:v>Review the application-owned PostgreSQL worker foundation on PR #13; merge remains separately gated.</x:v>
-      </x:c>
-      <x:c r="J5" s="112" t="n">
-        <x:v>46259.666666666664</x:v>
-      </x:c>
-      <x:c r="K5" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
-      </x:c>
-      <x:c r="L5" s="112" t="n">
-        <x:v>46255.666666666664</x:v>
-      </x:c>
+      <x:c r="A5" s="111"/>
+      <x:c r="B5" s="111"/>
+      <x:c r="C5" s="111"/>
+      <x:c r="D5" s="111"/>
+      <x:c r="E5" s="111"/>
+      <x:c r="F5" s="111"/>
+      <x:c r="G5" s="111"/>
+      <x:c r="H5" s="111"/>
+      <x:c r="I5" s="111"/>
+      <x:c r="J5" s="112"/>
+      <x:c r="K5" s="111"/>
+      <x:c r="L5" s="112"/>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
-      <x:c r="A6" s="111" t="str">
-        <x:v>P02-T12A</x:v>
-      </x:c>
-      <x:c r="B6" s="111" t="str">
-        <x:v>P02</x:v>
-      </x:c>
-      <x:c r="C6" s="111" t="str">
-        <x:v>Backend and database foundation</x:v>
-      </x:c>
-      <x:c r="D6" s="111" t="str">
-        <x:v>Durable async work</x:v>
-      </x:c>
-      <x:c r="E6" s="111" t="str">
-        <x:v>Prove canary-specific idempotency and lease fencing</x:v>
-      </x:c>
-      <x:c r="F6" s="111" t="str">
-        <x:v>In Review</x:v>
-      </x:c>
-      <x:c r="G6" s="111" t="str">
-        <x:v>Engineering</x:v>
-      </x:c>
-      <x:c r="H6" s="111" t="str">
-        <x:v>Founder review + fresh CI</x:v>
-      </x:c>
-      <x:c r="I6" s="111" t="str">
-        <x:v>Review atomic enqueue/replay, stale-token rejection, effect reconciliation, and exact-role evidence in PR #13.</x:v>
-      </x:c>
-      <x:c r="J6" s="112" t="n">
-        <x:v>46259.666666666664</x:v>
-      </x:c>
-      <x:c r="K6" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
-      </x:c>
-      <x:c r="L6" s="112" t="n">
-        <x:v>46255.666666666664</x:v>
-      </x:c>
+      <x:c r="A6" s="111"/>
+      <x:c r="B6" s="111"/>
+      <x:c r="C6" s="111"/>
+      <x:c r="D6" s="111"/>
+      <x:c r="E6" s="111"/>
+      <x:c r="F6" s="111"/>
+      <x:c r="G6" s="111"/>
+      <x:c r="H6" s="111"/>
+      <x:c r="I6" s="111"/>
+      <x:c r="J6" s="112"/>
+      <x:c r="K6" s="111"/>
+      <x:c r="L6" s="112"/>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
-      <x:c r="A7" s="111" t="str">
-        <x:v>P02-NET-001</x:v>
-      </x:c>
-      <x:c r="B7" s="111" t="str">
-        <x:v>P02</x:v>
-      </x:c>
-      <x:c r="C7" s="111" t="str">
-        <x:v>Backend and database foundation</x:v>
-      </x:c>
-      <x:c r="D7" s="111" t="str">
-        <x:v>Local security</x:v>
-      </x:c>
-      <x:c r="E7" s="111" t="str">
-        <x:v>Bind local PostgreSQL host exposure to IPv4 loopback</x:v>
-      </x:c>
-      <x:c r="F7" s="111" t="str">
-        <x:v>In Review</x:v>
-      </x:c>
-      <x:c r="G7" s="111" t="str">
-        <x:v>Engineering</x:v>
-      </x:c>
-      <x:c r="H7" s="111" t="str">
-        <x:v>Founder review + fresh CI</x:v>
-      </x:c>
-      <x:c r="I7" s="111" t="str">
-        <x:v>Verify the tracked Compose mapping remains 127.0.0.1-only and the named volume is preserved.</x:v>
-      </x:c>
-      <x:c r="J7" s="112" t="n">
-        <x:v>46259.666666666664</x:v>
-      </x:c>
-      <x:c r="K7" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
-      </x:c>
-      <x:c r="L7" s="112" t="n">
-        <x:v>46255.666666666664</x:v>
-      </x:c>
+      <x:c r="A7" s="111"/>
+      <x:c r="B7" s="111"/>
+      <x:c r="C7" s="111"/>
+      <x:c r="D7" s="111"/>
+      <x:c r="E7" s="111"/>
+      <x:c r="F7" s="111"/>
+      <x:c r="G7" s="111"/>
+      <x:c r="H7" s="111"/>
+      <x:c r="I7" s="111"/>
+      <x:c r="J7" s="112"/>
+      <x:c r="K7" s="111"/>
+      <x:c r="L7" s="112"/>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
-      <x:c r="A8" s="111" t="str">
-        <x:v>P07-E2E-001</x:v>
-      </x:c>
-      <x:c r="B8" s="111" t="str">
-        <x:v>P07</x:v>
-      </x:c>
-      <x:c r="C8" s="111" t="str">
-        <x:v>Core end-to-end vertical slice</x:v>
-      </x:c>
-      <x:c r="D8" s="111" t="str">
-        <x:v>Core vertical slice</x:v>
-      </x:c>
-      <x:c r="E8" s="111" t="str">
-        <x:v>Complete the member-to-creator end-to-end product flow</x:v>
-      </x:c>
-      <x:c r="F8" s="111" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="G8" s="111" t="str">
-        <x:v>Engineering</x:v>
-      </x:c>
-      <x:c r="H8" s="111" t="str">
-        <x:v>Phase 4–6 dependencies</x:v>
-      </x:c>
-      <x:c r="I8" s="111" t="str">
-        <x:v>Do not begin the product slice until creator approval, media entitlement, and payment-ledger prerequisites are accepted.</x:v>
-      </x:c>
+      <x:c r="A8" s="111"/>
+      <x:c r="B8" s="111"/>
+      <x:c r="C8" s="111"/>
+      <x:c r="D8" s="111"/>
+      <x:c r="E8" s="111"/>
+      <x:c r="F8" s="111"/>
+      <x:c r="G8" s="111"/>
+      <x:c r="H8" s="111"/>
+      <x:c r="I8" s="111"/>
       <x:c r="J8" s="112"/>
-      <x:c r="K8" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/PLAN.md#11-phase-7--core-end-to-end-vertical-slice</x:v>
-      </x:c>
-      <x:c r="L8" s="112" t="n">
-        <x:v>46255.666666666664</x:v>
-      </x:c>
+      <x:c r="K8" s="111"/>
+      <x:c r="L8" s="112"/>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
-      <x:c r="A9" s="111" t="str">
-        <x:v>P14-QA-001</x:v>
-      </x:c>
-      <x:c r="B9" s="111" t="str">
-        <x:v>P14</x:v>
-      </x:c>
-      <x:c r="C9" s="111" t="str">
-        <x:v>QA, security, private beta, and launch</x:v>
-      </x:c>
-      <x:c r="D9" s="111" t="str">
-        <x:v>Deterministic E2E</x:v>
-      </x:c>
-      <x:c r="E9" s="111" t="str">
-        <x:v>Make promotion material E2E independent of calendar date</x:v>
-      </x:c>
-      <x:c r="F9" s="111" t="str">
-        <x:v>In Review</x:v>
-      </x:c>
-      <x:c r="G9" s="111" t="str">
-        <x:v>Engineering</x:v>
-      </x:c>
-      <x:c r="H9" s="111" t="str">
-        <x:v>Fresh CI</x:v>
-      </x:c>
-      <x:c r="I9" s="111" t="str">
-        <x:v>Keep the Playwright test clock fixed before navigation so active-promotion fixtures do not expire with wall time.</x:v>
-      </x:c>
-      <x:c r="J9" s="112" t="n">
-        <x:v>46259.666666666664</x:v>
-      </x:c>
-      <x:c r="K9" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
-      </x:c>
-      <x:c r="L9" s="112" t="n">
-        <x:v>46255.666666666664</x:v>
-      </x:c>
+      <x:c r="A9" s="111"/>
+      <x:c r="B9" s="111"/>
+      <x:c r="C9" s="111"/>
+      <x:c r="D9" s="111"/>
+      <x:c r="E9" s="111"/>
+      <x:c r="F9" s="111"/>
+      <x:c r="G9" s="111"/>
+      <x:c r="H9" s="111"/>
+      <x:c r="I9" s="111"/>
+      <x:c r="J9" s="112"/>
+      <x:c r="K9" s="111"/>
+      <x:c r="L9" s="112"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5860,7 +5740,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31b72b6e3a224058"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda1cc3b4d7234481"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6068,18 +5948,42 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
-      <x:c r="A7" s="111"/>
-      <x:c r="B7" s="111"/>
-      <x:c r="C7" s="111"/>
-      <x:c r="D7" s="111"/>
-      <x:c r="E7" s="111"/>
-      <x:c r="F7" s="111"/>
-      <x:c r="G7" s="111"/>
-      <x:c r="H7" s="111"/>
-      <x:c r="I7" s="111"/>
-      <x:c r="J7" s="111"/>
-      <x:c r="K7" s="111"/>
-      <x:c r="L7" s="111"/>
+      <x:c r="A7" s="112" t="n">
+        <x:v>46255.666666666664</x:v>
+      </x:c>
+      <x:c r="B7" s="111" t="str">
+        <x:v>P02-T11</x:v>
+      </x:c>
+      <x:c r="C7" s="111" t="str">
+        <x:v>P02</x:v>
+      </x:c>
+      <x:c r="D7" s="111" t="str">
+        <x:v>Publish and reconcile the Phase 2 worker foundation.</x:v>
+      </x:c>
+      <x:c r="E7" s="111" t="str">
+        <x:v>PR #13 merged into dev as 6311522 from reviewed head 8a8688f; post-merge CI 32535922437 passed all three jobs, and the five scoped tracker records moved from In Review to Done.</x:v>
+      </x:c>
+      <x:c r="F7" s="111" t="str">
+        <x:v>The durable canary foundation and PLAN-aligned tracker are now published, and the operating views accurately separate completed evidence from the remaining Phase 2 and Phase 4 gates.</x:v>
+      </x:c>
+      <x:c r="G7" s="111" t="str">
+        <x:v>No product flow, provider, Redis store, deployment, live credential, creator approval, role promotion, or private-operations activation was added.</x:v>
+      </x:c>
+      <x:c r="H7" s="111" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13 · https://github.com/QK-Connoisseur/PDoki/actions/runs/32535922437</x:v>
+      </x:c>
+      <x:c r="I7" s="111" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="J7" s="111" t="str">
+        <x:v>Any new implementation and this reconciliation branch's publication remain separately gated.</x:v>
+      </x:c>
+      <x:c r="K7" s="111" t="str">
+        <x:v>Seek a separate decision on the Phase 4 private-operations identity/access design and local verification scope.</x:v>
+      </x:c>
+      <x:c r="L7" s="111" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" s="111"/>
@@ -6886,7 +6790,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18a5b4d9a8544742"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaff5266ed9647be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7080,13 +6984,13 @@
         <x:v>46259.666666666664</x:v>
       </x:c>
       <x:c r="F7" s="111" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G7" s="111" t="str">
-        <x:v>Draft PR #13 is open with the fixed canary foundation; merge and deployment remain gated.</x:v>
+        <x:v>PR #13 merged into dev as 6311522 from reviewed head 8a8688f; exact-head and post-merge CI passed all three jobs.</x:v>
       </x:c>
       <x:c r="H7" s="111" t="str">
-        <x:v>Review the tracker update and fresh exact-head CI, then decide whether to merge.</x:v>
+        <x:v>Preserve the fixed-canary and no-product-flow boundary; treat every further Phase 2 implementation or deployment step as separately gated.</x:v>
       </x:c>
       <x:c r="I7" s="111" t="str">
         <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
@@ -7453,7 +7357,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb048690bc2e412d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09a1f47b77a3457f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13037,7 +12941,7 @@
         <x:v>Current focus</x:v>
       </x:c>
       <x:c r="B104" s="111" t="str">
-        <x:v>Draft PR #13 is Phase 2 only and remains In Review. It adds a fixed canary worker foundation, not a product-flow migration or deployment.</x:v>
+        <x:v>PR #13 merged into dev as 6311522 and post-merge CI passed. Its fixed canary worker foundation is published, while Phase 2 remains partial and no product flow or deployment was added.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="42" customHeight="1">
@@ -13061,7 +12965,7 @@
         <x:v>Last refreshed</x:v>
       </x:c>
       <x:c r="B107" s="111" t="str">
-        <x:v>2026-08-21 by Codex during the authorized tracker rework for draft PR #13.</x:v>
+        <x:v>2026-08-21 by Codex during the authorized post-merge tracker and status reconciliation.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="15.75" customHeight="1"/>
@@ -16676,7 +16580,7 @@
       </x:c>
       <x:c r="E4" s="109" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A4,'Delivery Tracker'!$H$4:$H$400,"Done")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F4" s="109" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$B$4:$B$400,$A4)</x:f>
@@ -16684,7 +16588,7 @@
       </x:c>
       <x:c r="G4" s="118" t="n">
         <x:f>IF(F4=0,0,E4/F4)</x:f>
-        <x:v>0.6666666666666666</x:v>
+        <x:v>0.8333333333333334</x:v>
       </x:c>
       <x:c r="H4" s="109" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A4,'Delivery Tracker'!$H$4:$H$400,"In Progress")</x:f>
@@ -16692,7 +16596,7 @@
       </x:c>
       <x:c r="I4" s="109" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A4,'Delivery Tracker'!$H$4:$H$400,"In Review")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J4" s="109" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A4,'Delivery Tracker'!$H$4:$H$400,"Blocked")</x:f>
@@ -16703,16 +16607,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L4" s="109" t="str">
-        <x:v>Align the execution tracker with PLAN.md and keep decisions/evidence current.</x:v>
+        <x:v>Maintain the PLAN-aligned execution tracker, decision register, review queue, and daily debrief history.</x:v>
       </x:c>
       <x:c r="M4" s="109" t="str">
-        <x:v>Publish the tracker reconciliation in PR #13, then keep owners and dates current.</x:v>
+        <x:v>Assign and maintain owners and next-check dates for remaining active decisions; preserve legacy records.</x:v>
       </x:c>
       <x:c r="N4" s="109" t="str">
         <x:v>Clean baseline; tracker reflects reality; MVP approved; open decisions have an owner and date.</x:v>
       </x:c>
       <x:c r="O4" s="109" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/PLAN.md</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
       </x:c>
       <x:c r="P4" s="110" t="n">
         <x:v>46255.666666666664</x:v>
@@ -16790,7 +16694,7 @@
       </x:c>
       <x:c r="E6" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A6,'Delivery Tracker'!$H$4:$H$400,"Done")</x:f>
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F6" s="111" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$B$4:$B$400,$A6)</x:f>
@@ -16798,7 +16702,7 @@
       </x:c>
       <x:c r="G6" s="119" t="n">
         <x:f>IF(F6=0,0,E6/F6)</x:f>
-        <x:v>0.0625</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="H6" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A6,'Delivery Tracker'!$H$4:$H$400,"In Progress")</x:f>
@@ -16806,7 +16710,7 @@
       </x:c>
       <x:c r="I6" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A6,'Delivery Tracker'!$H$4:$H$400,"In Review")</x:f>
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J6" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A6,'Delivery Tracker'!$H$4:$H$400,"Blocked")</x:f>
@@ -16817,10 +16721,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="L6" s="111" t="str">
-        <x:v>Review draft PR #13: application-owned PostgreSQL worker foundation and fixed canary only.</x:v>
+        <x:v>PR #13 published the application-owned PostgreSQL worker foundation and fixed non-secret canary; no product flow uses it.</x:v>
       </x:c>
       <x:c r="M6" s="111" t="str">
-        <x:v>Fresh exact-head CI and founder review; merge remains separately gated.</x:v>
+        <x:v>Keep Phase 2 partial: staging, restore/backups, monitoring, Redis/shared throttling, general idempotency, and deployment remain open.</x:v>
       </x:c>
       <x:c r="N6" s="111" t="str">
         <x:v>HTTPS staging; repeatable migrations; backup restoration; monitoring; durable worker foundation reviewed.</x:v>
@@ -17474,7 +17378,7 @@
       </x:c>
       <x:c r="E18" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A18,'Delivery Tracker'!$H$4:$H$400,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F18" s="111" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$B$4:$B$400,$A18)</x:f>
@@ -17482,7 +17386,7 @@
       </x:c>
       <x:c r="G18" s="119" t="n">
         <x:f>IF(F18=0,0,E18/F18)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.045454545454545456</x:v>
       </x:c>
       <x:c r="H18" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A18,'Delivery Tracker'!$H$4:$H$400,"In Progress")</x:f>
@@ -17490,7 +17394,7 @@
       </x:c>
       <x:c r="I18" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A18,'Delivery Tracker'!$H$4:$H$400,"In Review")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J18" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A18,'Delivery Tracker'!$H$4:$H$400,"Blocked")</x:f>
@@ -17501,7 +17405,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="L18" s="111" t="str">
-        <x:v>CI/E2E foundations exist; product E2E, security drills, beta, and launch gates remain open.</x:v>
+        <x:v>CI/E2E foundations and the deterministic promotion clock fix are published; product E2E, security drills, beta, and launch gates remain open.</x:v>
       </x:c>
       <x:c r="M18" s="111" t="str">
         <x:v>Keep expanding domain tests; do not schedule beta until legal, payments, identity, recovery, and support gates exist.</x:v>
@@ -17510,7 +17414,7 @@
         <x:v>Restore/security/processor/content/support drills pass; launch gates are satisfied; no critical findings.</x:v>
       </x:c>
       <x:c r="O18" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/actions</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/actions/runs/32535922437</x:v>
       </x:c>
       <x:c r="P18" s="112" t="n">
         <x:v>46255.666666666664</x:v>
@@ -17596,7 +17500,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R376c4f1564a14df6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30351a00dab44d8d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25430,7 +25334,7 @@
         <x:v>Reclassify the tracker to PLAN.md Phases 0–14</x:v>
       </x:c>
       <x:c r="H152" s="111" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I152" s="111" t="str">
         <x:v>N/A</x:v>
@@ -25441,15 +25345,11 @@
       <x:c r="K152" s="111" t="str">
         <x:v>Engineering</x:v>
       </x:c>
-      <x:c r="L152" s="111" t="str">
-        <x:v>Founder review</x:v>
-      </x:c>
+      <x:c r="L152" s="111"/>
       <x:c r="M152" s="111" t="str">
-        <x:v>Review the reorganized workbook in draft PR #13; preserve the legacy tracker as the source snapshot.</x:v>
-      </x:c>
-      <x:c r="N152" s="112" t="n">
-        <x:v>46255.666666666664</x:v>
-      </x:c>
+        <x:v>Use the PLAN-aligned tracker as the operating view and keep owners, dates, evidence, and daily debriefs current.</x:v>
+      </x:c>
+      <x:c r="N152" s="112"/>
       <x:c r="O152" s="111" t="str">
         <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
       </x:c>
@@ -25460,7 +25360,7 @@
         <x:v>Make PLAN.md the phase source of truth and separate workflow from maturity.</x:v>
       </x:c>
       <x:c r="R152" s="111" t="str">
-        <x:v>No legacy task or note was deleted; the old Master Tracker remains visible.</x:v>
+        <x:v>Published through PR #13. No legacy task, note, backlog item, assumption, or expense value was deleted.</x:v>
       </x:c>
       <x:c r="S152" s="111" t="str">
         <x:v>PLAN.md Phase 0 task 3</x:v>
@@ -25487,7 +25387,7 @@
         <x:v>Add a background-job queue</x:v>
       </x:c>
       <x:c r="H153" s="111" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I153" s="111" t="str">
         <x:v>Backend Implemented</x:v>
@@ -25498,15 +25398,11 @@
       <x:c r="K153" s="111" t="str">
         <x:v>Engineering</x:v>
       </x:c>
-      <x:c r="L153" s="111" t="str">
-        <x:v>Founder review + fresh CI</x:v>
-      </x:c>
+      <x:c r="L153" s="111"/>
       <x:c r="M153" s="111" t="str">
-        <x:v>Review the application-owned PostgreSQL worker foundation on PR #13; merge remains separately gated.</x:v>
-      </x:c>
-      <x:c r="N153" s="112" t="n">
-        <x:v>46259.666666666664</x:v>
-      </x:c>
+        <x:v>Keep the foundation canary-only while deployment, monitoring, Redis/shared throttling, general idempotency, and product-flow migrations remain separately gated.</x:v>
+      </x:c>
+      <x:c r="N153" s="112"/>
       <x:c r="O153" s="111" t="str">
         <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
       </x:c>
@@ -25517,7 +25413,7 @@
         <x:v>Production-shaped durable job migration, separate worker process, leases, retry, terminal handling, telemetry, and a fixed canary.</x:v>
       </x:c>
       <x:c r="R153" s="111" t="str">
-        <x:v>Foundation only: no product flow, provider, deployment, or live credentials.</x:v>
+        <x:v>Published through PR #13 as a foundation only; no product flow, provider, deployment, or live credentials were added.</x:v>
       </x:c>
       <x:c r="S153" s="111" t="str">
         <x:v>PLAN.md Phase 2 task 11</x:v>
@@ -25546,7 +25442,7 @@
         <x:v>Prove canary-specific idempotency and lease fencing</x:v>
       </x:c>
       <x:c r="H154" s="111" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I154" s="111" t="str">
         <x:v>Backend Implemented</x:v>
@@ -25557,15 +25453,11 @@
       <x:c r="K154" s="111" t="str">
         <x:v>Engineering</x:v>
       </x:c>
-      <x:c r="L154" s="111" t="str">
-        <x:v>Founder review + fresh CI</x:v>
-      </x:c>
+      <x:c r="L154" s="111"/>
       <x:c r="M154" s="111" t="str">
-        <x:v>Review atomic enqueue/replay, stale-token rejection, effect reconciliation, and exact-role evidence in PR #13.</x:v>
-      </x:c>
-      <x:c r="N154" s="112" t="n">
-        <x:v>46259.666666666664</x:v>
-      </x:c>
+        <x:v>Treat this as canary-specific evidence only; design the reusable consequential-operation idempotency framework in a separately approved slice.</x:v>
+      </x:c>
+      <x:c r="N154" s="112"/>
       <x:c r="O154" s="111" t="str">
         <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
       </x:c>
@@ -25576,7 +25468,7 @@
         <x:v>Canary-specific idempotency proof supporting the durable worker foundation.</x:v>
       </x:c>
       <x:c r="R154" s="111" t="str">
-        <x:v>This is not the reusable product-wide idempotency framework.</x:v>
+        <x:v>Published through PR #13. This does not implement the reusable product-wide idempotency framework.</x:v>
       </x:c>
       <x:c r="S154" s="111" t="str">
         <x:v>Supports PLAN.md Phase 2 task 12</x:v>
@@ -25715,7 +25607,7 @@
         <x:v>Bind local PostgreSQL host exposure to IPv4 loopback</x:v>
       </x:c>
       <x:c r="H157" s="111" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I157" s="111" t="str">
         <x:v>Backend Implemented</x:v>
@@ -25726,15 +25618,11 @@
       <x:c r="K157" s="111" t="str">
         <x:v>Engineering</x:v>
       </x:c>
-      <x:c r="L157" s="111" t="str">
-        <x:v>Founder review + fresh CI</x:v>
-      </x:c>
+      <x:c r="L157" s="111"/>
       <x:c r="M157" s="111" t="str">
-        <x:v>Verify the tracked Compose mapping remains 127.0.0.1-only and the named volume is preserved.</x:v>
-      </x:c>
-      <x:c r="N157" s="112" t="n">
-        <x:v>46259.666666666664</x:v>
-      </x:c>
+        <x:v>Preserve the 127.0.0.1-only local default; deployed network controls and restricted credentials remain separate gates.</x:v>
+      </x:c>
+      <x:c r="N157" s="112"/>
       <x:c r="O157" s="111" t="str">
         <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
       </x:c>
@@ -25745,7 +25633,7 @@
         <x:v>Reduce LAN exposure of the local static-development database credential.</x:v>
       </x:c>
       <x:c r="R157" s="111" t="str">
-        <x:v>Local-only hardening; no staging or production configuration.</x:v>
+        <x:v>Published through PR #13 as local-only hardening; no staging or production configuration changed.</x:v>
       </x:c>
       <x:c r="S157" s="111" t="str">
         <x:v>PR #13 supplemental hardening</x:v>
@@ -25941,7 +25829,7 @@
         <x:v>Make promotion material E2E independent of calendar date</x:v>
       </x:c>
       <x:c r="H161" s="111" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I161" s="111" t="str">
         <x:v>Integrated</x:v>
@@ -25952,15 +25840,11 @@
       <x:c r="K161" s="111" t="str">
         <x:v>Engineering</x:v>
       </x:c>
-      <x:c r="L161" s="111" t="str">
-        <x:v>Fresh CI</x:v>
-      </x:c>
+      <x:c r="L161" s="111"/>
       <x:c r="M161" s="111" t="str">
-        <x:v>Keep the Playwright test clock fixed before navigation so active-promotion fixtures do not expire with wall time.</x:v>
-      </x:c>
-      <x:c r="N161" s="112" t="n">
-        <x:v>46259.666666666664</x:v>
-      </x:c>
+        <x:v>Keep calendar-dependent fixtures under an explicit test clock and retain the real-stack Playwright regression.</x:v>
+      </x:c>
+      <x:c r="N161" s="112"/>
       <x:c r="O161" s="111" t="str">
         <x:v>https://github.com/QK-Connoisseur/PDoki/pull/13</x:v>
       </x:c>
@@ -25971,7 +25855,7 @@
         <x:v>Freeze the test clock without changing product or fixture behavior.</x:v>
       </x:c>
       <x:c r="R161" s="111" t="str">
-        <x:v>Initial PR #13 E2E failure was a date rollover; replacement exact-head CI passed before this tracker update.</x:v>
+        <x:v>Published through PR #13 after exact-head and post-merge CI passed; no product or fixture behavior changed.</x:v>
       </x:c>
       <x:c r="S161" s="111" t="str">
         <x:v>PR #13 CI repair</x:v>
@@ -26010,7 +25894,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbdf806c34dff43b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb30765db0de34139"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(phase4): reconcile private operations foundation status
</commit_message>
<xml_diff>
--- a/docs/product/Pumdoki_MasterTracker_V4.xlsx
+++ b/docs/product/Pumdoki_MasterTracker_V4.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R12e2c5b5ac1b4d7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R30bf9d4c2b7040a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R6f93f56df0fd4ff1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="Re521642b14464a8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R8365b901f1604472"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legacy Overview 2026-08-16" sheetId="6" r:id="Rc70cd342071647eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="7" r:id="R80e8838af68d49d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Roadmap" sheetId="8" r:id="Rd7f006c4824a4aec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Tracker" sheetId="9" r:id="Rd8a4c6d6313d4495"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Blocker Queue" sheetId="10" r:id="R782ce6d6a0d54a1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Log" sheetId="11" r:id="R7aa2384c19104e32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Register" sheetId="12" r:id="R53c371dadb354279"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R548733a661f649c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R624abc9087394d7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R783ce9771804426a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="R3b4f3c39396940f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="Ra0a28975a35f45d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legacy Overview 2026-08-16" sheetId="6" r:id="Rbe4c589f2dd24ff5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="7" r:id="Re5595ebadf3f48bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Roadmap" sheetId="8" r:id="Rc56c4dcd11cb4199"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Tracker" sheetId="9" r:id="R3c5f6e24cea74b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Blocker Queue" sheetId="10" r:id="R14f92625727e4465"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Log" sheetId="11" r:id="Rdb421418db234377"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Register" sheetId="12" r:id="R1bd9cc832e7e408e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2014,7 +2014,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="164">
+  <x:cellXfs count="172">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -2497,6 +2497,30 @@
     <x:xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="21" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2906,8 +2930,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorkItemsTable" displayName="WorkItemsTable" ref="A3:S161" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:S161"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorkItemsTable" displayName="WorkItemsTable" ref="A3:S164" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:S164"/>
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="Work ID"/>
     <x:tableColumn id="2" name="Phase ID"/>
@@ -2934,8 +2958,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ReviewQueueTable" displayName="ReviewQueueTable" ref="A3:L4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:L4"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ReviewQueueTable" displayName="ReviewQueueTable" ref="A3:L7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:L7"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Work ID"/>
     <x:tableColumn id="2" name="Phase"/>
@@ -3226,7 +3250,7 @@
     </x:row>
     <x:row r="2" ht="21.75" customHeight="1">
       <x:c r="A2" s="92" t="str">
-        <x:v>PLAN.md-aligned view · refreshed August 21, 2026 · record counts are navigation metrics, not phase completion or production-readiness claims</x:v>
+        <x:v>PLAN.md-aligned view · refreshed August 23, 2026 · record counts are navigation metrics; Phase State is the canonical judgment.</x:v>
       </x:c>
       <x:c r="B2" s="92"/>
       <x:c r="C2" s="92"/>
@@ -3273,7 +3297,7 @@
       <x:c r="D5"/>
       <x:c r="E5"/>
       <x:c r="I5" s="130" t="str">
-        <x:v>Decide whether to authorize an isolated private-operations identity/access design and local verification slice. This is not approval to mount the review router, approve creators, promote roles, deploy, or configure live identity infrastructure.</x:v>
+        <x:v>Review this draft Phase 4 foundation and decide whether its exact head may merge. This is not authorization to mount the router, configure live infrastructure, approve creators, promote roles, deploy, or treat G1–G12 as evaluated.</x:v>
       </x:c>
       <x:c r="J5" s="130"/>
       <x:c r="K5" s="130"/>
@@ -3286,7 +3310,7 @@
         <x:v>Work</x:v>
       </x:c>
       <x:c r="B6" s="111" t="str">
-        <x:v>Private-operations identity/access design decision</x:v>
+        <x:v>Private-operations identity/access foundation review</x:v>
       </x:c>
       <x:c r="D6"/>
       <x:c r="E6"/>
@@ -3302,7 +3326,7 @@
         <x:v>Workflow</x:v>
       </x:c>
       <x:c r="B7" s="111" t="str">
-        <x:v>Ready</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="I7" s="131"/>
       <x:c r="J7" s="131"/>
@@ -3316,7 +3340,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B8" s="111" t="str">
-        <x:v>Design and local verification only; no router mount or APPROVED transition</x:v>
+        <x:v>Local dormant foundation only; router unmounted; no APPROVED transition, live IdP/session, runtime DB roles, deployment, or activation</x:v>
       </x:c>
       <x:c r="I8" s="131"/>
       <x:c r="J8" s="131"/>
@@ -3330,10 +3354,10 @@
         <x:v>Evidence</x:v>
       </x:c>
       <x:c r="B9" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/docs/operations/README.md</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/codex/phase4-private-ops-access-foundation/docs/architecture/phase4-slice3-private-operations-access-foundation.md</x:v>
       </x:c>
       <x:c r="I9" s="131" t="str">
-        <x:v>Phase 4 remains partial: creator application and dormant non-approval foundations are published; operational identity, legal, provider, approval, and publishing gates remain open.</x:v>
+        <x:v>Phase 4 remains partial. Provider-neutral identity/access primitives are in review, while every live provider, legal, hosting, session, permission, deployment, approval, and publishing gate remains open.</x:v>
       </x:c>
       <x:c r="J9" s="131"/>
       <x:c r="K9" s="131"/>
@@ -3393,7 +3417,7 @@
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="150" t="n">
         <x:f>COUNTA('Delivery Tracker'!$A$4:$A$400)</x:f>
-        <x:v>158</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="B13" s="151"/>
       <x:c r="C13" s="150" t="n">
@@ -3408,7 +3432,7 @@
       <x:c r="F13" s="151"/>
       <x:c r="G13" s="150" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$H$4:$H$400,"In Review")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H13" s="151"/>
       <x:c r="I13" s="150" t="n">
@@ -3423,7 +3447,7 @@
       <x:c r="L13" s="151"/>
       <x:c r="M13" s="158" t="n">
         <x:f>IF(A13=0,0,C13/A13)</x:f>
-        <x:v>0.17088607594936708</x:v>
+        <x:v>0.16770186335403728</x:v>
       </x:c>
       <x:c r="N13" s="151"/>
     </x:row>
@@ -3764,11 +3788,11 @@
       </x:c>
       <x:c r="F22" s="111" t="n">
         <x:f>'Phase Roadmap'!F8</x:f>
-        <x:v>32</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="G22" s="119" t="n">
         <x:f>'Phase Roadmap'!G8</x:f>
-        <x:v>0.0625</x:v>
+        <x:v>0.05714285714285714</x:v>
       </x:c>
       <x:c r="H22" s="111" t="n">
         <x:f>'Phase Roadmap'!H8</x:f>
@@ -3776,7 +3800,7 @@
       </x:c>
       <x:c r="I22" s="111" t="n">
         <x:f>'Phase Roadmap'!I8</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J22" s="111" t="n">
         <x:f>'Phase Roadmap'!J8</x:f>
@@ -3788,15 +3812,15 @@
       </x:c>
       <x:c r="L22" s="111" t="str">
         <x:f>'Phase Roadmap'!L8</x:f>
-        <x:v>Creator application and dormant non-approval review foundations are published; activation remains blocked.</x:v>
+        <x:v>Creator application and dormant non-approval review foundations are published. A local provider-neutral private-operations identity/access foundation is in review; the router remains unmounted.</x:v>
       </x:c>
       <x:c r="M22" s="111" t="str">
         <x:f>'Phase Roadmap'!M8</x:f>
-        <x:v>Design and locally verify the private operator identity/access boundary; do not activate APPROVED.</x:v>
+        <x:v>Review the foundation without activation; G1–G12 require deployed release/config evidence and remain NOT EVALUATED.</x:v>
       </x:c>
       <x:c r="N22" s="111" t="str">
         <x:f>'Phase Roadmap'!O8</x:f>
-        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/1</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/codex/phase4-private-ops-access-foundation/docs/architecture/phase4-slice3-private-operations-access-foundation.md</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="48" customHeight="1">
@@ -4194,15 +4218,15 @@
       </x:c>
       <x:c r="L29" s="111" t="str">
         <x:f>'Phase Roadmap'!L15</x:f>
-        <x:v>Private shell and dormant review seam exist; production identity, hosting, permissions, and UI do not.</x:v>
+        <x:v>Private shell and dormant review seam exist. A local Slice 3 identity/access foundation is in review; no deployed provider, hosting, session, runtime role, or UI exists.</x:v>
       </x:c>
       <x:c r="M29" s="111" t="str">
         <x:f>'Phase Roadmap'!M15</x:f>
-        <x:v>Approve an isolated private-operations identity/access design and local/staging verification slice.</x:v>
+        <x:v>Review the local foundation without activation. Separately decide live provider/claims, restricted origin/hosting, hardware MFA/recovery, operations session/CSRF, runtime DB grants, audit/incident evidence, and deployment.</x:v>
       </x:c>
       <x:c r="N29" s="111" t="str">
         <x:f>'Phase Roadmap'!O15</x:f>
-        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/docs/operations/README.md</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/codex/phase4-private-ops-access-foundation/docs/architecture/phase4-slice3-private-operations-access-foundation.md</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="48" customHeight="1">
@@ -4457,7 +4481,7 @@
         <x:v>Phase 4</x:v>
       </x:c>
       <x:c r="H36" s="111" t="str">
-        <x:v>Foundation published; operational/legal/identity gates remain open.</x:v>
+        <x:v>Local identity/access foundation is in review; activation, legal, provider, hosting, session, runtime-role, and deployment gates remain open.</x:v>
       </x:c>
       <x:c r="I36" s="111" t="str">
         <x:v>Post-MVP</x:v>
@@ -4519,19 +4543,19 @@
         <x:v>Published base</x:v>
       </x:c>
       <x:c r="F38" s="111" t="str">
-        <x:v>dev @ 6311522</x:v>
+        <x:v>dev @ 492d62c</x:v>
       </x:c>
       <x:c r="G38" s="111" t="str">
-        <x:v>PR #13</x:v>
+        <x:v>Latest merge</x:v>
       </x:c>
       <x:c r="H38" s="111" t="str">
-        <x:v>Merged</x:v>
+        <x:v>PR #14</x:v>
       </x:c>
       <x:c r="I38" s="111" t="str">
-        <x:v>Post-merge CI</x:v>
+        <x:v>Next approval</x:v>
       </x:c>
       <x:c r="J38" s="111" t="str">
-        <x:v>32535922437 — green</x:v>
+        <x:v>Review the Phase 4 draft PR; merge remains separately gated.</x:v>
       </x:c>
       <x:c r="K38" s="111" t="str"/>
       <x:c r="L38" s="111" t="str"/>
@@ -5620,81 +5644,147 @@
     </x:row>
     <x:row r="4" ht="54" customHeight="1">
       <x:c r="A4" s="109" t="str">
-        <x:v>P07-E2E-001</x:v>
+        <x:v>P04-OPS-001</x:v>
       </x:c>
       <x:c r="B4" s="109" t="str">
-        <x:v>P07</x:v>
+        <x:v>P04</x:v>
       </x:c>
       <x:c r="C4" s="109" t="str">
-        <x:v>Core end-to-end vertical slice</x:v>
+        <x:v>Legal, trust, and creator onboarding</x:v>
       </x:c>
       <x:c r="D4" s="109" t="str">
-        <x:v>Core vertical slice</x:v>
+        <x:v>Private operations &amp; moderation</x:v>
       </x:c>
       <x:c r="E4" s="109" t="str">
-        <x:v>Complete the member-to-creator end-to-end product flow</x:v>
+        <x:v>Verify signed private-operations assertions</x:v>
       </x:c>
       <x:c r="F4" s="109" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="G4" s="109" t="str">
         <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H4" s="109" t="str">
-        <x:v>Phase 4–6 dependencies</x:v>
+        <x:v>Founder review</x:v>
       </x:c>
       <x:c r="I4" s="109" t="str">
-        <x:v>Do not begin the product slice until creator approval, media entitlement, and payment-ledger prerequisites are accepted.</x:v>
+        <x:v>Review the provider-neutral assertion boundary; live IdP selection and deployment remain separate.</x:v>
       </x:c>
       <x:c r="J4" s="110"/>
       <x:c r="K4" s="109" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/codex/phase4-private-ops-access-foundation/docs/architecture/phase4-slice3-private-operations-access-foundation.md</x:v>
+      </x:c>
+      <x:c r="L4" s="110" t="n">
+        <x:v>46257.666666666664</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="54" customHeight="1">
+      <x:c r="A5" s="111" t="str">
+        <x:v>P04-OPS-002</x:v>
+      </x:c>
+      <x:c r="B5" s="111" t="str">
+        <x:v>P04</x:v>
+      </x:c>
+      <x:c r="C5" s="111" t="str">
+        <x:v>Legal, trust, and creator onboarding</x:v>
+      </x:c>
+      <x:c r="D5" s="111" t="str">
+        <x:v>Private operations &amp; moderation</x:v>
+      </x:c>
+      <x:c r="E5" s="111" t="str">
+        <x:v>Enforce explicit operator provisioning and transaction-time authorization</x:v>
+      </x:c>
+      <x:c r="F5" s="111" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="G5" s="111" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="H5" s="111" t="str">
+        <x:v>Founder review</x:v>
+      </x:c>
+      <x:c r="I5" s="111" t="str">
+        <x:v>Review DB-owned mappings, grants, immutable history, and transaction-time reauthorization; keep activation separate.</x:v>
+      </x:c>
+      <x:c r="J5" s="112"/>
+      <x:c r="K5" s="111" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/codex/phase4-private-ops-access-foundation/docs/architecture/phase4-slice3-private-operations-access-foundation.md</x:v>
+      </x:c>
+      <x:c r="L5" s="112" t="n">
+        <x:v>46257.666666666664</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="54" customHeight="1">
+      <x:c r="A6" s="111" t="str">
+        <x:v>P04-OPS-003</x:v>
+      </x:c>
+      <x:c r="B6" s="111" t="str">
+        <x:v>P04</x:v>
+      </x:c>
+      <x:c r="C6" s="111" t="str">
+        <x:v>Legal, trust, and creator onboarding</x:v>
+      </x:c>
+      <x:c r="D6" s="111" t="str">
+        <x:v>Private operations &amp; moderation</x:v>
+      </x:c>
+      <x:c r="E6" s="111" t="str">
+        <x:v>Verify the dormant private request-integrity boundary</x:v>
+      </x:c>
+      <x:c r="F6" s="111" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="G6" s="111" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="H6" s="111" t="str">
+        <x:v>Founder review</x:v>
+      </x:c>
+      <x:c r="I6" s="111" t="str">
+        <x:v>Review origin, JSON/CSRF/body-limit, direct-peer evidence, and redaction seams; hosting and live sessions remain separate.</x:v>
+      </x:c>
+      <x:c r="J6" s="112"/>
+      <x:c r="K6" s="111" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/codex/phase4-private-ops-access-foundation/docs/architecture/phase4-slice3-private-operations-access-foundation.md</x:v>
+      </x:c>
+      <x:c r="L6" s="112" t="n">
+        <x:v>46257.666666666664</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="54" customHeight="1">
+      <x:c r="A7" s="111" t="str">
+        <x:v>P07-E2E-001</x:v>
+      </x:c>
+      <x:c r="B7" s="111" t="str">
+        <x:v>P07</x:v>
+      </x:c>
+      <x:c r="C7" s="111" t="str">
+        <x:v>Core end-to-end vertical slice</x:v>
+      </x:c>
+      <x:c r="D7" s="111" t="str">
+        <x:v>Core vertical slice</x:v>
+      </x:c>
+      <x:c r="E7" s="111" t="str">
+        <x:v>Complete the member-to-creator end-to-end product flow</x:v>
+      </x:c>
+      <x:c r="F7" s="111" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="G7" s="111" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="H7" s="111" t="str">
+        <x:v>Phase 4–6 dependencies</x:v>
+      </x:c>
+      <x:c r="I7" s="111" t="str">
+        <x:v>Do not begin the product slice until creator approval, media entitlement, and payment-ledger prerequisites are accepted.</x:v>
+      </x:c>
+      <x:c r="J7" s="112"/>
+      <x:c r="K7" s="111" t="str">
         <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/PLAN.md#11-phase-7--core-end-to-end-vertical-slice</x:v>
       </x:c>
-      <x:c r="L4" s="110" t="n">
+      <x:c r="L7" s="112" t="n">
         <x:v>46255.666666666664</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="54" customHeight="1">
-      <x:c r="A5" s="111"/>
-      <x:c r="B5" s="111"/>
-      <x:c r="C5" s="111"/>
-      <x:c r="D5" s="111"/>
-      <x:c r="E5" s="111"/>
-      <x:c r="F5" s="111"/>
-      <x:c r="G5" s="111"/>
-      <x:c r="H5" s="111"/>
-      <x:c r="I5" s="111"/>
-      <x:c r="J5" s="112"/>
-      <x:c r="K5" s="111"/>
-      <x:c r="L5" s="112"/>
-    </x:row>
-    <x:row r="6" ht="54" customHeight="1">
-      <x:c r="A6" s="111"/>
-      <x:c r="B6" s="111"/>
-      <x:c r="C6" s="111"/>
-      <x:c r="D6" s="111"/>
-      <x:c r="E6" s="111"/>
-      <x:c r="F6" s="111"/>
-      <x:c r="G6" s="111"/>
-      <x:c r="H6" s="111"/>
-      <x:c r="I6" s="111"/>
-      <x:c r="J6" s="112"/>
-      <x:c r="K6" s="111"/>
-      <x:c r="L6" s="112"/>
-    </x:row>
-    <x:row r="7" ht="54" customHeight="1">
-      <x:c r="A7" s="111"/>
-      <x:c r="B7" s="111"/>
-      <x:c r="C7" s="111"/>
-      <x:c r="D7" s="111"/>
-      <x:c r="E7" s="111"/>
-      <x:c r="F7" s="111"/>
-      <x:c r="G7" s="111"/>
-      <x:c r="H7" s="111"/>
-      <x:c r="I7" s="111"/>
-      <x:c r="J7" s="112"/>
-      <x:c r="K7" s="111"/>
-      <x:c r="L7" s="112"/>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
       <x:c r="A8" s="111"/>
@@ -5740,7 +5830,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda1cc3b4d7234481"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f62cf831dd9471f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5986,18 +6076,42 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
-      <x:c r="A8" s="111"/>
-      <x:c r="B8" s="111"/>
-      <x:c r="C8" s="111"/>
-      <x:c r="D8" s="111"/>
-      <x:c r="E8" s="111"/>
-      <x:c r="F8" s="111"/>
-      <x:c r="G8" s="111"/>
-      <x:c r="H8" s="111"/>
-      <x:c r="I8" s="111"/>
-      <x:c r="J8" s="111"/>
-      <x:c r="K8" s="111"/>
-      <x:c r="L8" s="111"/>
+      <x:c r="A8" s="112" t="n">
+        <x:v>46257.666666666664</x:v>
+      </x:c>
+      <x:c r="B8" s="111" t="str">
+        <x:v>P04-OPS-001</x:v>
+      </x:c>
+      <x:c r="C8" s="111" t="str">
+        <x:v>P04</x:v>
+      </x:c>
+      <x:c r="D8" s="111" t="str">
+        <x:v>Build a dormant private-operations identity/access foundation.</x:v>
+      </x:c>
+      <x:c r="E8" s="111" t="str">
+        <x:v>Added strict signed-assertion verification, DB-owned exact operator mappings and permission grants, transaction-time reauthorization, request-integrity seams, immutable history protections, and direct-peer/redacted audit evidence.</x:v>
+      </x:c>
+      <x:c r="F8" s="111" t="str">
+        <x:v>The next operations review work can be evaluated against production-shaped local trust-boundary primitives instead of trusting injected identities or caller-supplied permissions.</x:v>
+      </x:c>
+      <x:c r="G8" s="111" t="str">
+        <x:v>The review router remains unmounted. No APPROVED transition, role promotion, identity collection/files, live provider or issuer, operations session/server, private origin, runtime DB roles, deployment, or live configuration was added; G1–G12 remain NOT EVALUATED.</x:v>
+      </x:c>
+      <x:c r="H8" s="111" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/codex/phase4-private-ops-access-foundation/docs/architecture/phase4-slice3-private-operations-access-foundation.md · implementation commit 9904334 · 287 API / 166 web / 24 contracts / 15 focused DB-review tests</x:v>
+      </x:c>
+      <x:c r="I8" s="111" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="J8" s="111" t="str">
+        <x:v>Draft-PR publication is authorized; merge and every activation/deployment step remain separately gated.</x:v>
+      </x:c>
+      <x:c r="K8" s="111" t="str">
+        <x:v>Publish the draft PR, require exact-head CI, and review the dormant trust boundary without activation.</x:v>
+      </x:c>
+      <x:c r="L8" s="111" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" s="111"/>
@@ -6790,7 +6904,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaff5266ed9647be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red51b6980e7a4637"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7258,19 +7372,19 @@
         <x:v>46240.666666666664</x:v>
       </x:c>
       <x:c r="F16" s="111" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="G16" s="111" t="str">
-        <x:v>Templates exist, but live restricted origin, verifier, enrollment, testing, and approval do not.</x:v>
+        <x:v>A local provider-neutral foundation now verifies signed assertions and DB-owned exact operator/grant authorization. The router remains unmounted; no live IdP, origin, session, runtime DB roles, or deployment exists. G1–G12 remain NOT EVALUATED.</x:v>
       </x:c>
       <x:c r="H16" s="111" t="str">
-        <x:v>Approve an isolated identity/access design and local/staging verification slice.</x:v>
+        <x:v>Review the draft PR and exact-head CI. Preserve the dormant boundary; deployment, live provisioning, and activation require separate evidence and approval.</x:v>
       </x:c>
       <x:c r="I16" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/docs/operations/README.md</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/codex/phase4-private-ops-access-foundation/docs/architecture/phase4-slice3-private-operations-access-foundation.md</x:v>
       </x:c>
       <x:c r="J16" s="112" t="n">
-        <x:v>46255.666666666664</x:v>
+        <x:v>46257.666666666664</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="55" customHeight="1">
@@ -7357,7 +7471,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09a1f47b77a3457f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R416a2ee1b5e14ba8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12941,7 +13055,7 @@
         <x:v>Current focus</x:v>
       </x:c>
       <x:c r="B104" s="111" t="str">
-        <x:v>PR #13 merged into dev as 6311522 and post-merge CI passed. Its fixed canary worker foundation is published, while Phase 2 remains partial and no product flow or deployment was added.</x:v>
+        <x:v>Phase 4 Slice 3 is locally implemented at commit 9904334 and authorized for draft-PR review: strict provider-neutral assertion verification, DB-owned operator/grant authorization, and request-integrity seams. It is not mounted, deployed, or operational.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="42" customHeight="1">
@@ -12949,7 +13063,7 @@
         <x:v>Phase 4</x:v>
       </x:c>
       <x:c r="B105" s="111" t="str">
-        <x:v>Creator application and dormant non-approval review foundations are published; private operations identity/access, legal, provider, approval, role-promotion, and publishing gates remain open.</x:v>
+        <x:v>Creator application and dormant non-approval review foundations are published. The Slice 3 local foundation is in review; legal, live provider/issuer, hosting, session, runtime-role, approval, role-promotion, identity, publishing, and deployment gates remain open. G1–G12 remain NOT EVALUATED.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="42" customHeight="1">
@@ -12965,7 +13079,7 @@
         <x:v>Last refreshed</x:v>
       </x:c>
       <x:c r="B107" s="111" t="str">
-        <x:v>2026-08-21 by Codex during the authorized post-merge tracker and status reconciliation.</x:v>
+        <x:v>2026-08-23 by Codex during the authorized Phase 4 Slice 3 local implementation and draft-publication preparation.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="15.75" customHeight="1"/>
@@ -16812,11 +16926,11 @@
       </x:c>
       <x:c r="F8" s="111" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$B$4:$B$400,$A8)</x:f>
-        <x:v>32</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="G8" s="119" t="n">
         <x:f>IF(F8=0,0,E8/F8)</x:f>
-        <x:v>0.0625</x:v>
+        <x:v>0.05714285714285714</x:v>
       </x:c>
       <x:c r="H8" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A8,'Delivery Tracker'!$H$4:$H$400,"In Progress")</x:f>
@@ -16824,7 +16938,7 @@
       </x:c>
       <x:c r="I8" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A8,'Delivery Tracker'!$H$4:$H$400,"In Review")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J8" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A8,'Delivery Tracker'!$H$4:$H$400,"Blocked")</x:f>
@@ -16835,19 +16949,19 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="L8" s="111" t="str">
-        <x:v>Creator application and dormant non-approval review foundations are published; activation remains blocked.</x:v>
+        <x:v>Creator application and dormant non-approval review foundations are published. A local provider-neutral private-operations identity/access foundation is in review; the router remains unmounted.</x:v>
       </x:c>
       <x:c r="M8" s="111" t="str">
-        <x:v>Design and locally verify the private operator identity/access boundary; do not activate APPROVED.</x:v>
+        <x:v>Review the foundation without activation; G1–G12 require deployed release/config evidence and remain NOT EVALUATED.</x:v>
       </x:c>
       <x:c r="N8" s="111" t="str">
         <x:v>Counsel-approved policies; secure identity/evidence; publishing blocked until approval; reports are auditable.</x:v>
       </x:c>
       <x:c r="O8" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/pull/1</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/codex/phase4-private-ops-access-foundation/docs/architecture/phase4-slice3-private-operations-access-foundation.md</x:v>
       </x:c>
       <x:c r="P8" s="112" t="n">
-        <x:v>46255.666666666664</x:v>
+        <x:v>46257.666666666664</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
@@ -17234,19 +17348,19 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="L15" s="111" t="str">
-        <x:v>Private shell and dormant review seam exist; production identity, hosting, permissions, and UI do not.</x:v>
+        <x:v>Private shell and dormant review seam exist. A local Slice 3 identity/access foundation is in review; no deployed provider, hosting, session, runtime role, or UI exists.</x:v>
       </x:c>
       <x:c r="M15" s="111" t="str">
-        <x:v>Approve an isolated private-operations identity/access design and local/staging verification slice.</x:v>
+        <x:v>Review the local foundation without activation. Separately decide live provider/claims, restricted origin/hosting, hardware MFA/recovery, operations session/CSRF, runtime DB grants, audit/incident evidence, and deployment.</x:v>
       </x:c>
       <x:c r="N15" s="111" t="str">
         <x:v>Founder operates without DB access; reports/payments/verification are manageable; sensitive access is audited.</x:v>
       </x:c>
       <x:c r="O15" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/docs/operations/README.md</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/codex/phase4-private-ops-access-foundation/docs/architecture/phase4-slice3-private-operations-access-foundation.md</x:v>
       </x:c>
       <x:c r="P15" s="112" t="n">
-        <x:v>46255.666666666664</x:v>
+        <x:v>46257.666666666664</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="58" customHeight="1">
@@ -17500,7 +17614,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30351a00dab44d8d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ab08625e901458b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25861,12 +25975,183 @@
         <x:v>PR #13 CI repair</x:v>
       </x:c>
     </x:row>
+    <x:row r="162" ht="46" customHeight="1">
+      <x:c r="A162" s="170" t="str">
+        <x:v>P04-OPS-001</x:v>
+      </x:c>
+      <x:c r="B162" s="170" t="str">
+        <x:v>P04</x:v>
+      </x:c>
+      <x:c r="C162" s="170" t="str">
+        <x:v>Legal, trust, and creator onboarding</x:v>
+      </x:c>
+      <x:c r="D162" s="170" t="str">
+        <x:v>P11</x:v>
+      </x:c>
+      <x:c r="E162" s="170" t="str">
+        <x:v>Supplemental</x:v>
+      </x:c>
+      <x:c r="F162" s="170" t="str">
+        <x:v>Private operations &amp; moderation</x:v>
+      </x:c>
+      <x:c r="G162" s="170" t="str">
+        <x:v>Verify signed private-operations assertions</x:v>
+      </x:c>
+      <x:c r="H162" s="170" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="I162" s="170" t="str">
+        <x:v>Backend Implemented</x:v>
+      </x:c>
+      <x:c r="J162" s="170" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K162" s="170" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="L162" s="170" t="str">
+        <x:v>Founder review</x:v>
+      </x:c>
+      <x:c r="M162" s="170" t="str">
+        <x:v>Review the strict issuer, audience, timing, subject, and hardware-method checks; keep live identity-provider selection and deployment separate.</x:v>
+      </x:c>
+      <x:c r="N162" s="170"/>
+      <x:c r="O162" s="170" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/codex/phase4-private-ops-access-foundation/docs/architecture/phase4-slice3-private-operations-access-foundation.md</x:v>
+      </x:c>
+      <x:c r="P162" s="171" t="n">
+        <x:v>46257.666666666664</x:v>
+      </x:c>
+      <x:c r="Q162" s="170" t="str">
+        <x:v>Provider-neutral signed assertion verification for the dormant private-operations boundary.</x:v>
+      </x:c>
+      <x:c r="R162" s="170" t="str">
+        <x:v>Locally implemented in commit 9904334. No live issuer, key service, provider account, operations session, server mount, or deployment was added; G1–G12 remain NOT EVALUATED.</x:v>
+      </x:c>
+      <x:c r="S162" s="170" t="str">
+        <x:v>Supports PLAN Phase 4 and the Phase 11 private-operations dependency.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" ht="46" customHeight="1">
+      <x:c r="A163" s="170" t="str">
+        <x:v>P04-OPS-002</x:v>
+      </x:c>
+      <x:c r="B163" s="170" t="str">
+        <x:v>P04</x:v>
+      </x:c>
+      <x:c r="C163" s="170" t="str">
+        <x:v>Legal, trust, and creator onboarding</x:v>
+      </x:c>
+      <x:c r="D163" s="170" t="str">
+        <x:v>P11</x:v>
+      </x:c>
+      <x:c r="E163" s="170" t="str">
+        <x:v>Supplemental</x:v>
+      </x:c>
+      <x:c r="F163" s="170" t="str">
+        <x:v>Private operations &amp; moderation</x:v>
+      </x:c>
+      <x:c r="G163" s="170" t="str">
+        <x:v>Enforce explicit operator provisioning and transaction-time authorization</x:v>
+      </x:c>
+      <x:c r="H163" s="170" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="I163" s="170" t="str">
+        <x:v>Backend Implemented</x:v>
+      </x:c>
+      <x:c r="J163" s="170" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K163" s="170" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="L163" s="170" t="str">
+        <x:v>Founder review</x:v>
+      </x:c>
+      <x:c r="M163" s="170" t="str">
+        <x:v>Review exact issuer/subject mapping, active permission grants, immutable history, and same-transaction reauthorization; keep live provisioning and runtime DB roles separate.</x:v>
+      </x:c>
+      <x:c r="N163" s="170"/>
+      <x:c r="O163" s="170" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/codex/phase4-private-ops-access-foundation/docs/architecture/phase4-slice3-private-operations-access-foundation.md</x:v>
+      </x:c>
+      <x:c r="P163" s="171" t="n">
+        <x:v>46257.666666666664</x:v>
+      </x:c>
+      <x:c r="Q163" s="170" t="str">
+        <x:v>Database-owned operator identity and permission evidence for dormant non-approval reviews.</x:v>
+      </x:c>
+      <x:c r="R163" s="170" t="str">
+        <x:v>Locally implemented in commit 9904334 with additive migration evidence. The public router remains unmounted; no APPROVED transition, role promotion, or identity mutation was added.</x:v>
+      </x:c>
+      <x:c r="S163" s="170" t="str">
+        <x:v>Supports PLAN Phase 4 and the Phase 11 private-operations dependency.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="46" customHeight="1">
+      <x:c r="A164" s="170" t="str">
+        <x:v>P04-OPS-003</x:v>
+      </x:c>
+      <x:c r="B164" s="170" t="str">
+        <x:v>P04</x:v>
+      </x:c>
+      <x:c r="C164" s="170" t="str">
+        <x:v>Legal, trust, and creator onboarding</x:v>
+      </x:c>
+      <x:c r="D164" s="170" t="str">
+        <x:v>P11</x:v>
+      </x:c>
+      <x:c r="E164" s="170" t="str">
+        <x:v>Supplemental</x:v>
+      </x:c>
+      <x:c r="F164" s="170" t="str">
+        <x:v>Private operations &amp; moderation</x:v>
+      </x:c>
+      <x:c r="G164" s="170" t="str">
+        <x:v>Verify the dormant private request-integrity boundary</x:v>
+      </x:c>
+      <x:c r="H164" s="170" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="I164" s="170" t="str">
+        <x:v>Backend Implemented</x:v>
+      </x:c>
+      <x:c r="J164" s="170" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K164" s="170" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="L164" s="170" t="str">
+        <x:v>Founder review</x:v>
+      </x:c>
+      <x:c r="M164" s="170" t="str">
+        <x:v>Review exact HTTPS origin, JSON and 16 KB limits, injected CSRF, direct-peer IP evidence, and credential redaction; keep hosting, proxy, and live session controls separate.</x:v>
+      </x:c>
+      <x:c r="N164" s="170"/>
+      <x:c r="O164" s="170" t="str">
+        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/codex/phase4-private-ops-access-foundation/docs/architecture/phase4-slice3-private-operations-access-foundation.md</x:v>
+      </x:c>
+      <x:c r="P164" s="171" t="n">
+        <x:v>46257.666666666664</x:v>
+      </x:c>
+      <x:c r="Q164" s="170" t="str">
+        <x:v>Test-only request-integrity composition and safe audit evidence for the unmounted operations router.</x:v>
+      </x:c>
+      <x:c r="R164" s="170" t="str">
+        <x:v>Locally implemented in commit 9904334. No operations server, private origin, proxy configuration, live session, rate-limit store, or deployment was added.</x:v>
+      </x:c>
+      <x:c r="S164" s="170" t="str">
+        <x:v>Supports PLAN Phase 4 and the Phase 11 private-operations dependency.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:S1"/>
     <x:mergeCell ref="A2:S2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="H4:H161">
+  <x:conditionalFormatting sqref="H4:H164">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Done"/>
     <x:cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="In Review"/>
@@ -25876,25 +26161,25 @@
     <x:cfRule type="containsText" dxfId="24" priority="7" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="5">
-    <x:dataValidation type="list" sqref="H4:H161">
+    <x:dataValidation type="list" sqref="H4:H164">
       <x:formula1>"Not Started,Ready,In Progress,In Review,Blocked,Done,Deferred"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I4:I161">
+    <x:dataValidation type="list" sqref="I4:I164">
       <x:formula1>"Decision Locked,UI Prototype,Backend Implemented,Integrated,Production-Ready,N/A"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="J4:J161">
+    <x:dataValidation type="list" sqref="J4:J164">
       <x:formula1>"Critical,High,Medium,Low"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K4:K161">
+    <x:dataValidation type="list" sqref="K4:K164">
       <x:formula1>"Founder,Engineering,Operations,Counsel,Unassigned"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="E4:E161">
+    <x:dataValidation type="list" sqref="E4:E164">
       <x:formula1>"PLAN task,PLAN phase gate,Supplemental,Legacy-mapped task,Published slice,Decision,Exit criterion"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb30765db0de34139"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R496efc3fe0a44e0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>